<commit_message>
Checklist log update 2026-09-06T05:40:23.528Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K421"/>
+  <dimension ref="A1:K435"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15134,9 +15134,499 @@
         <v>S-mtnd5bqd-0rl1e</v>
       </c>
     </row>
+    <row r="422">
+      <c r="A422" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B422" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C422" t="str">
+        <v>06:30</v>
+      </c>
+      <c r="D422" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E422" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F422" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G422" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H422" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I422" t="str">
+        <v/>
+      </c>
+      <c r="J422" t="str">
+        <v/>
+      </c>
+      <c r="K422" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B423" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C423" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D423" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E423" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F423" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G423" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H423" t="str">
+        <v>N</v>
+      </c>
+      <c r="I423" t="str">
+        <v/>
+      </c>
+      <c r="J423" t="str">
+        <v/>
+      </c>
+      <c r="K423" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B424" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C424" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D424" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E424" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F424" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G424" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H424" t="str">
+        <v>N</v>
+      </c>
+      <c r="I424" t="str">
+        <v/>
+      </c>
+      <c r="J424" t="str">
+        <v/>
+      </c>
+      <c r="K424" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B425" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C425" t="str">
+        <v>06:30</v>
+      </c>
+      <c r="D425" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E425" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F425" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G425" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H425" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I425" t="str">
+        <v/>
+      </c>
+      <c r="J425" t="str">
+        <v/>
+      </c>
+      <c r="K425" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B426" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C426" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D426" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E426" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F426" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G426" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H426" t="str">
+        <v>N</v>
+      </c>
+      <c r="I426" t="str">
+        <v/>
+      </c>
+      <c r="J426" t="str">
+        <v/>
+      </c>
+      <c r="K426" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B427" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C427" t="str">
+        <v>07:19</v>
+      </c>
+      <c r="D427" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E427" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F427" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G427" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H427" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I427" t="str">
+        <v/>
+      </c>
+      <c r="J427" t="str">
+        <v/>
+      </c>
+      <c r="K427" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B428" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C428" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D428" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E428" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F428" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G428" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H428" t="str">
+        <v>N</v>
+      </c>
+      <c r="I428" t="str">
+        <v>not running</v>
+      </c>
+      <c r="J428" t="str">
+        <v/>
+      </c>
+      <c r="K428" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B429" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C429" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D429" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E429" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F429" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G429" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H429" t="str">
+        <v>N</v>
+      </c>
+      <c r="I429" t="str">
+        <v>not running</v>
+      </c>
+      <c r="J429" t="str">
+        <v/>
+      </c>
+      <c r="K429" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B430" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C430" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D430" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E430" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F430" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G430" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H430" t="str">
+        <v>N</v>
+      </c>
+      <c r="I430" t="str">
+        <v/>
+      </c>
+      <c r="J430" t="str">
+        <v/>
+      </c>
+      <c r="K430" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B431" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C431" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D431" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E431" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F431" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G431" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H431" t="str">
+        <v>N</v>
+      </c>
+      <c r="I431" t="str">
+        <v/>
+      </c>
+      <c r="J431" t="str">
+        <v/>
+      </c>
+      <c r="K431" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B432" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C432" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D432" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E432" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F432" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G432" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H432" t="str">
+        <v>N</v>
+      </c>
+      <c r="I432" t="str">
+        <v/>
+      </c>
+      <c r="J432" t="str">
+        <v/>
+      </c>
+      <c r="K432" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B433" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C433" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D433" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E433" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F433" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G433" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H433" t="str">
+        <v>N</v>
+      </c>
+      <c r="I433" t="str">
+        <v/>
+      </c>
+      <c r="J433" t="str">
+        <v/>
+      </c>
+      <c r="K433" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B434" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C434" t="str">
+        <v>07:18</v>
+      </c>
+      <c r="D434" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E434" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F434" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G434" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H434" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I434" t="str">
+        <v>65%</v>
+      </c>
+      <c r="J434" t="str">
+        <v/>
+      </c>
+      <c r="K434" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B435" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C435" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D435" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E435" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F435" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G435" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H435" t="str">
+        <v>N</v>
+      </c>
+      <c r="I435" t="str">
+        <v/>
+      </c>
+      <c r="J435" t="str">
+        <v/>
+      </c>
+      <c r="K435" t="str">
+        <v>S-mtou7bqe-43gji</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K421"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K435"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-06T10:48:03.704Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K435"/>
+  <dimension ref="A1:K449"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15624,9 +15624,499 @@
         <v>S-mtou7bqe-43gji</v>
       </c>
     </row>
+    <row r="436">
+      <c r="A436" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B436" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C436" t="str">
+        <v>21:46</v>
+      </c>
+      <c r="D436" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E436" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F436" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G436" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H436" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I436" t="str">
+        <v/>
+      </c>
+      <c r="J436" t="str">
+        <v/>
+      </c>
+      <c r="K436" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B437" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C437" t="str">
+        <v>04:25</v>
+      </c>
+      <c r="D437" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E437" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F437" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G437" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H437" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I437" t="str">
+        <v/>
+      </c>
+      <c r="J437" t="str">
+        <v/>
+      </c>
+      <c r="K437" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B438" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C438" t="str">
+        <v>04:25</v>
+      </c>
+      <c r="D438" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E438" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F438" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G438" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H438" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I438" t="str">
+        <v/>
+      </c>
+      <c r="J438" t="str">
+        <v/>
+      </c>
+      <c r="K438" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B439" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C439" t="str">
+        <v>04:25</v>
+      </c>
+      <c r="D439" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E439" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F439" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G439" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H439" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I439" t="str">
+        <v/>
+      </c>
+      <c r="J439" t="str">
+        <v/>
+      </c>
+      <c r="K439" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B440" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C440" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D440" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E440" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F440" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G440" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H440" t="str">
+        <v>N</v>
+      </c>
+      <c r="I440" t="str">
+        <v/>
+      </c>
+      <c r="J440" t="str">
+        <v/>
+      </c>
+      <c r="K440" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B441" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C441" t="str">
+        <v>21:46</v>
+      </c>
+      <c r="D441" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E441" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F441" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G441" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H441" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I441" t="str">
+        <v/>
+      </c>
+      <c r="J441" t="str">
+        <v/>
+      </c>
+      <c r="K441" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B442" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C442" t="str">
+        <v>21:46</v>
+      </c>
+      <c r="D442" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E442" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F442" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G442" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H442" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I442" t="str">
+        <v/>
+      </c>
+      <c r="J442" t="str">
+        <v/>
+      </c>
+      <c r="K442" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B443" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C443" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D443" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E443" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F443" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G443" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H443" t="str">
+        <v>N</v>
+      </c>
+      <c r="I443" t="str">
+        <v/>
+      </c>
+      <c r="J443" t="str">
+        <v/>
+      </c>
+      <c r="K443" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B444" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C444" t="str">
+        <v>01:17</v>
+      </c>
+      <c r="D444" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E444" t="str">
+        <v>ts</v>
+      </c>
+      <c r="F444" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G444" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H444" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I444" t="str">
+        <v/>
+      </c>
+      <c r="J444" t="str">
+        <v/>
+      </c>
+      <c r="K444" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B445" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C445" t="str">
+        <v>04:17</v>
+      </c>
+      <c r="D445" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E445" t="str">
+        <v>tp</v>
+      </c>
+      <c r="F445" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G445" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H445" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I445" t="str">
+        <v/>
+      </c>
+      <c r="J445" t="str">
+        <v/>
+      </c>
+      <c r="K445" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B446" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C446" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D446" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E446" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F446" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G446" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H446" t="str">
+        <v>N</v>
+      </c>
+      <c r="I446" t="str">
+        <v/>
+      </c>
+      <c r="J446" t="str">
+        <v/>
+      </c>
+      <c r="K446" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B447" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C447" t="str">
+        <v>04:17</v>
+      </c>
+      <c r="D447" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E447" t="str">
+        <v>ts tp</v>
+      </c>
+      <c r="F447" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G447" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H447" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I447" t="str">
+        <v/>
+      </c>
+      <c r="J447" t="str">
+        <v/>
+      </c>
+      <c r="K447" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B448" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C448" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D448" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E448" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F448" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G448" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H448" t="str">
+        <v>N</v>
+      </c>
+      <c r="I448" t="str">
+        <v/>
+      </c>
+      <c r="J448" t="str">
+        <v/>
+      </c>
+      <c r="K448" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B449" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C449" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D449" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="E449" t="str">
+        <v>TS TP</v>
+      </c>
+      <c r="F449" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G449" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H449" t="str">
+        <v>N</v>
+      </c>
+      <c r="I449" t="str">
+        <v/>
+      </c>
+      <c r="J449" t="str">
+        <v/>
+      </c>
+      <c r="K449" t="str">
+        <v>S-mtpduvu8-c0056</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K435"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K449"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-07T07:22:01.125Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K449"/>
+  <dimension ref="A1:K463"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -16114,9 +16114,499 @@
         <v>S-mtpduvu8-c0056</v>
       </c>
     </row>
+    <row r="450">
+      <c r="A450" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B450" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C450" t="str">
+        <v>06:30</v>
+      </c>
+      <c r="D450" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E450" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F450" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G450" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H450" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I450" t="str">
+        <v/>
+      </c>
+      <c r="J450" t="str">
+        <v/>
+      </c>
+      <c r="K450" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B451" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C451" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D451" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E451" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="F451" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G451" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H451" t="str">
+        <v>N</v>
+      </c>
+      <c r="I451" t="str">
+        <v/>
+      </c>
+      <c r="J451" t="str">
+        <v/>
+      </c>
+      <c r="K451" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B452" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C452" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D452" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E452" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="F452" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G452" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H452" t="str">
+        <v>N</v>
+      </c>
+      <c r="I452" t="str">
+        <v/>
+      </c>
+      <c r="J452" t="str">
+        <v/>
+      </c>
+      <c r="K452" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B453" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C453" t="str">
+        <v>06:30</v>
+      </c>
+      <c r="D453" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E453" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F453" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G453" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H453" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I453" t="str">
+        <v/>
+      </c>
+      <c r="J453" t="str">
+        <v/>
+      </c>
+      <c r="K453" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B454" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C454" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D454" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E454" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="F454" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G454" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H454" t="str">
+        <v>N</v>
+      </c>
+      <c r="I454" t="str">
+        <v/>
+      </c>
+      <c r="J454" t="str">
+        <v/>
+      </c>
+      <c r="K454" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B455" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C455" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="D455" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E455" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F455" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G455" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H455" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I455" t="str">
+        <v/>
+      </c>
+      <c r="J455" t="str">
+        <v/>
+      </c>
+      <c r="K455" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B456" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C456" t="str">
+        <v>10:30</v>
+      </c>
+      <c r="D456" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E456" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F456" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G456" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H456" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I456" t="str">
+        <v/>
+      </c>
+      <c r="J456" t="str">
+        <v/>
+      </c>
+      <c r="K456" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B457" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C457" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D457" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E457" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="F457" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G457" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H457" t="str">
+        <v>N</v>
+      </c>
+      <c r="I457" t="str">
+        <v/>
+      </c>
+      <c r="J457" t="str">
+        <v/>
+      </c>
+      <c r="K457" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B458" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C458" t="str">
+        <v>17:21</v>
+      </c>
+      <c r="D458" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E458" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F458" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G458" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H458" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I458" t="str">
+        <v/>
+      </c>
+      <c r="J458" t="str">
+        <v/>
+      </c>
+      <c r="K458" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B459" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C459" t="str">
+        <v>17:01</v>
+      </c>
+      <c r="D459" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E459" t="str">
+        <v>Luke</v>
+      </c>
+      <c r="F459" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G459" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H459" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I459" t="str">
+        <v/>
+      </c>
+      <c r="J459" t="str">
+        <v/>
+      </c>
+      <c r="K459" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B460" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C460" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D460" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E460" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="F460" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G460" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H460" t="str">
+        <v>N</v>
+      </c>
+      <c r="I460" t="str">
+        <v/>
+      </c>
+      <c r="J460" t="str">
+        <v/>
+      </c>
+      <c r="K460" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B461" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C461" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D461" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E461" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="F461" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G461" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H461" t="str">
+        <v>N</v>
+      </c>
+      <c r="I461" t="str">
+        <v/>
+      </c>
+      <c r="J461" t="str">
+        <v/>
+      </c>
+      <c r="K461" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B462" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C462" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D462" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E462" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="F462" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G462" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H462" t="str">
+        <v>N</v>
+      </c>
+      <c r="I462" t="str">
+        <v/>
+      </c>
+      <c r="J462" t="str">
+        <v/>
+      </c>
+      <c r="K462" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="B463" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C463" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D463" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="E463" t="str">
+        <v>LS KEN</v>
+      </c>
+      <c r="F463" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G463" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H463" t="str">
+        <v>N</v>
+      </c>
+      <c r="I463" t="str">
+        <v/>
+      </c>
+      <c r="J463" t="str">
+        <v/>
+      </c>
+      <c r="K463" t="str">
+        <v>S-mtqj6nrp-4v2oa</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K449"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K463"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-10T21:03:09.396Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K463"/>
+  <dimension ref="A1:K477"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -16604,9 +16604,499 @@
         <v>S-mtqj6nrp-4v2oa</v>
       </c>
     </row>
+    <row r="464">
+      <c r="A464" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B464" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C464" t="str">
+        <v>18:20</v>
+      </c>
+      <c r="D464" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E464" t="str">
+        <v>AH KB</v>
+      </c>
+      <c r="F464" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G464" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H464" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I464" t="str">
+        <v/>
+      </c>
+      <c r="J464" t="str">
+        <v/>
+      </c>
+      <c r="K464" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B465" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C465" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D465" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E465" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F465" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G465" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H465" t="str">
+        <v>N</v>
+      </c>
+      <c r="I465" t="str">
+        <v/>
+      </c>
+      <c r="J465" t="str">
+        <v/>
+      </c>
+      <c r="K465" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B466" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C466" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D466" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E466" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F466" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G466" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H466" t="str">
+        <v>N</v>
+      </c>
+      <c r="I466" t="str">
+        <v/>
+      </c>
+      <c r="J466" t="str">
+        <v/>
+      </c>
+      <c r="K466" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B467" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C467" t="str">
+        <v>18:30</v>
+      </c>
+      <c r="D467" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E467" t="str">
+        <v>AH</v>
+      </c>
+      <c r="F467" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G467" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H467" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I467" t="str">
+        <v/>
+      </c>
+      <c r="J467" t="str">
+        <v/>
+      </c>
+      <c r="K467" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B468" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C468" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D468" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E468" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F468" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G468" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H468" t="str">
+        <v>N</v>
+      </c>
+      <c r="I468" t="str">
+        <v/>
+      </c>
+      <c r="J468" t="str">
+        <v/>
+      </c>
+      <c r="K468" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B469" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C469" t="str">
+        <v>19:30</v>
+      </c>
+      <c r="D469" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E469" t="str">
+        <v>AH</v>
+      </c>
+      <c r="F469" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G469" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H469" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I469" t="str">
+        <v/>
+      </c>
+      <c r="J469" t="str">
+        <v/>
+      </c>
+      <c r="K469" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B470" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C470" t="str">
+        <v>21:15</v>
+      </c>
+      <c r="D470" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E470" t="str">
+        <v>AH</v>
+      </c>
+      <c r="F470" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G470" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H470" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I470" t="str">
+        <v/>
+      </c>
+      <c r="J470" t="str">
+        <v/>
+      </c>
+      <c r="K470" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B471" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C471" t="str">
+        <v>02:45</v>
+      </c>
+      <c r="D471" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E471" t="str">
+        <v>KB</v>
+      </c>
+      <c r="F471" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G471" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H471" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I471" t="str">
+        <v/>
+      </c>
+      <c r="J471" t="str">
+        <v/>
+      </c>
+      <c r="K471" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B472" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C472" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D472" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E472" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F472" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G472" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H472" t="str">
+        <v>N</v>
+      </c>
+      <c r="I472" t="str">
+        <v/>
+      </c>
+      <c r="J472" t="str">
+        <v/>
+      </c>
+      <c r="K472" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B473" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C473" t="str">
+        <v>02:25</v>
+      </c>
+      <c r="D473" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E473" t="str">
+        <v>KB</v>
+      </c>
+      <c r="F473" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G473" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H473" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I473" t="str">
+        <v>Overflowing</v>
+      </c>
+      <c r="J473" t="str">
+        <v/>
+      </c>
+      <c r="K473" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B474" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C474" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D474" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E474" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F474" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G474" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H474" t="str">
+        <v>N</v>
+      </c>
+      <c r="I474" t="str">
+        <v/>
+      </c>
+      <c r="J474" t="str">
+        <v/>
+      </c>
+      <c r="K474" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B475" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C475" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D475" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E475" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F475" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G475" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H475" t="str">
+        <v>N</v>
+      </c>
+      <c r="I475" t="str">
+        <v/>
+      </c>
+      <c r="J475" t="str">
+        <v/>
+      </c>
+      <c r="K475" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B476" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C476" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D476" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E476" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F476" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G476" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H476" t="str">
+        <v>N</v>
+      </c>
+      <c r="I476" t="str">
+        <v/>
+      </c>
+      <c r="J476" t="str">
+        <v/>
+      </c>
+      <c r="K476" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B477" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C477" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D477" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E477" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F477" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G477" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H477" t="str">
+        <v>N</v>
+      </c>
+      <c r="I477" t="str">
+        <v/>
+      </c>
+      <c r="J477" t="str">
+        <v/>
+      </c>
+      <c r="K477" t="str">
+        <v>S-mtvt66hi-obk7b</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K463"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K477"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-11T06:59:36.768Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K477"/>
+  <dimension ref="A1:K491"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17094,9 +17094,499 @@
         <v>S-mtvt66hi-obk7b</v>
       </c>
     </row>
+    <row r="478">
+      <c r="A478" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B478" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C478" t="str">
+        <v>07:05</v>
+      </c>
+      <c r="D478" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E478" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F478" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G478" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H478" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I478" t="str">
+        <v/>
+      </c>
+      <c r="J478" t="str">
+        <v/>
+      </c>
+      <c r="K478" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B479" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C479" t="str">
+        <v>08:05</v>
+      </c>
+      <c r="D479" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E479" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F479" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G479" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H479" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I479" t="str">
+        <v>NA</v>
+      </c>
+      <c r="J479" t="str">
+        <v/>
+      </c>
+      <c r="K479" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B480" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C480" t="str">
+        <v>07:04</v>
+      </c>
+      <c r="D480" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E480" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F480" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G480" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H480" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I480" t="str">
+        <v>NA</v>
+      </c>
+      <c r="J480" t="str">
+        <v/>
+      </c>
+      <c r="K480" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B481" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C481" t="str">
+        <v>07:04</v>
+      </c>
+      <c r="D481" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E481" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F481" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G481" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H481" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I481" t="str">
+        <v/>
+      </c>
+      <c r="J481" t="str">
+        <v/>
+      </c>
+      <c r="K481" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B482" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C482" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D482" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E482" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="F482" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G482" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H482" t="str">
+        <v>N</v>
+      </c>
+      <c r="I482" t="str">
+        <v/>
+      </c>
+      <c r="J482" t="str">
+        <v/>
+      </c>
+      <c r="K482" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B483" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C483" t="str">
+        <v>07:05</v>
+      </c>
+      <c r="D483" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E483" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F483" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G483" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H483" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I483" t="str">
+        <v/>
+      </c>
+      <c r="J483" t="str">
+        <v/>
+      </c>
+      <c r="K483" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B484" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C484" t="str">
+        <v>09:04</v>
+      </c>
+      <c r="D484" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E484" t="str">
+        <v>AS</v>
+      </c>
+      <c r="F484" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G484" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H484" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I484" t="str">
+        <v/>
+      </c>
+      <c r="J484" t="str">
+        <v/>
+      </c>
+      <c r="K484" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B485" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C485" t="str">
+        <v>15:49</v>
+      </c>
+      <c r="D485" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E485" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F485" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G485" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H485" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I485" t="str">
+        <v/>
+      </c>
+      <c r="J485" t="str">
+        <v/>
+      </c>
+      <c r="K485" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B486" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C486" t="str">
+        <v>16:59</v>
+      </c>
+      <c r="D486" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E486" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F486" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G486" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H486" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I486" t="str">
+        <v/>
+      </c>
+      <c r="J486" t="str">
+        <v/>
+      </c>
+      <c r="K486" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B487" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C487" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D487" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E487" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="F487" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G487" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H487" t="str">
+        <v>N</v>
+      </c>
+      <c r="I487" t="str">
+        <v/>
+      </c>
+      <c r="J487" t="str">
+        <v/>
+      </c>
+      <c r="K487" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B488" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C488" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D488" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E488" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="F488" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G488" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H488" t="str">
+        <v>N</v>
+      </c>
+      <c r="I488" t="str">
+        <v/>
+      </c>
+      <c r="J488" t="str">
+        <v/>
+      </c>
+      <c r="K488" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B489" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C489" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D489" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E489" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="F489" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G489" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H489" t="str">
+        <v>N</v>
+      </c>
+      <c r="I489" t="str">
+        <v/>
+      </c>
+      <c r="J489" t="str">
+        <v/>
+      </c>
+      <c r="K489" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B490" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C490" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D490" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E490" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="F490" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G490" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H490" t="str">
+        <v>N</v>
+      </c>
+      <c r="I490" t="str">
+        <v/>
+      </c>
+      <c r="J490" t="str">
+        <v/>
+      </c>
+      <c r="K490" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B491" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C491" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D491" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="E491" t="str">
+        <v>Tim &amp; Amber</v>
+      </c>
+      <c r="F491" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G491" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H491" t="str">
+        <v>N</v>
+      </c>
+      <c r="I491" t="str">
+        <v/>
+      </c>
+      <c r="J491" t="str">
+        <v/>
+      </c>
+      <c r="K491" t="str">
+        <v>S-mtvun4j7-0zw3k</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K477"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K491"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-11T07:16:39.331Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -17417,13 +17417,13 @@
         <v>Day</v>
       </c>
       <c r="C487" t="str">
-        <v>(not entered)</v>
+        <v>16:59</v>
       </c>
       <c r="D487" t="str">
         <v>Tim &amp; Amber</v>
       </c>
       <c r="E487" t="str">
-        <v>Tim &amp; Amber</v>
+        <v>AS</v>
       </c>
       <c r="F487" t="str">
         <v>During Processing</v>
@@ -17432,7 +17432,7 @@
         <v>Empty drop box at end of shift</v>
       </c>
       <c r="H487" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I487" t="str">
         <v/>
@@ -17522,7 +17522,7 @@
         <v>Day</v>
       </c>
       <c r="C490" t="str">
-        <v>(not entered)</v>
+        <v>17:00</v>
       </c>
       <c r="D490" t="str">
         <v>Tim &amp; Amber</v>
@@ -17537,7 +17537,7 @@
         <v>Check drinking water tank level</v>
       </c>
       <c r="H490" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I490" t="str">
         <v/>
@@ -17557,13 +17557,13 @@
         <v>Day</v>
       </c>
       <c r="C491" t="str">
-        <v>(not entered)</v>
+        <v>17:00</v>
       </c>
       <c r="D491" t="str">
         <v>Tim &amp; Amber</v>
       </c>
       <c r="E491" t="str">
-        <v>Tim &amp; Amber</v>
+        <v>TR CF</v>
       </c>
       <c r="F491" t="str">
         <v>Once a Week</v>
@@ -17572,7 +17572,7 @@
         <v>Empty all bins and wheel barrows</v>
       </c>
       <c r="H491" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I491" t="str">
         <v/>

</xml_diff>

<commit_message>
Checklist log update 2026-09-13T02:11:55.916Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K491"/>
+  <dimension ref="A1:K505"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17584,9 +17584,499 @@
         <v>S-mtvun4j7-0zw3k</v>
       </c>
     </row>
+    <row r="492">
+      <c r="A492" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B492" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C492" t="str">
+        <v>18:20</v>
+      </c>
+      <c r="D492" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E492" t="str">
+        <v>AH KB</v>
+      </c>
+      <c r="F492" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G492" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H492" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I492" t="str">
+        <v/>
+      </c>
+      <c r="J492" t="str">
+        <v/>
+      </c>
+      <c r="K492" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B493" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C493" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D493" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E493" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F493" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G493" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H493" t="str">
+        <v>N</v>
+      </c>
+      <c r="I493" t="str">
+        <v/>
+      </c>
+      <c r="J493" t="str">
+        <v/>
+      </c>
+      <c r="K493" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B494" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C494" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D494" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E494" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F494" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G494" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H494" t="str">
+        <v>N</v>
+      </c>
+      <c r="I494" t="str">
+        <v/>
+      </c>
+      <c r="J494" t="str">
+        <v/>
+      </c>
+      <c r="K494" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B495" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C495" t="str">
+        <v>19:10</v>
+      </c>
+      <c r="D495" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E495" t="str">
+        <v>KB</v>
+      </c>
+      <c r="F495" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G495" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H495" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I495" t="str">
+        <v/>
+      </c>
+      <c r="J495" t="str">
+        <v/>
+      </c>
+      <c r="K495" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B496" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C496" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D496" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E496" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F496" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G496" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H496" t="str">
+        <v>N</v>
+      </c>
+      <c r="I496" t="str">
+        <v/>
+      </c>
+      <c r="J496" t="str">
+        <v/>
+      </c>
+      <c r="K496" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B497" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C497" t="str">
+        <v>18:25</v>
+      </c>
+      <c r="D497" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E497" t="str">
+        <v>KB AH</v>
+      </c>
+      <c r="F497" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G497" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H497" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I497" t="str">
+        <v/>
+      </c>
+      <c r="J497" t="str">
+        <v/>
+      </c>
+      <c r="K497" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B498" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C498" t="str">
+        <v>21:30</v>
+      </c>
+      <c r="D498" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E498" t="str">
+        <v>KB</v>
+      </c>
+      <c r="F498" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G498" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H498" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I498" t="str">
+        <v/>
+      </c>
+      <c r="J498" t="str">
+        <v/>
+      </c>
+      <c r="K498" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B499" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C499" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D499" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E499" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F499" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G499" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H499" t="str">
+        <v>N</v>
+      </c>
+      <c r="I499" t="str">
+        <v/>
+      </c>
+      <c r="J499" t="str">
+        <v/>
+      </c>
+      <c r="K499" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B500" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C500" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D500" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E500" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F500" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G500" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H500" t="str">
+        <v>N</v>
+      </c>
+      <c r="I500" t="str">
+        <v/>
+      </c>
+      <c r="J500" t="str">
+        <v/>
+      </c>
+      <c r="K500" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B501" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C501" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D501" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E501" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F501" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G501" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H501" t="str">
+        <v>N</v>
+      </c>
+      <c r="I501" t="str">
+        <v/>
+      </c>
+      <c r="J501" t="str">
+        <v/>
+      </c>
+      <c r="K501" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B502" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C502" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D502" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E502" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F502" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G502" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H502" t="str">
+        <v>N</v>
+      </c>
+      <c r="I502" t="str">
+        <v/>
+      </c>
+      <c r="J502" t="str">
+        <v/>
+      </c>
+      <c r="K502" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B503" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C503" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D503" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E503" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F503" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G503" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H503" t="str">
+        <v>N</v>
+      </c>
+      <c r="I503" t="str">
+        <v/>
+      </c>
+      <c r="J503" t="str">
+        <v/>
+      </c>
+      <c r="K503" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B504" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C504" t="str">
+        <v>01:11</v>
+      </c>
+      <c r="D504" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E504" t="str">
+        <v>AH KB</v>
+      </c>
+      <c r="F504" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G504" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H504" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I504" t="str">
+        <v/>
+      </c>
+      <c r="J504" t="str">
+        <v/>
+      </c>
+      <c r="K504" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B505" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C505" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D505" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="E505" t="str">
+        <v>Anthony/ Kyle</v>
+      </c>
+      <c r="F505" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G505" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H505" t="str">
+        <v>N</v>
+      </c>
+      <c r="I505" t="str">
+        <v/>
+      </c>
+      <c r="J505" t="str">
+        <v/>
+      </c>
+      <c r="K505" t="str">
+        <v>S-mtyiu5yc-moqjw</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K491"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K505"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-13T07:33:14.967Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K505"/>
+  <dimension ref="A1:K519"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -18074,9 +18074,499 @@
         <v>S-mtyiu5yc-moqjw</v>
       </c>
     </row>
+    <row r="506">
+      <c r="A506" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B506" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C506" t="str">
+        <v>06:00</v>
+      </c>
+      <c r="D506" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E506" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F506" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G506" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H506" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I506" t="str">
+        <v/>
+      </c>
+      <c r="J506" t="str">
+        <v/>
+      </c>
+      <c r="K506" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B507" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C507" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D507" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E507" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="F507" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G507" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H507" t="str">
+        <v>N</v>
+      </c>
+      <c r="I507" t="str">
+        <v/>
+      </c>
+      <c r="J507" t="str">
+        <v/>
+      </c>
+      <c r="K507" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B508" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C508" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D508" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E508" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="F508" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G508" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H508" t="str">
+        <v>N</v>
+      </c>
+      <c r="I508" t="str">
+        <v/>
+      </c>
+      <c r="J508" t="str">
+        <v/>
+      </c>
+      <c r="K508" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B509" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C509" t="str">
+        <v>06:12</v>
+      </c>
+      <c r="D509" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E509" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F509" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G509" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H509" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I509" t="str">
+        <v/>
+      </c>
+      <c r="J509" t="str">
+        <v/>
+      </c>
+      <c r="K509" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B510" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C510" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D510" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E510" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="F510" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G510" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H510" t="str">
+        <v>N</v>
+      </c>
+      <c r="I510" t="str">
+        <v/>
+      </c>
+      <c r="J510" t="str">
+        <v/>
+      </c>
+      <c r="K510" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B511" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C511" t="str">
+        <v>06:50</v>
+      </c>
+      <c r="D511" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E511" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F511" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G511" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H511" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I511" t="str">
+        <v/>
+      </c>
+      <c r="J511" t="str">
+        <v/>
+      </c>
+      <c r="K511" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B512" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C512" t="str">
+        <v>09:13</v>
+      </c>
+      <c r="D512" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E512" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F512" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G512" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H512" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I512" t="str">
+        <v/>
+      </c>
+      <c r="J512" t="str">
+        <v/>
+      </c>
+      <c r="K512" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B513" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C513" t="str">
+        <v>15:34</v>
+      </c>
+      <c r="D513" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E513" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F513" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G513" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H513" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I513" t="str">
+        <v/>
+      </c>
+      <c r="J513" t="str">
+        <v/>
+      </c>
+      <c r="K513" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B514" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C514" t="str">
+        <v>17:32</v>
+      </c>
+      <c r="D514" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E514" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F514" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G514" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H514" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I514" t="str">
+        <v/>
+      </c>
+      <c r="J514" t="str">
+        <v/>
+      </c>
+      <c r="K514" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B515" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C515" t="str">
+        <v>17:30</v>
+      </c>
+      <c r="D515" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E515" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F515" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G515" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H515" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I515" t="str">
+        <v/>
+      </c>
+      <c r="J515" t="str">
+        <v/>
+      </c>
+      <c r="K515" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B516" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C516" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D516" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E516" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="F516" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G516" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H516" t="str">
+        <v>N</v>
+      </c>
+      <c r="I516" t="str">
+        <v/>
+      </c>
+      <c r="J516" t="str">
+        <v/>
+      </c>
+      <c r="K516" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B517" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C517" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D517" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E517" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="F517" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G517" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H517" t="str">
+        <v>N</v>
+      </c>
+      <c r="I517" t="str">
+        <v/>
+      </c>
+      <c r="J517" t="str">
+        <v/>
+      </c>
+      <c r="K517" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B518" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C518" t="str">
+        <v>17:32</v>
+      </c>
+      <c r="D518" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E518" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F518" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G518" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H518" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I518" t="str">
+        <v/>
+      </c>
+      <c r="J518" t="str">
+        <v/>
+      </c>
+      <c r="K518" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="B519" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C519" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D519" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="E519" t="str">
+        <v>Tim/Rob</v>
+      </c>
+      <c r="F519" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G519" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H519" t="str">
+        <v>N</v>
+      </c>
+      <c r="I519" t="str">
+        <v/>
+      </c>
+      <c r="J519" t="str">
+        <v/>
+      </c>
+      <c r="K519" t="str">
+        <v>S-mtyiu6tz-wi9mw</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K505"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K519"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-14T19:30:08.516Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K519"/>
+  <dimension ref="A1:K533"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -18564,9 +18564,499 @@
         <v>S-mtyiu6tz-wi9mw</v>
       </c>
     </row>
+    <row r="520">
+      <c r="A520" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B520" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C520" t="str">
+        <v>18:16</v>
+      </c>
+      <c r="D520" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E520" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F520" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G520" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H520" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I520" t="str">
+        <v/>
+      </c>
+      <c r="J520" t="str">
+        <v/>
+      </c>
+      <c r="K520" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B521" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C521" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D521" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E521" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F521" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G521" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H521" t="str">
+        <v>N</v>
+      </c>
+      <c r="I521" t="str">
+        <v/>
+      </c>
+      <c r="J521" t="str">
+        <v/>
+      </c>
+      <c r="K521" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B522" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C522" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D522" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E522" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F522" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G522" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H522" t="str">
+        <v>N</v>
+      </c>
+      <c r="I522" t="str">
+        <v/>
+      </c>
+      <c r="J522" t="str">
+        <v/>
+      </c>
+      <c r="K522" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B523" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C523" t="str">
+        <v>18:34</v>
+      </c>
+      <c r="D523" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E523" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F523" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G523" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H523" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I523" t="str">
+        <v/>
+      </c>
+      <c r="J523" t="str">
+        <v/>
+      </c>
+      <c r="K523" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B524" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C524" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D524" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E524" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F524" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G524" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H524" t="str">
+        <v>N</v>
+      </c>
+      <c r="I524" t="str">
+        <v/>
+      </c>
+      <c r="J524" t="str">
+        <v/>
+      </c>
+      <c r="K524" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B525" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C525" t="str">
+        <v>18:17</v>
+      </c>
+      <c r="D525" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E525" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F525" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G525" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H525" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I525" t="str">
+        <v/>
+      </c>
+      <c r="J525" t="str">
+        <v/>
+      </c>
+      <c r="K525" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B526" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C526" t="str">
+        <v>22:12</v>
+      </c>
+      <c r="D526" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E526" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F526" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G526" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H526" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I526" t="str">
+        <v/>
+      </c>
+      <c r="J526" t="str">
+        <v/>
+      </c>
+      <c r="K526" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B527" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C527" t="str">
+        <v>03:22</v>
+      </c>
+      <c r="D527" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E527" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F527" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G527" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H527" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I527" t="str">
+        <v/>
+      </c>
+      <c r="J527" t="str">
+        <v/>
+      </c>
+      <c r="K527" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B528" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C528" t="str">
+        <v>05:29</v>
+      </c>
+      <c r="D528" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E528" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F528" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G528" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H528" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I528" t="str">
+        <v/>
+      </c>
+      <c r="J528" t="str">
+        <v/>
+      </c>
+      <c r="K528" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B529" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C529" t="str">
+        <v>05:23</v>
+      </c>
+      <c r="D529" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E529" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F529" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G529" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H529" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I529" t="str">
+        <v/>
+      </c>
+      <c r="J529" t="str">
+        <v/>
+      </c>
+      <c r="K529" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B530" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C530" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D530" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E530" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F530" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G530" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H530" t="str">
+        <v>N</v>
+      </c>
+      <c r="I530" t="str">
+        <v/>
+      </c>
+      <c r="J530" t="str">
+        <v/>
+      </c>
+      <c r="K530" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B531" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C531" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D531" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E531" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F531" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G531" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H531" t="str">
+        <v>N</v>
+      </c>
+      <c r="I531" t="str">
+        <v/>
+      </c>
+      <c r="J531" t="str">
+        <v/>
+      </c>
+      <c r="K531" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B532" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C532" t="str">
+        <v>18:32</v>
+      </c>
+      <c r="D532" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E532" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F532" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G532" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H532" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I532" t="str">
+        <v>50%</v>
+      </c>
+      <c r="J532" t="str">
+        <v/>
+      </c>
+      <c r="K532" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B533" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C533" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D533" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E533" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F533" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G533" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H533" t="str">
+        <v>N</v>
+      </c>
+      <c r="I533" t="str">
+        <v/>
+      </c>
+      <c r="J533" t="str">
+        <v/>
+      </c>
+      <c r="K533" t="str">
+        <v>S-mu0yu73b-i96ip</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K519"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K533"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-15T11:03:16.452Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K533"/>
+  <dimension ref="A1:K547"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19054,9 +19054,499 @@
         <v>S-mu0yu73b-i96ip</v>
       </c>
     </row>
+    <row r="534">
+      <c r="A534" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B534" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C534" t="str">
+        <v>18:27</v>
+      </c>
+      <c r="D534" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E534" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F534" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G534" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H534" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I534" t="str">
+        <v/>
+      </c>
+      <c r="J534" t="str">
+        <v/>
+      </c>
+      <c r="K534" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B535" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C535" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D535" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E535" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F535" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G535" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H535" t="str">
+        <v>N</v>
+      </c>
+      <c r="I535" t="str">
+        <v/>
+      </c>
+      <c r="J535" t="str">
+        <v/>
+      </c>
+      <c r="K535" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B536" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C536" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D536" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E536" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F536" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G536" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H536" t="str">
+        <v>N</v>
+      </c>
+      <c r="I536" t="str">
+        <v/>
+      </c>
+      <c r="J536" t="str">
+        <v/>
+      </c>
+      <c r="K536" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B537" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C537" t="str">
+        <v>18:34</v>
+      </c>
+      <c r="D537" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E537" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F537" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G537" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H537" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I537" t="str">
+        <v/>
+      </c>
+      <c r="J537" t="str">
+        <v/>
+      </c>
+      <c r="K537" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B538" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C538" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D538" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E538" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F538" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G538" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H538" t="str">
+        <v>N</v>
+      </c>
+      <c r="I538" t="str">
+        <v/>
+      </c>
+      <c r="J538" t="str">
+        <v/>
+      </c>
+      <c r="K538" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B539" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C539" t="str">
+        <v>18:40</v>
+      </c>
+      <c r="D539" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E539" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F539" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G539" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H539" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I539" t="str">
+        <v/>
+      </c>
+      <c r="J539" t="str">
+        <v/>
+      </c>
+      <c r="K539" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B540" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C540" t="str">
+        <v>21:03</v>
+      </c>
+      <c r="D540" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E540" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F540" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G540" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H540" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I540" t="str">
+        <v/>
+      </c>
+      <c r="J540" t="str">
+        <v/>
+      </c>
+      <c r="K540" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B541" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C541" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D541" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E541" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F541" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G541" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H541" t="str">
+        <v>N</v>
+      </c>
+      <c r="I541" t="str">
+        <v/>
+      </c>
+      <c r="J541" t="str">
+        <v/>
+      </c>
+      <c r="K541" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B542" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C542" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D542" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E542" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F542" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G542" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H542" t="str">
+        <v>N</v>
+      </c>
+      <c r="I542" t="str">
+        <v/>
+      </c>
+      <c r="J542" t="str">
+        <v/>
+      </c>
+      <c r="K542" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B543" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C543" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D543" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E543" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F543" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G543" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H543" t="str">
+        <v>N</v>
+      </c>
+      <c r="I543" t="str">
+        <v/>
+      </c>
+      <c r="J543" t="str">
+        <v/>
+      </c>
+      <c r="K543" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B544" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C544" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D544" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E544" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F544" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G544" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H544" t="str">
+        <v>N</v>
+      </c>
+      <c r="I544" t="str">
+        <v/>
+      </c>
+      <c r="J544" t="str">
+        <v/>
+      </c>
+      <c r="K544" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B545" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C545" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D545" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E545" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F545" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G545" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H545" t="str">
+        <v>N</v>
+      </c>
+      <c r="I545" t="str">
+        <v/>
+      </c>
+      <c r="J545" t="str">
+        <v/>
+      </c>
+      <c r="K545" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B546" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C546" t="str">
+        <v>20:59</v>
+      </c>
+      <c r="D546" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E546" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F546" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G546" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H546" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I546" t="str">
+        <v>50%</v>
+      </c>
+      <c r="J546" t="str">
+        <v/>
+      </c>
+      <c r="K546" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="B547" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C547" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D547" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="E547" t="str">
+        <v>DH AH KEN</v>
+      </c>
+      <c r="F547" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G547" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H547" t="str">
+        <v>N</v>
+      </c>
+      <c r="I547" t="str">
+        <v/>
+      </c>
+      <c r="J547" t="str">
+        <v/>
+      </c>
+      <c r="K547" t="str">
+        <v>S-mu2k791g-8buc6</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K533"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K547"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-15T18:55:15.475Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -19056,7 +19056,7 @@
     </row>
     <row r="534">
       <c r="A534" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B534" t="str">
         <v>Night</v>
@@ -19091,7 +19091,7 @@
     </row>
     <row r="535">
       <c r="A535" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B535" t="str">
         <v>Night</v>
@@ -19126,7 +19126,7 @@
     </row>
     <row r="536">
       <c r="A536" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B536" t="str">
         <v>Night</v>
@@ -19161,7 +19161,7 @@
     </row>
     <row r="537">
       <c r="A537" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B537" t="str">
         <v>Night</v>
@@ -19196,7 +19196,7 @@
     </row>
     <row r="538">
       <c r="A538" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B538" t="str">
         <v>Night</v>
@@ -19231,7 +19231,7 @@
     </row>
     <row r="539">
       <c r="A539" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B539" t="str">
         <v>Night</v>
@@ -19266,7 +19266,7 @@
     </row>
     <row r="540">
       <c r="A540" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B540" t="str">
         <v>Night</v>
@@ -19301,13 +19301,13 @@
     </row>
     <row r="541">
       <c r="A541" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B541" t="str">
         <v>Night</v>
       </c>
       <c r="C541" t="str">
-        <v>(not entered)</v>
+        <v>03:33</v>
       </c>
       <c r="D541" t="str">
         <v>DH AH KEN</v>
@@ -19322,7 +19322,7 @@
         <v>Purge mills — 200 pumps each</v>
       </c>
       <c r="H541" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I541" t="str">
         <v/>
@@ -19336,13 +19336,13 @@
     </row>
     <row r="542">
       <c r="A542" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B542" t="str">
         <v>Night</v>
       </c>
       <c r="C542" t="str">
-        <v>(not entered)</v>
+        <v>05:35</v>
       </c>
       <c r="D542" t="str">
         <v>DH AH KEN</v>
@@ -19357,7 +19357,7 @@
         <v>Inspect &amp; clean steam vent</v>
       </c>
       <c r="H542" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I542" t="str">
         <v/>
@@ -19371,13 +19371,13 @@
     </row>
     <row r="543">
       <c r="A543" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B543" t="str">
         <v>Night</v>
       </c>
       <c r="C543" t="str">
-        <v>(not entered)</v>
+        <v>05:29</v>
       </c>
       <c r="D543" t="str">
         <v>DH AH KEN</v>
@@ -19392,7 +19392,7 @@
         <v>Empty drop box at end of shift</v>
       </c>
       <c r="H543" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I543" t="str">
         <v/>
@@ -19406,13 +19406,13 @@
     </row>
     <row r="544">
       <c r="A544" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B544" t="str">
         <v>Night</v>
       </c>
       <c r="C544" t="str">
-        <v>(not entered)</v>
+        <v>23:22</v>
       </c>
       <c r="D544" t="str">
         <v>DH AH KEN</v>
@@ -19427,7 +19427,7 @@
         <v>Deep clean around mills</v>
       </c>
       <c r="H544" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I544" t="str">
         <v/>
@@ -19441,7 +19441,7 @@
     </row>
     <row r="545">
       <c r="A545" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B545" t="str">
         <v>Night</v>
@@ -19476,7 +19476,7 @@
     </row>
     <row r="546">
       <c r="A546" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B546" t="str">
         <v>Night</v>
@@ -19511,7 +19511,7 @@
     </row>
     <row r="547">
       <c r="A547" t="str">
-        <v>2026-09-15</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B547" t="str">
         <v>Night</v>

</xml_diff>

<commit_message>
Checklist log update 2026-09-16T00:56:57.380Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K547"/>
+  <dimension ref="A1:K561"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19544,9 +19544,499 @@
         <v>S-mu2k791g-8buc6</v>
       </c>
     </row>
+    <row r="548">
+      <c r="A548" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B548" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C548" t="str">
+        <v>07:37</v>
+      </c>
+      <c r="D548" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E548" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F548" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G548" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H548" t="str">
+        <v>N</v>
+      </c>
+      <c r="I548" t="str">
+        <v/>
+      </c>
+      <c r="J548" t="str">
+        <v/>
+      </c>
+      <c r="K548" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B549" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C549" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D549" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E549" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F549" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G549" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H549" t="str">
+        <v>N</v>
+      </c>
+      <c r="I549" t="str">
+        <v/>
+      </c>
+      <c r="J549" t="str">
+        <v/>
+      </c>
+      <c r="K549" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B550" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C550" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D550" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E550" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F550" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G550" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H550" t="str">
+        <v>N</v>
+      </c>
+      <c r="I550" t="str">
+        <v/>
+      </c>
+      <c r="J550" t="str">
+        <v/>
+      </c>
+      <c r="K550" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B551" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C551" t="str">
+        <v>07:37</v>
+      </c>
+      <c r="D551" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E551" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F551" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G551" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H551" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I551" t="str">
+        <v/>
+      </c>
+      <c r="J551" t="str">
+        <v/>
+      </c>
+      <c r="K551" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B552" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C552" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D552" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E552" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F552" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G552" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H552" t="str">
+        <v>N</v>
+      </c>
+      <c r="I552" t="str">
+        <v/>
+      </c>
+      <c r="J552" t="str">
+        <v/>
+      </c>
+      <c r="K552" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B553" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C553" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D553" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E553" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F553" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G553" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H553" t="str">
+        <v>N</v>
+      </c>
+      <c r="I553" t="str">
+        <v/>
+      </c>
+      <c r="J553" t="str">
+        <v/>
+      </c>
+      <c r="K553" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B554" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C554" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D554" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E554" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F554" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G554" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H554" t="str">
+        <v>N</v>
+      </c>
+      <c r="I554" t="str">
+        <v/>
+      </c>
+      <c r="J554" t="str">
+        <v/>
+      </c>
+      <c r="K554" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B555" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C555" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D555" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E555" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F555" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G555" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H555" t="str">
+        <v>N</v>
+      </c>
+      <c r="I555" t="str">
+        <v/>
+      </c>
+      <c r="J555" t="str">
+        <v/>
+      </c>
+      <c r="K555" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B556" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C556" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D556" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E556" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F556" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G556" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H556" t="str">
+        <v>N</v>
+      </c>
+      <c r="I556" t="str">
+        <v/>
+      </c>
+      <c r="J556" t="str">
+        <v/>
+      </c>
+      <c r="K556" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B557" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C557" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D557" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E557" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F557" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G557" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H557" t="str">
+        <v>N</v>
+      </c>
+      <c r="I557" t="str">
+        <v/>
+      </c>
+      <c r="J557" t="str">
+        <v/>
+      </c>
+      <c r="K557" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B558" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C558" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D558" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E558" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F558" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G558" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H558" t="str">
+        <v>N</v>
+      </c>
+      <c r="I558" t="str">
+        <v/>
+      </c>
+      <c r="J558" t="str">
+        <v/>
+      </c>
+      <c r="K558" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B559" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C559" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D559" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E559" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F559" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G559" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H559" t="str">
+        <v>N</v>
+      </c>
+      <c r="I559" t="str">
+        <v/>
+      </c>
+      <c r="J559" t="str">
+        <v/>
+      </c>
+      <c r="K559" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B560" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C560" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D560" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E560" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F560" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G560" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H560" t="str">
+        <v>N</v>
+      </c>
+      <c r="I560" t="str">
+        <v/>
+      </c>
+      <c r="J560" t="str">
+        <v/>
+      </c>
+      <c r="K560" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B561" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C561" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D561" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="E561" t="str">
+        <v>tp rp</v>
+      </c>
+      <c r="F561" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G561" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H561" t="str">
+        <v>N</v>
+      </c>
+      <c r="I561" t="str">
+        <v/>
+      </c>
+      <c r="J561" t="str">
+        <v/>
+      </c>
+      <c r="K561" t="str">
+        <v>S-mu370isd-53lzd</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K547"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K561"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-16T08:19:09.454Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K561"/>
+  <dimension ref="A1:K575"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20034,9 +20034,499 @@
         <v>S-mu370isd-53lzd</v>
       </c>
     </row>
+    <row r="562">
+      <c r="A562" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B562" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C562" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D562" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E562" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F562" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G562" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H562" t="str">
+        <v>N</v>
+      </c>
+      <c r="I562" t="str">
+        <v/>
+      </c>
+      <c r="J562" t="str">
+        <v/>
+      </c>
+      <c r="K562" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B563" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C563" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D563" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E563" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F563" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G563" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H563" t="str">
+        <v>N</v>
+      </c>
+      <c r="I563" t="str">
+        <v/>
+      </c>
+      <c r="J563" t="str">
+        <v/>
+      </c>
+      <c r="K563" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B564" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C564" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D564" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E564" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F564" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G564" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H564" t="str">
+        <v>N</v>
+      </c>
+      <c r="I564" t="str">
+        <v/>
+      </c>
+      <c r="J564" t="str">
+        <v/>
+      </c>
+      <c r="K564" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B565" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C565" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D565" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E565" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F565" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G565" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H565" t="str">
+        <v>N</v>
+      </c>
+      <c r="I565" t="str">
+        <v/>
+      </c>
+      <c r="J565" t="str">
+        <v/>
+      </c>
+      <c r="K565" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B566" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C566" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D566" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E566" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F566" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G566" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H566" t="str">
+        <v>N</v>
+      </c>
+      <c r="I566" t="str">
+        <v/>
+      </c>
+      <c r="J566" t="str">
+        <v/>
+      </c>
+      <c r="K566" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B567" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C567" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D567" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E567" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F567" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G567" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H567" t="str">
+        <v>N</v>
+      </c>
+      <c r="I567" t="str">
+        <v/>
+      </c>
+      <c r="J567" t="str">
+        <v/>
+      </c>
+      <c r="K567" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B568" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C568" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D568" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E568" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F568" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G568" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H568" t="str">
+        <v>N</v>
+      </c>
+      <c r="I568" t="str">
+        <v/>
+      </c>
+      <c r="J568" t="str">
+        <v/>
+      </c>
+      <c r="K568" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B569" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C569" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D569" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E569" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F569" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G569" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H569" t="str">
+        <v>N</v>
+      </c>
+      <c r="I569" t="str">
+        <v/>
+      </c>
+      <c r="J569" t="str">
+        <v/>
+      </c>
+      <c r="K569" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B570" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C570" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D570" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E570" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F570" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G570" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H570" t="str">
+        <v>N</v>
+      </c>
+      <c r="I570" t="str">
+        <v/>
+      </c>
+      <c r="J570" t="str">
+        <v/>
+      </c>
+      <c r="K570" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B571" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C571" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D571" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E571" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F571" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G571" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H571" t="str">
+        <v>N</v>
+      </c>
+      <c r="I571" t="str">
+        <v/>
+      </c>
+      <c r="J571" t="str">
+        <v/>
+      </c>
+      <c r="K571" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B572" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C572" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D572" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E572" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F572" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G572" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H572" t="str">
+        <v>N</v>
+      </c>
+      <c r="I572" t="str">
+        <v/>
+      </c>
+      <c r="J572" t="str">
+        <v/>
+      </c>
+      <c r="K572" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B573" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C573" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D573" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E573" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F573" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G573" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H573" t="str">
+        <v>N</v>
+      </c>
+      <c r="I573" t="str">
+        <v/>
+      </c>
+      <c r="J573" t="str">
+        <v/>
+      </c>
+      <c r="K573" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B574" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C574" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D574" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E574" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F574" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G574" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H574" t="str">
+        <v>N</v>
+      </c>
+      <c r="I574" t="str">
+        <v/>
+      </c>
+      <c r="J574" t="str">
+        <v/>
+      </c>
+      <c r="K574" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="B575" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C575" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D575" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="E575" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="F575" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G575" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H575" t="str">
+        <v>N</v>
+      </c>
+      <c r="I575" t="str">
+        <v/>
+      </c>
+      <c r="J575" t="str">
+        <v/>
+      </c>
+      <c r="K575" t="str">
+        <v>S-mu3txgv2-1ehyl</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K561"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K575"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-16T08:33:48.328Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -19549,16 +19549,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B548" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C548" t="str">
-        <v>07:37</v>
+        <v>(not entered)</v>
       </c>
       <c r="D548" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E548" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F548" t="str">
         <v>Before Startup</v>
@@ -19576,7 +19576,7 @@
         <v/>
       </c>
       <c r="K548" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="549">
@@ -19584,16 +19584,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B549" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C549" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D549" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E549" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F549" t="str">
         <v>Before Startup</v>
@@ -19611,7 +19611,7 @@
         <v/>
       </c>
       <c r="K549" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="550">
@@ -19619,16 +19619,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B550" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C550" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D550" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E550" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F550" t="str">
         <v>Before Startup</v>
@@ -19646,7 +19646,7 @@
         <v/>
       </c>
       <c r="K550" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="551">
@@ -19654,16 +19654,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B551" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C551" t="str">
-        <v>07:37</v>
+        <v>(not entered)</v>
       </c>
       <c r="D551" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E551" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F551" t="str">
         <v>Before Startup</v>
@@ -19672,7 +19672,7 @@
         <v>Check Grecon Tank is on operational level</v>
       </c>
       <c r="H551" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="I551" t="str">
         <v/>
@@ -19681,7 +19681,7 @@
         <v/>
       </c>
       <c r="K551" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="552">
@@ -19689,16 +19689,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B552" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C552" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D552" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E552" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F552" t="str">
         <v>Before Startup</v>
@@ -19716,7 +19716,7 @@
         <v/>
       </c>
       <c r="K552" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="553">
@@ -19724,16 +19724,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B553" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C553" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D553" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E553" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F553" t="str">
         <v>During Processing</v>
@@ -19751,7 +19751,7 @@
         <v/>
       </c>
       <c r="K553" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="554">
@@ -19759,16 +19759,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B554" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C554" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D554" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E554" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F554" t="str">
         <v>During Processing</v>
@@ -19786,7 +19786,7 @@
         <v/>
       </c>
       <c r="K554" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="555">
@@ -19794,16 +19794,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B555" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C555" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D555" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E555" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F555" t="str">
         <v>During Processing</v>
@@ -19821,7 +19821,7 @@
         <v/>
       </c>
       <c r="K555" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="556">
@@ -19829,16 +19829,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B556" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C556" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D556" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E556" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F556" t="str">
         <v>During Processing</v>
@@ -19856,7 +19856,7 @@
         <v/>
       </c>
       <c r="K556" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="557">
@@ -19864,16 +19864,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B557" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C557" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D557" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E557" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F557" t="str">
         <v>During Processing</v>
@@ -19891,7 +19891,7 @@
         <v/>
       </c>
       <c r="K557" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="558">
@@ -19899,16 +19899,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B558" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C558" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D558" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E558" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F558" t="str">
         <v>Once a Week</v>
@@ -19926,7 +19926,7 @@
         <v/>
       </c>
       <c r="K558" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="559">
@@ -19934,16 +19934,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B559" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C559" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D559" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E559" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F559" t="str">
         <v>Once a Week</v>
@@ -19961,7 +19961,7 @@
         <v/>
       </c>
       <c r="K559" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="560">
@@ -19969,16 +19969,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B560" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C560" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D560" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E560" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F560" t="str">
         <v>Once a Week</v>
@@ -19996,7 +19996,7 @@
         <v/>
       </c>
       <c r="K560" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="561">
@@ -20004,16 +20004,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B561" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C561" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D561" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="E561" t="str">
-        <v>tp rp</v>
+        <v>(not entered)</v>
       </c>
       <c r="F561" t="str">
         <v>Once a Week</v>
@@ -20031,7 +20031,7 @@
         <v/>
       </c>
       <c r="K561" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="562">
@@ -20039,16 +20039,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B562" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C562" t="str">
-        <v>(not entered)</v>
+        <v>07:37</v>
       </c>
       <c r="D562" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E562" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F562" t="str">
         <v>Before Startup</v>
@@ -20057,7 +20057,7 @@
         <v>Check Grecon is OK</v>
       </c>
       <c r="H562" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I562" t="str">
         <v/>
@@ -20066,7 +20066,7 @@
         <v/>
       </c>
       <c r="K562" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="563">
@@ -20074,16 +20074,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B563" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C563" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D563" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E563" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F563" t="str">
         <v>Before Startup</v>
@@ -20101,7 +20101,7 @@
         <v/>
       </c>
       <c r="K563" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="564">
@@ -20109,16 +20109,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B564" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C564" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D564" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E564" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F564" t="str">
         <v>Before Startup</v>
@@ -20136,7 +20136,7 @@
         <v/>
       </c>
       <c r="K564" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="565">
@@ -20144,16 +20144,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B565" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C565" t="str">
-        <v>(not entered)</v>
+        <v>07:37</v>
       </c>
       <c r="D565" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E565" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F565" t="str">
         <v>Before Startup</v>
@@ -20162,7 +20162,7 @@
         <v>Check Grecon Tank is on operational level</v>
       </c>
       <c r="H565" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I565" t="str">
         <v/>
@@ -20171,7 +20171,7 @@
         <v/>
       </c>
       <c r="K565" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="566">
@@ -20179,16 +20179,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B566" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C566" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D566" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E566" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F566" t="str">
         <v>Before Startup</v>
@@ -20206,7 +20206,7 @@
         <v/>
       </c>
       <c r="K566" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="567">
@@ -20214,16 +20214,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B567" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C567" t="str">
-        <v>(not entered)</v>
+        <v>10:57</v>
       </c>
       <c r="D567" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E567" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F567" t="str">
         <v>During Processing</v>
@@ -20232,7 +20232,7 @@
         <v>Check Mill Adjustment Sheet is up to date</v>
       </c>
       <c r="H567" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I567" t="str">
         <v/>
@@ -20241,7 +20241,7 @@
         <v/>
       </c>
       <c r="K567" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="568">
@@ -20249,16 +20249,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B568" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C568" t="str">
-        <v>(not entered)</v>
+        <v>10:57</v>
       </c>
       <c r="D568" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E568" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F568" t="str">
         <v>During Processing</v>
@@ -20267,7 +20267,7 @@
         <v>Purge mills — 200 pumps each</v>
       </c>
       <c r="H568" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I568" t="str">
         <v/>
@@ -20276,7 +20276,7 @@
         <v/>
       </c>
       <c r="K568" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="569">
@@ -20284,16 +20284,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B569" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C569" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D569" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E569" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F569" t="str">
         <v>During Processing</v>
@@ -20311,7 +20311,7 @@
         <v/>
       </c>
       <c r="K569" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="570">
@@ -20319,16 +20319,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B570" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C570" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D570" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E570" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F570" t="str">
         <v>During Processing</v>
@@ -20346,7 +20346,7 @@
         <v/>
       </c>
       <c r="K570" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="571">
@@ -20354,16 +20354,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B571" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C571" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D571" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E571" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F571" t="str">
         <v>During Processing</v>
@@ -20381,7 +20381,7 @@
         <v/>
       </c>
       <c r="K571" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="572">
@@ -20389,16 +20389,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B572" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C572" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D572" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E572" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F572" t="str">
         <v>Once a Week</v>
@@ -20416,7 +20416,7 @@
         <v/>
       </c>
       <c r="K572" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="573">
@@ -20424,16 +20424,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B573" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C573" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D573" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E573" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F573" t="str">
         <v>Once a Week</v>
@@ -20451,7 +20451,7 @@
         <v/>
       </c>
       <c r="K573" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="574">
@@ -20459,16 +20459,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B574" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C574" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D574" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E574" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F574" t="str">
         <v>Once a Week</v>
@@ -20486,7 +20486,7 @@
         <v/>
       </c>
       <c r="K574" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="575">
@@ -20494,16 +20494,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B575" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C575" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D575" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E575" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F575" t="str">
         <v>Once a Week</v>
@@ -20521,7 +20521,7 @@
         <v/>
       </c>
       <c r="K575" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checklist log update 2026-09-16T17:15:06.749Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -19549,16 +19549,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B548" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C548" t="str">
-        <v>(not entered)</v>
+        <v>07:37</v>
       </c>
       <c r="D548" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E548" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F548" t="str">
         <v>Before Startup</v>
@@ -19567,7 +19567,7 @@
         <v>Check Grecon is OK</v>
       </c>
       <c r="H548" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I548" t="str">
         <v/>
@@ -19576,7 +19576,7 @@
         <v/>
       </c>
       <c r="K548" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="549">
@@ -19584,16 +19584,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B549" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C549" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D549" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E549" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F549" t="str">
         <v>Before Startup</v>
@@ -19611,7 +19611,7 @@
         <v/>
       </c>
       <c r="K549" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="550">
@@ -19619,16 +19619,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B550" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C550" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D550" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E550" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F550" t="str">
         <v>Before Startup</v>
@@ -19646,7 +19646,7 @@
         <v/>
       </c>
       <c r="K550" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="551">
@@ -19654,16 +19654,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B551" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C551" t="str">
-        <v>(not entered)</v>
+        <v>07:37</v>
       </c>
       <c r="D551" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E551" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F551" t="str">
         <v>Before Startup</v>
@@ -19672,7 +19672,7 @@
         <v>Check Grecon Tank is on operational level</v>
       </c>
       <c r="H551" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I551" t="str">
         <v/>
@@ -19681,7 +19681,7 @@
         <v/>
       </c>
       <c r="K551" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="552">
@@ -19689,16 +19689,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B552" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C552" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D552" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E552" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F552" t="str">
         <v>Before Startup</v>
@@ -19716,7 +19716,7 @@
         <v/>
       </c>
       <c r="K552" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="553">
@@ -19724,16 +19724,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B553" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C553" t="str">
-        <v>(not entered)</v>
+        <v>10:57</v>
       </c>
       <c r="D553" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E553" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F553" t="str">
         <v>During Processing</v>
@@ -19742,7 +19742,7 @@
         <v>Check Mill Adjustment Sheet is up to date</v>
       </c>
       <c r="H553" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I553" t="str">
         <v/>
@@ -19751,7 +19751,7 @@
         <v/>
       </c>
       <c r="K553" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="554">
@@ -19759,16 +19759,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B554" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C554" t="str">
-        <v>(not entered)</v>
+        <v>10:57</v>
       </c>
       <c r="D554" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E554" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F554" t="str">
         <v>During Processing</v>
@@ -19777,7 +19777,7 @@
         <v>Purge mills — 200 pumps each</v>
       </c>
       <c r="H554" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I554" t="str">
         <v/>
@@ -19786,7 +19786,7 @@
         <v/>
       </c>
       <c r="K554" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="555">
@@ -19794,16 +19794,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B555" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C555" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D555" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E555" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F555" t="str">
         <v>During Processing</v>
@@ -19821,7 +19821,7 @@
         <v/>
       </c>
       <c r="K555" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="556">
@@ -19829,16 +19829,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B556" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C556" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D556" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E556" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F556" t="str">
         <v>During Processing</v>
@@ -19856,7 +19856,7 @@
         <v/>
       </c>
       <c r="K556" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="557">
@@ -19864,16 +19864,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B557" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C557" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D557" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E557" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F557" t="str">
         <v>During Processing</v>
@@ -19891,7 +19891,7 @@
         <v/>
       </c>
       <c r="K557" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="558">
@@ -19899,16 +19899,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B558" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C558" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D558" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E558" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F558" t="str">
         <v>Once a Week</v>
@@ -19926,7 +19926,7 @@
         <v/>
       </c>
       <c r="K558" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="559">
@@ -19934,16 +19934,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B559" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C559" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D559" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E559" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F559" t="str">
         <v>Once a Week</v>
@@ -19961,7 +19961,7 @@
         <v/>
       </c>
       <c r="K559" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="560">
@@ -19969,16 +19969,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B560" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C560" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D560" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E560" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F560" t="str">
         <v>Once a Week</v>
@@ -19996,7 +19996,7 @@
         <v/>
       </c>
       <c r="K560" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="561">
@@ -20004,16 +20004,16 @@
         <v>2026-09-16</v>
       </c>
       <c r="B561" t="str">
-        <v>Night</v>
+        <v>Day</v>
       </c>
       <c r="C561" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D561" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="E561" t="str">
-        <v>(not entered)</v>
+        <v>tp rp</v>
       </c>
       <c r="F561" t="str">
         <v>Once a Week</v>
@@ -20031,24 +20031,24 @@
         <v/>
       </c>
       <c r="K561" t="str">
-        <v>S-mu3txgv2-1ehyl</v>
+        <v>S-mu370isd-53lzd</v>
       </c>
     </row>
     <row r="562">
       <c r="A562" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B562" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C562" t="str">
-        <v>07:37</v>
+        <v>18:19</v>
       </c>
       <c r="D562" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E562" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F562" t="str">
         <v>Before Startup</v>
@@ -20066,24 +20066,24 @@
         <v/>
       </c>
       <c r="K562" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="563">
       <c r="A563" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B563" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C563" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D563" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E563" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F563" t="str">
         <v>Before Startup</v>
@@ -20101,24 +20101,24 @@
         <v/>
       </c>
       <c r="K563" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="564">
       <c r="A564" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B564" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C564" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D564" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E564" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F564" t="str">
         <v>Before Startup</v>
@@ -20136,24 +20136,24 @@
         <v/>
       </c>
       <c r="K564" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="565">
       <c r="A565" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B565" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C565" t="str">
-        <v>07:37</v>
+        <v>19:23</v>
       </c>
       <c r="D565" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E565" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F565" t="str">
         <v>Before Startup</v>
@@ -20171,24 +20171,24 @@
         <v/>
       </c>
       <c r="K565" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="566">
       <c r="A566" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B566" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C566" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D566" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E566" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F566" t="str">
         <v>Before Startup</v>
@@ -20206,24 +20206,24 @@
         <v/>
       </c>
       <c r="K566" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="567">
       <c r="A567" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B567" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C567" t="str">
-        <v>10:57</v>
+        <v>18:20</v>
       </c>
       <c r="D567" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E567" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F567" t="str">
         <v>During Processing</v>
@@ -20241,24 +20241,24 @@
         <v/>
       </c>
       <c r="K567" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="568">
       <c r="A568" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B568" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C568" t="str">
-        <v>10:57</v>
+        <v>21:50</v>
       </c>
       <c r="D568" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E568" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F568" t="str">
         <v>During Processing</v>
@@ -20276,24 +20276,24 @@
         <v/>
       </c>
       <c r="K568" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="569">
       <c r="A569" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B569" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C569" t="str">
-        <v>(not entered)</v>
+        <v>03:14</v>
       </c>
       <c r="D569" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E569" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F569" t="str">
         <v>During Processing</v>
@@ -20302,7 +20302,7 @@
         <v>Purge mills — 200 pumps each</v>
       </c>
       <c r="H569" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I569" t="str">
         <v/>
@@ -20311,24 +20311,24 @@
         <v/>
       </c>
       <c r="K569" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="570">
       <c r="A570" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B570" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C570" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D570" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E570" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F570" t="str">
         <v>During Processing</v>
@@ -20346,24 +20346,24 @@
         <v/>
       </c>
       <c r="K570" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="571">
       <c r="A571" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B571" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C571" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D571" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E571" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F571" t="str">
         <v>During Processing</v>
@@ -20381,24 +20381,24 @@
         <v/>
       </c>
       <c r="K571" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="572">
       <c r="A572" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B572" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C572" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D572" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E572" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F572" t="str">
         <v>Once a Week</v>
@@ -20416,24 +20416,24 @@
         <v/>
       </c>
       <c r="K572" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="573">
       <c r="A573" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B573" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C573" t="str">
         <v>(not entered)</v>
       </c>
       <c r="D573" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E573" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F573" t="str">
         <v>Once a Week</v>
@@ -20451,24 +20451,24 @@
         <v/>
       </c>
       <c r="K573" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="574">
       <c r="A574" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B574" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C574" t="str">
-        <v>(not entered)</v>
+        <v>03:15</v>
       </c>
       <c r="D574" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E574" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F574" t="str">
         <v>Once a Week</v>
@@ -20477,33 +20477,33 @@
         <v>Check drinking water tank level</v>
       </c>
       <c r="H574" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I574" t="str">
-        <v/>
+        <v>45%</v>
       </c>
       <c r="J574" t="str">
         <v/>
       </c>
       <c r="K574" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
     <row r="575">
       <c r="A575" t="str">
-        <v>2026-09-16</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B575" t="str">
-        <v>Day</v>
+        <v>Night</v>
       </c>
       <c r="C575" t="str">
-        <v>(not entered)</v>
+        <v>20:19</v>
       </c>
       <c r="D575" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="E575" t="str">
-        <v>tp rp</v>
+        <v>Dylan Anthony Kendell</v>
       </c>
       <c r="F575" t="str">
         <v>Once a Week</v>
@@ -20512,7 +20512,7 @@
         <v>Empty all bins and wheel barrows</v>
       </c>
       <c r="H575" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I575" t="str">
         <v/>
@@ -20521,7 +20521,7 @@
         <v/>
       </c>
       <c r="K575" t="str">
-        <v>S-mu370isd-53lzd</v>
+        <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checklist log update 2026-09-16T19:46:55.439Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -20322,7 +20322,7 @@
         <v>Night</v>
       </c>
       <c r="C570" t="str">
-        <v>(not entered)</v>
+        <v>05:00</v>
       </c>
       <c r="D570" t="str">
         <v>Dylan Anthony Kendell</v>
@@ -20337,7 +20337,7 @@
         <v>Inspect &amp; clean steam vent</v>
       </c>
       <c r="H570" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I570" t="str">
         <v/>
@@ -20357,7 +20357,7 @@
         <v>Night</v>
       </c>
       <c r="C571" t="str">
-        <v>(not entered)</v>
+        <v>05:38</v>
       </c>
       <c r="D571" t="str">
         <v>Dylan Anthony Kendell</v>
@@ -20372,7 +20372,7 @@
         <v>Empty drop box at end of shift</v>
       </c>
       <c r="H571" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I571" t="str">
         <v/>

</xml_diff>

<commit_message>
Checklist log update 2026-09-16T22:53:55.965Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K575"/>
+  <dimension ref="A1:K589"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20524,9 +20524,499 @@
         <v>S-mu3txgv2-1ehyl</v>
       </c>
     </row>
+    <row r="576">
+      <c r="A576" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B576" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C576" t="str">
+        <v>07:02</v>
+      </c>
+      <c r="D576" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E576" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F576" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G576" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H576" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I576" t="str">
+        <v/>
+      </c>
+      <c r="J576" t="str">
+        <v/>
+      </c>
+      <c r="K576" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B577" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C577" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D577" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E577" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F577" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G577" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H577" t="str">
+        <v>N</v>
+      </c>
+      <c r="I577" t="str">
+        <v/>
+      </c>
+      <c r="J577" t="str">
+        <v/>
+      </c>
+      <c r="K577" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B578" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C578" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D578" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E578" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F578" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G578" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H578" t="str">
+        <v>N</v>
+      </c>
+      <c r="I578" t="str">
+        <v/>
+      </c>
+      <c r="J578" t="str">
+        <v/>
+      </c>
+      <c r="K578" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B579" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C579" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D579" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E579" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F579" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G579" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H579" t="str">
+        <v>N</v>
+      </c>
+      <c r="I579" t="str">
+        <v/>
+      </c>
+      <c r="J579" t="str">
+        <v/>
+      </c>
+      <c r="K579" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B580" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C580" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D580" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E580" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F580" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G580" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H580" t="str">
+        <v>N</v>
+      </c>
+      <c r="I580" t="str">
+        <v/>
+      </c>
+      <c r="J580" t="str">
+        <v/>
+      </c>
+      <c r="K580" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B581" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C581" t="str">
+        <v>07:02</v>
+      </c>
+      <c r="D581" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E581" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F581" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G581" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H581" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I581" t="str">
+        <v/>
+      </c>
+      <c r="J581" t="str">
+        <v/>
+      </c>
+      <c r="K581" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B582" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C582" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D582" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E582" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F582" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G582" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H582" t="str">
+        <v>N</v>
+      </c>
+      <c r="I582" t="str">
+        <v/>
+      </c>
+      <c r="J582" t="str">
+        <v/>
+      </c>
+      <c r="K582" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B583" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C583" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D583" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E583" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F583" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G583" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H583" t="str">
+        <v>N</v>
+      </c>
+      <c r="I583" t="str">
+        <v/>
+      </c>
+      <c r="J583" t="str">
+        <v/>
+      </c>
+      <c r="K583" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B584" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C584" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D584" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E584" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F584" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G584" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H584" t="str">
+        <v>N</v>
+      </c>
+      <c r="I584" t="str">
+        <v/>
+      </c>
+      <c r="J584" t="str">
+        <v/>
+      </c>
+      <c r="K584" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B585" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C585" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D585" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E585" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F585" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G585" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H585" t="str">
+        <v>N</v>
+      </c>
+      <c r="I585" t="str">
+        <v/>
+      </c>
+      <c r="J585" t="str">
+        <v/>
+      </c>
+      <c r="K585" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B586" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C586" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D586" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E586" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F586" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G586" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H586" t="str">
+        <v>N</v>
+      </c>
+      <c r="I586" t="str">
+        <v/>
+      </c>
+      <c r="J586" t="str">
+        <v/>
+      </c>
+      <c r="K586" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B587" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C587" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D587" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E587" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F587" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G587" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H587" t="str">
+        <v>N</v>
+      </c>
+      <c r="I587" t="str">
+        <v/>
+      </c>
+      <c r="J587" t="str">
+        <v/>
+      </c>
+      <c r="K587" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B588" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C588" t="str">
+        <v>07:03</v>
+      </c>
+      <c r="D588" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E588" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F588" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G588" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H588" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I588" t="str">
+        <v>42%</v>
+      </c>
+      <c r="J588" t="str">
+        <v/>
+      </c>
+      <c r="K588" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="B589" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C589" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D589" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E589" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F589" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G589" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H589" t="str">
+        <v>N</v>
+      </c>
+      <c r="I589" t="str">
+        <v/>
+      </c>
+      <c r="J589" t="str">
+        <v/>
+      </c>
+      <c r="K589" t="str">
+        <v>S-mu4l6mv6-kuucc</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K575"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K589"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-17T18:07:55.510Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K589"/>
+  <dimension ref="A1:K603"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -21014,9 +21014,499 @@
         <v>S-mu4l6mv6-kuucc</v>
       </c>
     </row>
+    <row r="590">
+      <c r="A590" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B590" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C590" t="str">
+        <v>18:04</v>
+      </c>
+      <c r="D590" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E590" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F590" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G590" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H590" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I590" t="str">
+        <v/>
+      </c>
+      <c r="J590" t="str">
+        <v/>
+      </c>
+      <c r="K590" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B591" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C591" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D591" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E591" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F591" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G591" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H591" t="str">
+        <v>N</v>
+      </c>
+      <c r="I591" t="str">
+        <v/>
+      </c>
+      <c r="J591" t="str">
+        <v/>
+      </c>
+      <c r="K591" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B592" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C592" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D592" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E592" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F592" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G592" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H592" t="str">
+        <v>N</v>
+      </c>
+      <c r="I592" t="str">
+        <v/>
+      </c>
+      <c r="J592" t="str">
+        <v/>
+      </c>
+      <c r="K592" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B593" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C593" t="str">
+        <v>18:05</v>
+      </c>
+      <c r="D593" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E593" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F593" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G593" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H593" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I593" t="str">
+        <v/>
+      </c>
+      <c r="J593" t="str">
+        <v/>
+      </c>
+      <c r="K593" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B594" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C594" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D594" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E594" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F594" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G594" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H594" t="str">
+        <v>N</v>
+      </c>
+      <c r="I594" t="str">
+        <v/>
+      </c>
+      <c r="J594" t="str">
+        <v/>
+      </c>
+      <c r="K594" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B595" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C595" t="str">
+        <v>18:04</v>
+      </c>
+      <c r="D595" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E595" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F595" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G595" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H595" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I595" t="str">
+        <v/>
+      </c>
+      <c r="J595" t="str">
+        <v/>
+      </c>
+      <c r="K595" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B596" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C596" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="D596" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E596" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F596" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G596" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H596" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I596" t="str">
+        <v/>
+      </c>
+      <c r="J596" t="str">
+        <v/>
+      </c>
+      <c r="K596" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B597" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C597" t="str">
+        <v>03:40</v>
+      </c>
+      <c r="D597" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E597" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F597" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G597" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H597" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I597" t="str">
+        <v/>
+      </c>
+      <c r="J597" t="str">
+        <v/>
+      </c>
+      <c r="K597" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B598" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C598" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D598" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E598" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F598" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G598" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H598" t="str">
+        <v>N</v>
+      </c>
+      <c r="I598" t="str">
+        <v/>
+      </c>
+      <c r="J598" t="str">
+        <v/>
+      </c>
+      <c r="K598" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B599" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C599" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D599" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E599" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F599" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G599" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H599" t="str">
+        <v>N</v>
+      </c>
+      <c r="I599" t="str">
+        <v/>
+      </c>
+      <c r="J599" t="str">
+        <v/>
+      </c>
+      <c r="K599" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B600" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C600" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D600" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E600" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F600" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G600" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H600" t="str">
+        <v>N</v>
+      </c>
+      <c r="I600" t="str">
+        <v/>
+      </c>
+      <c r="J600" t="str">
+        <v/>
+      </c>
+      <c r="K600" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B601" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C601" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D601" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E601" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F601" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G601" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H601" t="str">
+        <v>N</v>
+      </c>
+      <c r="I601" t="str">
+        <v/>
+      </c>
+      <c r="J601" t="str">
+        <v/>
+      </c>
+      <c r="K601" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B602" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C602" t="str">
+        <v>20:59</v>
+      </c>
+      <c r="D602" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E602" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F602" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G602" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H602" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I602" t="str">
+        <v/>
+      </c>
+      <c r="J602" t="str">
+        <v/>
+      </c>
+      <c r="K602" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B603" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C603" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D603" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E603" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F603" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G603" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H603" t="str">
+        <v>N</v>
+      </c>
+      <c r="I603" t="str">
+        <v/>
+      </c>
+      <c r="J603" t="str">
+        <v/>
+      </c>
+      <c r="K603" t="str">
+        <v>S-mu5ueegg-wfhd9</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K589"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K603"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-18T05:51:31.498Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K603"/>
+  <dimension ref="A1:K617"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -21504,9 +21504,499 @@
         <v>S-mu5ueegg-wfhd9</v>
       </c>
     </row>
+    <row r="604">
+      <c r="A604" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B604" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C604" t="str">
+        <v>15:51</v>
+      </c>
+      <c r="D604" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E604" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F604" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G604" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H604" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I604" t="str">
+        <v/>
+      </c>
+      <c r="J604" t="str">
+        <v/>
+      </c>
+      <c r="K604" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B605" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C605" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D605" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E605" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F605" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G605" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H605" t="str">
+        <v>N</v>
+      </c>
+      <c r="I605" t="str">
+        <v/>
+      </c>
+      <c r="J605" t="str">
+        <v/>
+      </c>
+      <c r="K605" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B606" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C606" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D606" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E606" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F606" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G606" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H606" t="str">
+        <v>N</v>
+      </c>
+      <c r="I606" t="str">
+        <v/>
+      </c>
+      <c r="J606" t="str">
+        <v/>
+      </c>
+      <c r="K606" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B607" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C607" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D607" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E607" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F607" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G607" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H607" t="str">
+        <v>N</v>
+      </c>
+      <c r="I607" t="str">
+        <v/>
+      </c>
+      <c r="J607" t="str">
+        <v/>
+      </c>
+      <c r="K607" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B608" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C608" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D608" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E608" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F608" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G608" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H608" t="str">
+        <v>N</v>
+      </c>
+      <c r="I608" t="str">
+        <v/>
+      </c>
+      <c r="J608" t="str">
+        <v/>
+      </c>
+      <c r="K608" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B609" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C609" t="str">
+        <v>15:51</v>
+      </c>
+      <c r="D609" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E609" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F609" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G609" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H609" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I609" t="str">
+        <v/>
+      </c>
+      <c r="J609" t="str">
+        <v/>
+      </c>
+      <c r="K609" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B610" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C610" t="str">
+        <v>09:51</v>
+      </c>
+      <c r="D610" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E610" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F610" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G610" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H610" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I610" t="str">
+        <v/>
+      </c>
+      <c r="J610" t="str">
+        <v/>
+      </c>
+      <c r="K610" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B611" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C611" t="str">
+        <v>15:51</v>
+      </c>
+      <c r="D611" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E611" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F611" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G611" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H611" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I611" t="str">
+        <v/>
+      </c>
+      <c r="J611" t="str">
+        <v/>
+      </c>
+      <c r="K611" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B612" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C612" t="str">
+        <v>16:51</v>
+      </c>
+      <c r="D612" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E612" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F612" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G612" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H612" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I612" t="str">
+        <v/>
+      </c>
+      <c r="J612" t="str">
+        <v/>
+      </c>
+      <c r="K612" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B613" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C613" t="str">
+        <v>15:51</v>
+      </c>
+      <c r="D613" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E613" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F613" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G613" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H613" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I613" t="str">
+        <v/>
+      </c>
+      <c r="J613" t="str">
+        <v/>
+      </c>
+      <c r="K613" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B614" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C614" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D614" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E614" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F614" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G614" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H614" t="str">
+        <v>N</v>
+      </c>
+      <c r="I614" t="str">
+        <v/>
+      </c>
+      <c r="J614" t="str">
+        <v/>
+      </c>
+      <c r="K614" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B615" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C615" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D615" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E615" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F615" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G615" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H615" t="str">
+        <v>N</v>
+      </c>
+      <c r="I615" t="str">
+        <v/>
+      </c>
+      <c r="J615" t="str">
+        <v/>
+      </c>
+      <c r="K615" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B616" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C616" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D616" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E616" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F616" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G616" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H616" t="str">
+        <v>N</v>
+      </c>
+      <c r="I616" t="str">
+        <v/>
+      </c>
+      <c r="J616" t="str">
+        <v/>
+      </c>
+      <c r="K616" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B617" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C617" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D617" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E617" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F617" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G617" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H617" t="str">
+        <v>N</v>
+      </c>
+      <c r="I617" t="str">
+        <v/>
+      </c>
+      <c r="J617" t="str">
+        <v/>
+      </c>
+      <c r="K617" t="str">
+        <v>S-mu5uedko-tls3d</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K603"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K617"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-18T11:20:34.533Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K617"/>
+  <dimension ref="A1:K631"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -21994,9 +21994,499 @@
         <v>S-mu5uedko-tls3d</v>
       </c>
     </row>
+    <row r="618">
+      <c r="A618" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B618" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C618" t="str">
+        <v>18:17</v>
+      </c>
+      <c r="D618" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E618" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F618" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G618" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H618" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I618" t="str">
+        <v/>
+      </c>
+      <c r="J618" t="str">
+        <v/>
+      </c>
+      <c r="K618" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B619" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C619" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D619" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E619" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F619" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G619" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H619" t="str">
+        <v>N</v>
+      </c>
+      <c r="I619" t="str">
+        <v/>
+      </c>
+      <c r="J619" t="str">
+        <v/>
+      </c>
+      <c r="K619" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B620" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C620" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D620" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E620" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F620" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G620" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H620" t="str">
+        <v>N</v>
+      </c>
+      <c r="I620" t="str">
+        <v/>
+      </c>
+      <c r="J620" t="str">
+        <v/>
+      </c>
+      <c r="K620" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B621" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C621" t="str">
+        <v>18:18</v>
+      </c>
+      <c r="D621" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E621" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F621" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G621" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H621" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I621" t="str">
+        <v/>
+      </c>
+      <c r="J621" t="str">
+        <v/>
+      </c>
+      <c r="K621" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B622" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C622" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D622" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E622" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F622" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G622" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H622" t="str">
+        <v>N</v>
+      </c>
+      <c r="I622" t="str">
+        <v/>
+      </c>
+      <c r="J622" t="str">
+        <v/>
+      </c>
+      <c r="K622" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B623" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C623" t="str">
+        <v>18:20</v>
+      </c>
+      <c r="D623" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E623" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F623" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G623" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H623" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I623" t="str">
+        <v/>
+      </c>
+      <c r="J623" t="str">
+        <v/>
+      </c>
+      <c r="K623" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B624" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C624" t="str">
+        <v>21:20</v>
+      </c>
+      <c r="D624" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E624" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F624" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G624" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H624" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I624" t="str">
+        <v/>
+      </c>
+      <c r="J624" t="str">
+        <v/>
+      </c>
+      <c r="K624" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B625" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C625" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D625" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E625" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F625" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G625" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H625" t="str">
+        <v>N</v>
+      </c>
+      <c r="I625" t="str">
+        <v/>
+      </c>
+      <c r="J625" t="str">
+        <v/>
+      </c>
+      <c r="K625" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B626" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C626" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D626" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E626" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F626" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G626" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H626" t="str">
+        <v>N</v>
+      </c>
+      <c r="I626" t="str">
+        <v/>
+      </c>
+      <c r="J626" t="str">
+        <v/>
+      </c>
+      <c r="K626" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B627" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C627" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D627" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E627" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F627" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G627" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H627" t="str">
+        <v>N</v>
+      </c>
+      <c r="I627" t="str">
+        <v/>
+      </c>
+      <c r="J627" t="str">
+        <v/>
+      </c>
+      <c r="K627" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B628" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C628" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D628" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E628" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F628" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G628" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H628" t="str">
+        <v>N</v>
+      </c>
+      <c r="I628" t="str">
+        <v/>
+      </c>
+      <c r="J628" t="str">
+        <v/>
+      </c>
+      <c r="K628" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B629" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C629" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D629" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E629" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F629" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G629" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H629" t="str">
+        <v>N</v>
+      </c>
+      <c r="I629" t="str">
+        <v/>
+      </c>
+      <c r="J629" t="str">
+        <v/>
+      </c>
+      <c r="K629" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B630" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C630" t="str">
+        <v>18:31</v>
+      </c>
+      <c r="D630" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E630" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F630" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G630" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H630" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I630" t="str">
+        <v>35%</v>
+      </c>
+      <c r="J630" t="str">
+        <v/>
+      </c>
+      <c r="K630" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B631" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C631" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D631" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E631" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F631" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G631" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H631" t="str">
+        <v>N</v>
+      </c>
+      <c r="I631" t="str">
+        <v/>
+      </c>
+      <c r="J631" t="str">
+        <v/>
+      </c>
+      <c r="K631" t="str">
+        <v>S-mu6oqcnx-g3417</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K617"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K631"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-19T09:56:35.329Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K631"/>
+  <dimension ref="A1:K645"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -22484,9 +22484,499 @@
         <v>S-mu6oqcnx-g3417</v>
       </c>
     </row>
+    <row r="632">
+      <c r="A632" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B632" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C632" t="str">
+        <v>18:17</v>
+      </c>
+      <c r="D632" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E632" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F632" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G632" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H632" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I632" t="str">
+        <v/>
+      </c>
+      <c r="J632" t="str">
+        <v/>
+      </c>
+      <c r="K632" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B633" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C633" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D633" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E633" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F633" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G633" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H633" t="str">
+        <v>N</v>
+      </c>
+      <c r="I633" t="str">
+        <v/>
+      </c>
+      <c r="J633" t="str">
+        <v/>
+      </c>
+      <c r="K633" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B634" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C634" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D634" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E634" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F634" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G634" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H634" t="str">
+        <v>N</v>
+      </c>
+      <c r="I634" t="str">
+        <v/>
+      </c>
+      <c r="J634" t="str">
+        <v/>
+      </c>
+      <c r="K634" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B635" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C635" t="str">
+        <v>18:18</v>
+      </c>
+      <c r="D635" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E635" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F635" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G635" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H635" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I635" t="str">
+        <v/>
+      </c>
+      <c r="J635" t="str">
+        <v/>
+      </c>
+      <c r="K635" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B636" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C636" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D636" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E636" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F636" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G636" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H636" t="str">
+        <v>N</v>
+      </c>
+      <c r="I636" t="str">
+        <v/>
+      </c>
+      <c r="J636" t="str">
+        <v/>
+      </c>
+      <c r="K636" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B637" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C637" t="str">
+        <v>18:20</v>
+      </c>
+      <c r="D637" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E637" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F637" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G637" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H637" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I637" t="str">
+        <v/>
+      </c>
+      <c r="J637" t="str">
+        <v/>
+      </c>
+      <c r="K637" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B638" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C638" t="str">
+        <v>21:20</v>
+      </c>
+      <c r="D638" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E638" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F638" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G638" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H638" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I638" t="str">
+        <v/>
+      </c>
+      <c r="J638" t="str">
+        <v/>
+      </c>
+      <c r="K638" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B639" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C639" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D639" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E639" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F639" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G639" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H639" t="str">
+        <v>N</v>
+      </c>
+      <c r="I639" t="str">
+        <v/>
+      </c>
+      <c r="J639" t="str">
+        <v/>
+      </c>
+      <c r="K639" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B640" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C640" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D640" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E640" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F640" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G640" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H640" t="str">
+        <v>N</v>
+      </c>
+      <c r="I640" t="str">
+        <v/>
+      </c>
+      <c r="J640" t="str">
+        <v/>
+      </c>
+      <c r="K640" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B641" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C641" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D641" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E641" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F641" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G641" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H641" t="str">
+        <v>N</v>
+      </c>
+      <c r="I641" t="str">
+        <v/>
+      </c>
+      <c r="J641" t="str">
+        <v/>
+      </c>
+      <c r="K641" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B642" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C642" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D642" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E642" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F642" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G642" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H642" t="str">
+        <v>N</v>
+      </c>
+      <c r="I642" t="str">
+        <v/>
+      </c>
+      <c r="J642" t="str">
+        <v/>
+      </c>
+      <c r="K642" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B643" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C643" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D643" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E643" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F643" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G643" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H643" t="str">
+        <v>N</v>
+      </c>
+      <c r="I643" t="str">
+        <v/>
+      </c>
+      <c r="J643" t="str">
+        <v/>
+      </c>
+      <c r="K643" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B644" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C644" t="str">
+        <v>18:31</v>
+      </c>
+      <c r="D644" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E644" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F644" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G644" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H644" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I644" t="str">
+        <v>35%</v>
+      </c>
+      <c r="J644" t="str">
+        <v/>
+      </c>
+      <c r="K644" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B645" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C645" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D645" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="E645" t="str">
+        <v>DH KEN</v>
+      </c>
+      <c r="F645" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G645" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H645" t="str">
+        <v>N</v>
+      </c>
+      <c r="I645" t="str">
+        <v/>
+      </c>
+      <c r="J645" t="str">
+        <v/>
+      </c>
+      <c r="K645" t="str">
+        <v>S-mu84kfc9-unl8w</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K631"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K645"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-19T19:40:03.716Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K645"/>
+  <dimension ref="A1:K659"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -22974,9 +22974,499 @@
         <v>S-mu84kfc9-unl8w</v>
       </c>
     </row>
+    <row r="646">
+      <c r="A646" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B646" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C646" t="str">
+        <v>18:44</v>
+      </c>
+      <c r="D646" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E646" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F646" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G646" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H646" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I646" t="str">
+        <v/>
+      </c>
+      <c r="J646" t="str">
+        <v/>
+      </c>
+      <c r="K646" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B647" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C647" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D647" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E647" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F647" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G647" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H647" t="str">
+        <v>N</v>
+      </c>
+      <c r="I647" t="str">
+        <v/>
+      </c>
+      <c r="J647" t="str">
+        <v/>
+      </c>
+      <c r="K647" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B648" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C648" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D648" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E648" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F648" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G648" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H648" t="str">
+        <v>N</v>
+      </c>
+      <c r="I648" t="str">
+        <v/>
+      </c>
+      <c r="J648" t="str">
+        <v/>
+      </c>
+      <c r="K648" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B649" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C649" t="str">
+        <v>18:47</v>
+      </c>
+      <c r="D649" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E649" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F649" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G649" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H649" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I649" t="str">
+        <v/>
+      </c>
+      <c r="J649" t="str">
+        <v/>
+      </c>
+      <c r="K649" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B650" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C650" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D650" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E650" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F650" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G650" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H650" t="str">
+        <v>N</v>
+      </c>
+      <c r="I650" t="str">
+        <v/>
+      </c>
+      <c r="J650" t="str">
+        <v/>
+      </c>
+      <c r="K650" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B651" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C651" t="str">
+        <v>19:03</v>
+      </c>
+      <c r="D651" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E651" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F651" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G651" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H651" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I651" t="str">
+        <v/>
+      </c>
+      <c r="J651" t="str">
+        <v/>
+      </c>
+      <c r="K651" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B652" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C652" t="str">
+        <v>21:22</v>
+      </c>
+      <c r="D652" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E652" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F652" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G652" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H652" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I652" t="str">
+        <v>changed drum at 7:45pm</v>
+      </c>
+      <c r="J652" t="str">
+        <v/>
+      </c>
+      <c r="K652" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B653" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C653" t="str">
+        <v>04:40</v>
+      </c>
+      <c r="D653" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E653" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F653" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G653" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H653" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I653" t="str">
+        <v/>
+      </c>
+      <c r="J653" t="str">
+        <v/>
+      </c>
+      <c r="K653" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B654" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C654" t="str">
+        <v>05:39</v>
+      </c>
+      <c r="D654" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E654" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F654" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G654" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H654" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I654" t="str">
+        <v/>
+      </c>
+      <c r="J654" t="str">
+        <v/>
+      </c>
+      <c r="K654" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B655" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C655" t="str">
+        <v>05:32</v>
+      </c>
+      <c r="D655" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E655" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F655" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G655" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H655" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I655" t="str">
+        <v/>
+      </c>
+      <c r="J655" t="str">
+        <v/>
+      </c>
+      <c r="K655" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B656" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C656" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D656" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E656" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F656" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G656" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H656" t="str">
+        <v>N</v>
+      </c>
+      <c r="I656" t="str">
+        <v/>
+      </c>
+      <c r="J656" t="str">
+        <v/>
+      </c>
+      <c r="K656" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B657" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C657" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D657" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E657" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F657" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G657" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H657" t="str">
+        <v>N</v>
+      </c>
+      <c r="I657" t="str">
+        <v/>
+      </c>
+      <c r="J657" t="str">
+        <v/>
+      </c>
+      <c r="K657" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B658" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C658" t="str">
+        <v>19:57</v>
+      </c>
+      <c r="D658" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E658" t="str">
+        <v>Dyl</v>
+      </c>
+      <c r="F658" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G658" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H658" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I658" t="str">
+        <v>30%</v>
+      </c>
+      <c r="J658" t="str">
+        <v/>
+      </c>
+      <c r="K658" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B659" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C659" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D659" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E659" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F659" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G659" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H659" t="str">
+        <v>N</v>
+      </c>
+      <c r="I659" t="str">
+        <v/>
+      </c>
+      <c r="J659" t="str">
+        <v/>
+      </c>
+      <c r="K659" t="str">
+        <v>S-mu8m75ez-d2tgx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K645"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K659"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-20T06:34:19.106Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K659"/>
+  <dimension ref="A1:K673"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -23464,9 +23464,499 @@
         <v>S-mu8m75ez-d2tgx</v>
       </c>
     </row>
+    <row r="660">
+      <c r="A660" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B660" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C660" t="str">
+        <v>09:31</v>
+      </c>
+      <c r="D660" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E660" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F660" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G660" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H660" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I660" t="str">
+        <v/>
+      </c>
+      <c r="J660" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K660" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B661" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C661" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D661" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E661" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F661" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G661" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H661" t="str">
+        <v>N</v>
+      </c>
+      <c r="I661" t="str">
+        <v/>
+      </c>
+      <c r="J661" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K661" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B662" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C662" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D662" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E662" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F662" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G662" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H662" t="str">
+        <v>N</v>
+      </c>
+      <c r="I662" t="str">
+        <v/>
+      </c>
+      <c r="J662" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K662" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B663" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C663" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D663" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E663" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F663" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G663" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H663" t="str">
+        <v>N</v>
+      </c>
+      <c r="I663" t="str">
+        <v/>
+      </c>
+      <c r="J663" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K663" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B664" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C664" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D664" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E664" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F664" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G664" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H664" t="str">
+        <v>N</v>
+      </c>
+      <c r="I664" t="str">
+        <v/>
+      </c>
+      <c r="J664" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K664" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B665" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C665" t="str">
+        <v>16:31</v>
+      </c>
+      <c r="D665" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E665" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F665" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G665" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H665" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I665" t="str">
+        <v/>
+      </c>
+      <c r="J665" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K665" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B666" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C666" t="str">
+        <v>10:32</v>
+      </c>
+      <c r="D666" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E666" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F666" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G666" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H666" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I666" t="str">
+        <v/>
+      </c>
+      <c r="J666" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K666" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B667" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C667" t="str">
+        <v>15:32</v>
+      </c>
+      <c r="D667" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E667" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F667" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G667" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H667" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I667" t="str">
+        <v/>
+      </c>
+      <c r="J667" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K667" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B668" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C668" t="str">
+        <v>16:32</v>
+      </c>
+      <c r="D668" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E668" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F668" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G668" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H668" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I668" t="str">
+        <v/>
+      </c>
+      <c r="J668" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K668" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B669" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C669" t="str">
+        <v>16:32</v>
+      </c>
+      <c r="D669" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E669" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F669" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G669" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H669" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I669" t="str">
+        <v/>
+      </c>
+      <c r="J669" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K669" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B670" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C670" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D670" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E670" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F670" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G670" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H670" t="str">
+        <v>N</v>
+      </c>
+      <c r="I670" t="str">
+        <v/>
+      </c>
+      <c r="J670" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K670" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B671" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C671" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D671" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E671" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F671" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G671" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H671" t="str">
+        <v>N</v>
+      </c>
+      <c r="I671" t="str">
+        <v/>
+      </c>
+      <c r="J671" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K671" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B672" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C672" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D672" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E672" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F672" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G672" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H672" t="str">
+        <v>N</v>
+      </c>
+      <c r="I672" t="str">
+        <v/>
+      </c>
+      <c r="J672" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K672" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B673" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C673" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D673" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="E673" t="str">
+        <v>TP TS</v>
+      </c>
+      <c r="F673" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G673" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H673" t="str">
+        <v>N</v>
+      </c>
+      <c r="I673" t="str">
+        <v/>
+      </c>
+      <c r="J673" t="str">
+        <v>Shut down due to no fiber, blew out all mills and cleaned dust around the mills. "Not a deep clean". Emptied Bunker due to hammer mill blocking early on shift. Cleaned down the ring road.</v>
+      </c>
+      <c r="K673" t="str">
+        <v>S-mu8m71j1-l85c1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K659"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K673"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-21T02:40:53.538Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K673"/>
+  <dimension ref="A1:K687"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -23954,9 +23954,499 @@
         <v>S-mu8m71j1-l85c1</v>
       </c>
     </row>
+    <row r="674">
+      <c r="A674" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B674" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C674" t="str">
+        <v>07:45</v>
+      </c>
+      <c r="D674" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E674" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F674" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G674" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H674" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I674" t="str">
+        <v/>
+      </c>
+      <c r="J674" t="str">
+        <v/>
+      </c>
+      <c r="K674" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B675" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C675" t="str">
+        <v>07:45</v>
+      </c>
+      <c r="D675" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E675" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F675" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G675" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H675" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I675" t="str">
+        <v/>
+      </c>
+      <c r="J675" t="str">
+        <v/>
+      </c>
+      <c r="K675" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B676" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C676" t="str">
+        <v>07:45</v>
+      </c>
+      <c r="D676" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E676" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F676" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G676" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H676" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I676" t="str">
+        <v/>
+      </c>
+      <c r="J676" t="str">
+        <v/>
+      </c>
+      <c r="K676" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B677" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C677" t="str">
+        <v>07:28</v>
+      </c>
+      <c r="D677" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E677" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F677" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G677" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H677" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I677" t="str">
+        <v/>
+      </c>
+      <c r="J677" t="str">
+        <v/>
+      </c>
+      <c r="K677" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B678" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C678" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D678" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E678" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F678" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G678" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H678" t="str">
+        <v>N</v>
+      </c>
+      <c r="I678" t="str">
+        <v/>
+      </c>
+      <c r="J678" t="str">
+        <v/>
+      </c>
+      <c r="K678" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B679" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C679" t="str">
+        <v>06:45</v>
+      </c>
+      <c r="D679" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E679" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F679" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G679" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H679" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I679" t="str">
+        <v/>
+      </c>
+      <c r="J679" t="str">
+        <v/>
+      </c>
+      <c r="K679" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B680" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C680" t="str">
+        <v>12:39</v>
+      </c>
+      <c r="D680" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E680" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F680" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G680" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H680" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I680" t="str">
+        <v>Purged late as late start-up, purged accordingly.</v>
+      </c>
+      <c r="J680" t="str">
+        <v/>
+      </c>
+      <c r="K680" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B681" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C681" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D681" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E681" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F681" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G681" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H681" t="str">
+        <v>N</v>
+      </c>
+      <c r="I681" t="str">
+        <v/>
+      </c>
+      <c r="J681" t="str">
+        <v/>
+      </c>
+      <c r="K681" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B682" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C682" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D682" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E682" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F682" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G682" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H682" t="str">
+        <v>N</v>
+      </c>
+      <c r="I682" t="str">
+        <v/>
+      </c>
+      <c r="J682" t="str">
+        <v/>
+      </c>
+      <c r="K682" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B683" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C683" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D683" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E683" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F683" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G683" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H683" t="str">
+        <v>N</v>
+      </c>
+      <c r="I683" t="str">
+        <v/>
+      </c>
+      <c r="J683" t="str">
+        <v/>
+      </c>
+      <c r="K683" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B684" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C684" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D684" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E684" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F684" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G684" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H684" t="str">
+        <v>N</v>
+      </c>
+      <c r="I684" t="str">
+        <v/>
+      </c>
+      <c r="J684" t="str">
+        <v/>
+      </c>
+      <c r="K684" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B685" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C685" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D685" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E685" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F685" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G685" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H685" t="str">
+        <v>N</v>
+      </c>
+      <c r="I685" t="str">
+        <v/>
+      </c>
+      <c r="J685" t="str">
+        <v/>
+      </c>
+      <c r="K685" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B686" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C686" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D686" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E686" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F686" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G686" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H686" t="str">
+        <v>N</v>
+      </c>
+      <c r="I686" t="str">
+        <v/>
+      </c>
+      <c r="J686" t="str">
+        <v/>
+      </c>
+      <c r="K686" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B687" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C687" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D687" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E687" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F687" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G687" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H687" t="str">
+        <v>N</v>
+      </c>
+      <c r="I687" t="str">
+        <v/>
+      </c>
+      <c r="J687" t="str">
+        <v/>
+      </c>
+      <c r="K687" t="str">
+        <v>S-muacgyuy-b8yh8</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K673"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K687"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-21T21:51:31.153Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K687"/>
+  <dimension ref="A1:K701"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -24444,9 +24444,499 @@
         <v>S-muacgyuy-b8yh8</v>
       </c>
     </row>
+    <row r="688">
+      <c r="A688" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B688" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C688" t="str">
+        <v>07:45</v>
+      </c>
+      <c r="D688" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E688" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F688" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G688" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H688" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I688" t="str">
+        <v/>
+      </c>
+      <c r="J688" t="str">
+        <v/>
+      </c>
+      <c r="K688" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B689" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C689" t="str">
+        <v>07:45</v>
+      </c>
+      <c r="D689" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E689" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F689" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G689" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H689" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I689" t="str">
+        <v/>
+      </c>
+      <c r="J689" t="str">
+        <v/>
+      </c>
+      <c r="K689" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B690" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C690" t="str">
+        <v>07:45</v>
+      </c>
+      <c r="D690" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E690" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F690" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G690" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H690" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I690" t="str">
+        <v/>
+      </c>
+      <c r="J690" t="str">
+        <v/>
+      </c>
+      <c r="K690" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B691" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C691" t="str">
+        <v>07:28</v>
+      </c>
+      <c r="D691" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E691" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F691" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G691" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H691" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I691" t="str">
+        <v/>
+      </c>
+      <c r="J691" t="str">
+        <v/>
+      </c>
+      <c r="K691" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B692" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C692" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D692" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E692" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F692" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G692" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H692" t="str">
+        <v>N</v>
+      </c>
+      <c r="I692" t="str">
+        <v/>
+      </c>
+      <c r="J692" t="str">
+        <v/>
+      </c>
+      <c r="K692" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B693" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C693" t="str">
+        <v>06:45</v>
+      </c>
+      <c r="D693" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E693" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F693" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G693" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H693" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I693" t="str">
+        <v/>
+      </c>
+      <c r="J693" t="str">
+        <v/>
+      </c>
+      <c r="K693" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B694" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C694" t="str">
+        <v>12:39</v>
+      </c>
+      <c r="D694" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E694" t="str">
+        <v>AS</v>
+      </c>
+      <c r="F694" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G694" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H694" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I694" t="str">
+        <v>Purged late as late start-up, purged accordingly.</v>
+      </c>
+      <c r="J694" t="str">
+        <v/>
+      </c>
+      <c r="K694" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B695" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C695" t="str">
+        <v>15:38</v>
+      </c>
+      <c r="D695" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E695" t="str">
+        <v>KB</v>
+      </c>
+      <c r="F695" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G695" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H695" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I695" t="str">
+        <v>only put 100 pumps</v>
+      </c>
+      <c r="J695" t="str">
+        <v/>
+      </c>
+      <c r="K695" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B696" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C696" t="str">
+        <v>16:27</v>
+      </c>
+      <c r="D696" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E696" t="str">
+        <v>TR</v>
+      </c>
+      <c r="F696" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G696" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H696" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I696" t="str">
+        <v/>
+      </c>
+      <c r="J696" t="str">
+        <v/>
+      </c>
+      <c r="K696" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B697" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C697" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D697" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E697" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F697" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G697" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H697" t="str">
+        <v>N</v>
+      </c>
+      <c r="I697" t="str">
+        <v/>
+      </c>
+      <c r="J697" t="str">
+        <v/>
+      </c>
+      <c r="K697" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B698" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C698" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D698" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E698" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F698" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G698" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H698" t="str">
+        <v>N</v>
+      </c>
+      <c r="I698" t="str">
+        <v/>
+      </c>
+      <c r="J698" t="str">
+        <v/>
+      </c>
+      <c r="K698" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B699" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C699" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D699" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E699" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F699" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G699" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H699" t="str">
+        <v>N</v>
+      </c>
+      <c r="I699" t="str">
+        <v/>
+      </c>
+      <c r="J699" t="str">
+        <v/>
+      </c>
+      <c r="K699" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B700" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C700" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D700" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E700" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F700" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G700" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H700" t="str">
+        <v>N</v>
+      </c>
+      <c r="I700" t="str">
+        <v/>
+      </c>
+      <c r="J700" t="str">
+        <v/>
+      </c>
+      <c r="K700" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="B701" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C701" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D701" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="E701" t="str">
+        <v>TS KB</v>
+      </c>
+      <c r="F701" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G701" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H701" t="str">
+        <v>N</v>
+      </c>
+      <c r="I701" t="str">
+        <v/>
+      </c>
+      <c r="J701" t="str">
+        <v/>
+      </c>
+      <c r="K701" t="str">
+        <v>S-mubha716-wky0z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K687"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K701"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-22T15:45:57.855Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K701"/>
+  <dimension ref="A1:K715"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -24934,9 +24934,499 @@
         <v>S-mubha716-wky0z</v>
       </c>
     </row>
+    <row r="702">
+      <c r="A702" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B702" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C702" t="str">
+        <v>01:45</v>
+      </c>
+      <c r="D702" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E702" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F702" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G702" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H702" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I702" t="str">
+        <v/>
+      </c>
+      <c r="J702" t="str">
+        <v/>
+      </c>
+      <c r="K702" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B703" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C703" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D703" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E703" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F703" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G703" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H703" t="str">
+        <v>N</v>
+      </c>
+      <c r="I703" t="str">
+        <v/>
+      </c>
+      <c r="J703" t="str">
+        <v/>
+      </c>
+      <c r="K703" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B704" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C704" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D704" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E704" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F704" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G704" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H704" t="str">
+        <v>N</v>
+      </c>
+      <c r="I704" t="str">
+        <v/>
+      </c>
+      <c r="J704" t="str">
+        <v/>
+      </c>
+      <c r="K704" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B705" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C705" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D705" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E705" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F705" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G705" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H705" t="str">
+        <v>N</v>
+      </c>
+      <c r="I705" t="str">
+        <v/>
+      </c>
+      <c r="J705" t="str">
+        <v/>
+      </c>
+      <c r="K705" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B706" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C706" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D706" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E706" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F706" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G706" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H706" t="str">
+        <v>N</v>
+      </c>
+      <c r="I706" t="str">
+        <v/>
+      </c>
+      <c r="J706" t="str">
+        <v/>
+      </c>
+      <c r="K706" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B707" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C707" t="str">
+        <v>01:45</v>
+      </c>
+      <c r="D707" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E707" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F707" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G707" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H707" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I707" t="str">
+        <v/>
+      </c>
+      <c r="J707" t="str">
+        <v/>
+      </c>
+      <c r="K707" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B708" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C708" t="str">
+        <v>21:45</v>
+      </c>
+      <c r="D708" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E708" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F708" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G708" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H708" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I708" t="str">
+        <v/>
+      </c>
+      <c r="J708" t="str">
+        <v/>
+      </c>
+      <c r="K708" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B709" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C709" t="str">
+        <v>03:45</v>
+      </c>
+      <c r="D709" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E709" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F709" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G709" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H709" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I709" t="str">
+        <v/>
+      </c>
+      <c r="J709" t="str">
+        <v/>
+      </c>
+      <c r="K709" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B710" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C710" t="str">
+        <v>02:45</v>
+      </c>
+      <c r="D710" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E710" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F710" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G710" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H710" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I710" t="str">
+        <v/>
+      </c>
+      <c r="J710" t="str">
+        <v/>
+      </c>
+      <c r="K710" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B711" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C711" t="str">
+        <v>05:45</v>
+      </c>
+      <c r="D711" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E711" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F711" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G711" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H711" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I711" t="str">
+        <v/>
+      </c>
+      <c r="J711" t="str">
+        <v/>
+      </c>
+      <c r="K711" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B712" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C712" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D712" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E712" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F712" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G712" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H712" t="str">
+        <v>N</v>
+      </c>
+      <c r="I712" t="str">
+        <v/>
+      </c>
+      <c r="J712" t="str">
+        <v/>
+      </c>
+      <c r="K712" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B713" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C713" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D713" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E713" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F713" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G713" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H713" t="str">
+        <v>N</v>
+      </c>
+      <c r="I713" t="str">
+        <v/>
+      </c>
+      <c r="J713" t="str">
+        <v/>
+      </c>
+      <c r="K713" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B714" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C714" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D714" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E714" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F714" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G714" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H714" t="str">
+        <v>N</v>
+      </c>
+      <c r="I714" t="str">
+        <v/>
+      </c>
+      <c r="J714" t="str">
+        <v/>
+      </c>
+      <c r="K714" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B715" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C715" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D715" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="E715" t="str">
+        <v>TP BA 22/09/2026</v>
+      </c>
+      <c r="F715" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G715" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H715" t="str">
+        <v>N</v>
+      </c>
+      <c r="I715" t="str">
+        <v/>
+      </c>
+      <c r="J715" t="str">
+        <v/>
+      </c>
+      <c r="K715" t="str">
+        <v>S-mucug7bp-tymah</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K701"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K715"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-23T08:09:34.649Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K715"/>
+  <dimension ref="A1:K729"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -25424,9 +25424,499 @@
         <v>S-mucug7bp-tymah</v>
       </c>
     </row>
+    <row r="716">
+      <c r="A716" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B716" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C716" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D716" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E716" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F716" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G716" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H716" t="str">
+        <v>N</v>
+      </c>
+      <c r="I716" t="str">
+        <v/>
+      </c>
+      <c r="J716" t="str">
+        <v/>
+      </c>
+      <c r="K716" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B717" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C717" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D717" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E717" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F717" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G717" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H717" t="str">
+        <v>N</v>
+      </c>
+      <c r="I717" t="str">
+        <v/>
+      </c>
+      <c r="J717" t="str">
+        <v/>
+      </c>
+      <c r="K717" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B718" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C718" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D718" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E718" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F718" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G718" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H718" t="str">
+        <v>N</v>
+      </c>
+      <c r="I718" t="str">
+        <v/>
+      </c>
+      <c r="J718" t="str">
+        <v/>
+      </c>
+      <c r="K718" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B719" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C719" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D719" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E719" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F719" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G719" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H719" t="str">
+        <v>N</v>
+      </c>
+      <c r="I719" t="str">
+        <v/>
+      </c>
+      <c r="J719" t="str">
+        <v/>
+      </c>
+      <c r="K719" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B720" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C720" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D720" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E720" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F720" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G720" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H720" t="str">
+        <v>N</v>
+      </c>
+      <c r="I720" t="str">
+        <v/>
+      </c>
+      <c r="J720" t="str">
+        <v/>
+      </c>
+      <c r="K720" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B721" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C721" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D721" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E721" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F721" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G721" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H721" t="str">
+        <v>N</v>
+      </c>
+      <c r="I721" t="str">
+        <v/>
+      </c>
+      <c r="J721" t="str">
+        <v/>
+      </c>
+      <c r="K721" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B722" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C722" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D722" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E722" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F722" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G722" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H722" t="str">
+        <v>N</v>
+      </c>
+      <c r="I722" t="str">
+        <v/>
+      </c>
+      <c r="J722" t="str">
+        <v/>
+      </c>
+      <c r="K722" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B723" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C723" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D723" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E723" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F723" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G723" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H723" t="str">
+        <v>N</v>
+      </c>
+      <c r="I723" t="str">
+        <v/>
+      </c>
+      <c r="J723" t="str">
+        <v/>
+      </c>
+      <c r="K723" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B724" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C724" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D724" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E724" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F724" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G724" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H724" t="str">
+        <v>N</v>
+      </c>
+      <c r="I724" t="str">
+        <v/>
+      </c>
+      <c r="J724" t="str">
+        <v/>
+      </c>
+      <c r="K724" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B725" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C725" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D725" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E725" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F725" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G725" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H725" t="str">
+        <v>N</v>
+      </c>
+      <c r="I725" t="str">
+        <v/>
+      </c>
+      <c r="J725" t="str">
+        <v/>
+      </c>
+      <c r="K725" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B726" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C726" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D726" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E726" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F726" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G726" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H726" t="str">
+        <v>N</v>
+      </c>
+      <c r="I726" t="str">
+        <v/>
+      </c>
+      <c r="J726" t="str">
+        <v/>
+      </c>
+      <c r="K726" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B727" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C727" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D727" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E727" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F727" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G727" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H727" t="str">
+        <v>N</v>
+      </c>
+      <c r="I727" t="str">
+        <v/>
+      </c>
+      <c r="J727" t="str">
+        <v/>
+      </c>
+      <c r="K727" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B728" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C728" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D728" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E728" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F728" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G728" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H728" t="str">
+        <v>N</v>
+      </c>
+      <c r="I728" t="str">
+        <v/>
+      </c>
+      <c r="J728" t="str">
+        <v/>
+      </c>
+      <c r="K728" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B729" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C729" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D729" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="E729" t="str">
+        <v>TR TS KB</v>
+      </c>
+      <c r="F729" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G729" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H729" t="str">
+        <v>N</v>
+      </c>
+      <c r="I729" t="str">
+        <v/>
+      </c>
+      <c r="J729" t="str">
+        <v/>
+      </c>
+      <c r="K729" t="str">
+        <v>S-mucuf8db-yfkv8</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K715"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K729"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-23T08:13:37.689Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K729"/>
+  <dimension ref="A1:K743"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -25914,9 +25914,499 @@
         <v>S-mucuf8db-yfkv8</v>
       </c>
     </row>
+    <row r="730">
+      <c r="A730" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B730" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C730" t="str">
+        <v>18:15</v>
+      </c>
+      <c r="D730" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E730" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F730" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G730" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H730" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I730" t="str">
+        <v/>
+      </c>
+      <c r="J730" t="str">
+        <v/>
+      </c>
+      <c r="K730" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B731" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C731" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D731" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E731" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F731" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G731" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H731" t="str">
+        <v>N</v>
+      </c>
+      <c r="I731" t="str">
+        <v/>
+      </c>
+      <c r="J731" t="str">
+        <v/>
+      </c>
+      <c r="K731" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B732" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C732" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D732" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E732" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F732" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G732" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H732" t="str">
+        <v>N</v>
+      </c>
+      <c r="I732" t="str">
+        <v/>
+      </c>
+      <c r="J732" t="str">
+        <v/>
+      </c>
+      <c r="K732" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B733" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C733" t="str">
+        <v>18:15</v>
+      </c>
+      <c r="D733" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E733" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F733" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G733" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H733" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I733" t="str">
+        <v/>
+      </c>
+      <c r="J733" t="str">
+        <v/>
+      </c>
+      <c r="K733" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B734" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C734" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D734" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E734" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F734" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G734" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H734" t="str">
+        <v>N</v>
+      </c>
+      <c r="I734" t="str">
+        <v/>
+      </c>
+      <c r="J734" t="str">
+        <v/>
+      </c>
+      <c r="K734" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B735" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C735" t="str">
+        <v>18:30</v>
+      </c>
+      <c r="D735" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E735" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F735" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G735" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H735" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I735" t="str">
+        <v/>
+      </c>
+      <c r="J735" t="str">
+        <v/>
+      </c>
+      <c r="K735" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B736" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C736" t="str">
+        <v>18:00</v>
+      </c>
+      <c r="D736" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E736" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F736" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G736" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H736" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I736" t="str">
+        <v/>
+      </c>
+      <c r="J736" t="str">
+        <v/>
+      </c>
+      <c r="K736" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B737" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C737" t="str">
+        <v>03:00</v>
+      </c>
+      <c r="D737" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E737" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F737" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G737" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H737" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I737" t="str">
+        <v/>
+      </c>
+      <c r="J737" t="str">
+        <v/>
+      </c>
+      <c r="K737" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B738" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C738" t="str">
+        <v>05:30</v>
+      </c>
+      <c r="D738" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E738" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F738" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G738" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H738" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I738" t="str">
+        <v/>
+      </c>
+      <c r="J738" t="str">
+        <v/>
+      </c>
+      <c r="K738" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B739" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C739" t="str">
+        <v>05:15</v>
+      </c>
+      <c r="D739" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E739" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F739" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G739" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H739" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I739" t="str">
+        <v/>
+      </c>
+      <c r="J739" t="str">
+        <v/>
+      </c>
+      <c r="K739" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B740" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C740" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D740" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E740" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F740" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G740" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H740" t="str">
+        <v>N</v>
+      </c>
+      <c r="I740" t="str">
+        <v/>
+      </c>
+      <c r="J740" t="str">
+        <v/>
+      </c>
+      <c r="K740" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B741" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C741" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D741" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E741" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F741" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G741" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H741" t="str">
+        <v>N</v>
+      </c>
+      <c r="I741" t="str">
+        <v/>
+      </c>
+      <c r="J741" t="str">
+        <v/>
+      </c>
+      <c r="K741" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B742" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C742" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D742" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E742" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F742" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G742" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H742" t="str">
+        <v>N</v>
+      </c>
+      <c r="I742" t="str">
+        <v/>
+      </c>
+      <c r="J742" t="str">
+        <v/>
+      </c>
+      <c r="K742" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="B743" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C743" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D743" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="E743" t="str">
+        <v>BA/AS</v>
+      </c>
+      <c r="F743" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G743" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H743" t="str">
+        <v>N</v>
+      </c>
+      <c r="I743" t="str">
+        <v/>
+      </c>
+      <c r="J743" t="str">
+        <v/>
+      </c>
+      <c r="K743" t="str">
+        <v>S-mucujeby-a4wqj</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K729"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K743"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-24T07:36:30.760Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K743"/>
+  <dimension ref="A1:K757"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -26404,9 +26404,499 @@
         <v>S-mucujeby-a4wqj</v>
       </c>
     </row>
+    <row r="744">
+      <c r="A744" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B744" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C744" t="str">
+        <v>07:01</v>
+      </c>
+      <c r="D744" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E744" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F744" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G744" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H744" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I744" t="str">
+        <v/>
+      </c>
+      <c r="J744" t="str">
+        <v/>
+      </c>
+      <c r="K744" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B745" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C745" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D745" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E745" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="F745" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G745" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H745" t="str">
+        <v>N</v>
+      </c>
+      <c r="I745" t="str">
+        <v/>
+      </c>
+      <c r="J745" t="str">
+        <v/>
+      </c>
+      <c r="K745" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B746" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C746" t="str">
+        <v>14:58</v>
+      </c>
+      <c r="D746" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E746" t="str">
+        <v>kyle</v>
+      </c>
+      <c r="F746" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G746" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H746" t="str">
+        <v>N</v>
+      </c>
+      <c r="I746" t="str">
+        <v/>
+      </c>
+      <c r="J746" t="str">
+        <v/>
+      </c>
+      <c r="K746" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B747" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C747" t="str">
+        <v>07:01</v>
+      </c>
+      <c r="D747" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E747" t="str">
+        <v>rob</v>
+      </c>
+      <c r="F747" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G747" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H747" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I747" t="str">
+        <v/>
+      </c>
+      <c r="J747" t="str">
+        <v/>
+      </c>
+      <c r="K747" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B748" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C748" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D748" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E748" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="F748" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G748" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H748" t="str">
+        <v>N</v>
+      </c>
+      <c r="I748" t="str">
+        <v/>
+      </c>
+      <c r="J748" t="str">
+        <v/>
+      </c>
+      <c r="K748" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B749" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C749" t="str">
+        <v>07:01</v>
+      </c>
+      <c r="D749" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E749" t="str">
+        <v>kyle</v>
+      </c>
+      <c r="F749" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G749" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H749" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I749" t="str">
+        <v/>
+      </c>
+      <c r="J749" t="str">
+        <v/>
+      </c>
+      <c r="K749" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B750" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C750" t="str">
+        <v>21:15</v>
+      </c>
+      <c r="D750" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E750" t="str">
+        <v>kyle</v>
+      </c>
+      <c r="F750" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G750" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H750" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I750" t="str">
+        <v/>
+      </c>
+      <c r="J750" t="str">
+        <v/>
+      </c>
+      <c r="K750" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B751" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C751" t="str">
+        <v>15:21</v>
+      </c>
+      <c r="D751" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E751" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F751" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G751" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H751" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I751" t="str">
+        <v/>
+      </c>
+      <c r="J751" t="str">
+        <v/>
+      </c>
+      <c r="K751" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B752" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C752" t="str">
+        <v>17:22</v>
+      </c>
+      <c r="D752" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E752" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F752" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G752" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H752" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I752" t="str">
+        <v/>
+      </c>
+      <c r="J752" t="str">
+        <v/>
+      </c>
+      <c r="K752" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B753" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C753" t="str">
+        <v>17:31</v>
+      </c>
+      <c r="D753" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E753" t="str">
+        <v>ant klye</v>
+      </c>
+      <c r="F753" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G753" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H753" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I753" t="str">
+        <v/>
+      </c>
+      <c r="J753" t="str">
+        <v/>
+      </c>
+      <c r="K753" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B754" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C754" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D754" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E754" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="F754" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G754" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H754" t="str">
+        <v>N</v>
+      </c>
+      <c r="I754" t="str">
+        <v/>
+      </c>
+      <c r="J754" t="str">
+        <v/>
+      </c>
+      <c r="K754" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B755" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C755" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D755" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E755" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="F755" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G755" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H755" t="str">
+        <v>N</v>
+      </c>
+      <c r="I755" t="str">
+        <v/>
+      </c>
+      <c r="J755" t="str">
+        <v/>
+      </c>
+      <c r="K755" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B756" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C756" t="str">
+        <v>07:04</v>
+      </c>
+      <c r="D756" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E756" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="F756" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G756" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H756" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I756" t="str">
+        <v/>
+      </c>
+      <c r="J756" t="str">
+        <v/>
+      </c>
+      <c r="K756" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B757" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C757" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D757" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="E757" t="str">
+        <v>kyle anthony rob</v>
+      </c>
+      <c r="F757" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G757" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H757" t="str">
+        <v>N</v>
+      </c>
+      <c r="I757" t="str">
+        <v/>
+      </c>
+      <c r="J757" t="str">
+        <v/>
+      </c>
+      <c r="K757" t="str">
+        <v>S-muel7jz0-thwa1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K743"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K757"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-26T00:38:57.185Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K757"/>
+  <dimension ref="A1:K771"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -26894,9 +26894,499 @@
         <v>S-muel7jz0-thwa1</v>
       </c>
     </row>
+    <row r="758">
+      <c r="A758" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B758" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C758" t="str">
+        <v>07:13</v>
+      </c>
+      <c r="D758" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E758" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F758" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G758" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H758" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I758" t="str">
+        <v/>
+      </c>
+      <c r="J758" t="str">
+        <v/>
+      </c>
+      <c r="K758" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B759" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C759" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D759" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E759" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F759" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G759" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H759" t="str">
+        <v>N</v>
+      </c>
+      <c r="I759" t="str">
+        <v/>
+      </c>
+      <c r="J759" t="str">
+        <v/>
+      </c>
+      <c r="K759" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B760" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C760" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D760" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E760" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F760" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G760" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H760" t="str">
+        <v>N</v>
+      </c>
+      <c r="I760" t="str">
+        <v/>
+      </c>
+      <c r="J760" t="str">
+        <v/>
+      </c>
+      <c r="K760" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B761" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C761" t="str">
+        <v>07:13</v>
+      </c>
+      <c r="D761" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E761" t="str">
+        <v>kyle</v>
+      </c>
+      <c r="F761" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G761" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H761" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I761" t="str">
+        <v/>
+      </c>
+      <c r="J761" t="str">
+        <v/>
+      </c>
+      <c r="K761" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B762" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C762" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D762" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E762" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F762" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G762" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H762" t="str">
+        <v>N</v>
+      </c>
+      <c r="I762" t="str">
+        <v/>
+      </c>
+      <c r="J762" t="str">
+        <v/>
+      </c>
+      <c r="K762" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B763" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C763" t="str">
+        <v>07:15</v>
+      </c>
+      <c r="D763" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E763" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F763" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G763" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H763" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I763" t="str">
+        <v/>
+      </c>
+      <c r="J763" t="str">
+        <v/>
+      </c>
+      <c r="K763" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B764" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C764" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D764" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E764" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F764" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G764" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H764" t="str">
+        <v>N</v>
+      </c>
+      <c r="I764" t="str">
+        <v/>
+      </c>
+      <c r="J764" t="str">
+        <v/>
+      </c>
+      <c r="K764" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B765" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C765" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D765" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E765" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F765" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G765" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H765" t="str">
+        <v>N</v>
+      </c>
+      <c r="I765" t="str">
+        <v/>
+      </c>
+      <c r="J765" t="str">
+        <v/>
+      </c>
+      <c r="K765" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B766" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C766" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D766" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E766" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F766" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G766" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H766" t="str">
+        <v>N</v>
+      </c>
+      <c r="I766" t="str">
+        <v/>
+      </c>
+      <c r="J766" t="str">
+        <v/>
+      </c>
+      <c r="K766" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B767" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C767" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D767" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E767" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F767" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G767" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H767" t="str">
+        <v>N</v>
+      </c>
+      <c r="I767" t="str">
+        <v/>
+      </c>
+      <c r="J767" t="str">
+        <v/>
+      </c>
+      <c r="K767" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B768" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C768" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D768" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E768" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F768" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G768" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H768" t="str">
+        <v>N</v>
+      </c>
+      <c r="I768" t="str">
+        <v/>
+      </c>
+      <c r="J768" t="str">
+        <v/>
+      </c>
+      <c r="K768" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B769" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C769" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D769" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E769" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F769" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G769" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H769" t="str">
+        <v>N</v>
+      </c>
+      <c r="I769" t="str">
+        <v/>
+      </c>
+      <c r="J769" t="str">
+        <v/>
+      </c>
+      <c r="K769" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B770" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C770" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D770" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E770" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F770" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G770" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H770" t="str">
+        <v>N</v>
+      </c>
+      <c r="I770" t="str">
+        <v/>
+      </c>
+      <c r="J770" t="str">
+        <v/>
+      </c>
+      <c r="K770" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B771" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C771" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D771" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="E771" t="str">
+        <v>Anthony Kyle</v>
+      </c>
+      <c r="F771" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G771" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H771" t="str">
+        <v>N</v>
+      </c>
+      <c r="I771" t="str">
+        <v/>
+      </c>
+      <c r="J771" t="str">
+        <v/>
+      </c>
+      <c r="K771" t="str">
+        <v>S-muhgjdae-opx9j</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K757"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K771"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-26T08:05:33.789Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -27112,13 +27112,13 @@
         <v>Day</v>
       </c>
       <c r="C764" t="str">
-        <v>(not entered)</v>
+        <v>09:30</v>
       </c>
       <c r="D764" t="str">
         <v>Anthony Kyle</v>
       </c>
       <c r="E764" t="str">
-        <v>Anthony Kyle</v>
+        <v>KB</v>
       </c>
       <c r="F764" t="str">
         <v>During Processing</v>
@@ -27127,7 +27127,7 @@
         <v>Purge mills — 200 pumps each</v>
       </c>
       <c r="H764" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I764" t="str">
         <v/>
@@ -27147,13 +27147,13 @@
         <v>Day</v>
       </c>
       <c r="C765" t="str">
-        <v>(not entered)</v>
+        <v>15:10</v>
       </c>
       <c r="D765" t="str">
         <v>Anthony Kyle</v>
       </c>
       <c r="E765" t="str">
-        <v>Anthony Kyle</v>
+        <v>KB</v>
       </c>
       <c r="F765" t="str">
         <v>During Processing</v>
@@ -27162,7 +27162,7 @@
         <v>Purge mills — 200 pumps each</v>
       </c>
       <c r="H765" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I765" t="str">
         <v/>
@@ -27182,13 +27182,13 @@
         <v>Day</v>
       </c>
       <c r="C766" t="str">
-        <v>(not entered)</v>
+        <v>17:23</v>
       </c>
       <c r="D766" t="str">
         <v>Anthony Kyle</v>
       </c>
       <c r="E766" t="str">
-        <v>Anthony Kyle</v>
+        <v>Anthony</v>
       </c>
       <c r="F766" t="str">
         <v>During Processing</v>
@@ -27197,7 +27197,7 @@
         <v>Inspect &amp; clean steam vent</v>
       </c>
       <c r="H766" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I766" t="str">
         <v/>
@@ -27217,13 +27217,13 @@
         <v>Day</v>
       </c>
       <c r="C767" t="str">
-        <v>(not entered)</v>
+        <v>17:49</v>
       </c>
       <c r="D767" t="str">
         <v>Anthony Kyle</v>
       </c>
       <c r="E767" t="str">
-        <v>Anthony Kyle</v>
+        <v>KB</v>
       </c>
       <c r="F767" t="str">
         <v>During Processing</v>
@@ -27232,7 +27232,7 @@
         <v>Empty drop box at end of shift</v>
       </c>
       <c r="H767" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I767" t="str">
         <v/>

</xml_diff>

<commit_message>
Checklist log update 2026-09-26T08:18:45.811Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K771"/>
+  <dimension ref="A1:K785"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -27384,9 +27384,499 @@
         <v>S-muhgjdae-opx9j</v>
       </c>
     </row>
+    <row r="772">
+      <c r="A772" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B772" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C772" t="str">
+        <v>18:00</v>
+      </c>
+      <c r="D772" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E772" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F772" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G772" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H772" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I772" t="str">
+        <v/>
+      </c>
+      <c r="J772" t="str">
+        <v/>
+      </c>
+      <c r="K772" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B773" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C773" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D773" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E773" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F773" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G773" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H773" t="str">
+        <v>N</v>
+      </c>
+      <c r="I773" t="str">
+        <v/>
+      </c>
+      <c r="J773" t="str">
+        <v/>
+      </c>
+      <c r="K773" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B774" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C774" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D774" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E774" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F774" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G774" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H774" t="str">
+        <v>N</v>
+      </c>
+      <c r="I774" t="str">
+        <v/>
+      </c>
+      <c r="J774" t="str">
+        <v/>
+      </c>
+      <c r="K774" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B775" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C775" t="str">
+        <v>18:00</v>
+      </c>
+      <c r="D775" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E775" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F775" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G775" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H775" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I775" t="str">
+        <v/>
+      </c>
+      <c r="J775" t="str">
+        <v/>
+      </c>
+      <c r="K775" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B776" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C776" t="str">
+        <v>18:10</v>
+      </c>
+      <c r="D776" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E776" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F776" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G776" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H776" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I776" t="str">
+        <v/>
+      </c>
+      <c r="J776" t="str">
+        <v/>
+      </c>
+      <c r="K776" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B777" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C777" t="str">
+        <v>18:16</v>
+      </c>
+      <c r="D777" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E777" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F777" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G777" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H777" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I777" t="str">
+        <v/>
+      </c>
+      <c r="J777" t="str">
+        <v/>
+      </c>
+      <c r="K777" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B778" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C778" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="D778" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E778" t="str">
+        <v>Ken/BA</v>
+      </c>
+      <c r="F778" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G778" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H778" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I778" t="str">
+        <v/>
+      </c>
+      <c r="J778" t="str">
+        <v/>
+      </c>
+      <c r="K778" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B779" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C779" t="str">
+        <v>03:00</v>
+      </c>
+      <c r="D779" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E779" t="str">
+        <v>Ken/BA</v>
+      </c>
+      <c r="F779" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G779" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H779" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I779" t="str">
+        <v/>
+      </c>
+      <c r="J779" t="str">
+        <v/>
+      </c>
+      <c r="K779" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B780" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C780" t="str">
+        <v>05:30</v>
+      </c>
+      <c r="D780" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E780" t="str">
+        <v>Ken/BA</v>
+      </c>
+      <c r="F780" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G780" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H780" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I780" t="str">
+        <v/>
+      </c>
+      <c r="J780" t="str">
+        <v/>
+      </c>
+      <c r="K780" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B781" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C781" t="str">
+        <v>05:30</v>
+      </c>
+      <c r="D781" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E781" t="str">
+        <v>Ken/BA</v>
+      </c>
+      <c r="F781" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G781" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H781" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I781" t="str">
+        <v/>
+      </c>
+      <c r="J781" t="str">
+        <v/>
+      </c>
+      <c r="K781" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B782" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C782" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D782" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E782" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F782" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G782" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H782" t="str">
+        <v>N</v>
+      </c>
+      <c r="I782" t="str">
+        <v/>
+      </c>
+      <c r="J782" t="str">
+        <v/>
+      </c>
+      <c r="K782" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B783" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C783" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D783" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E783" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F783" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G783" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H783" t="str">
+        <v>N</v>
+      </c>
+      <c r="I783" t="str">
+        <v/>
+      </c>
+      <c r="J783" t="str">
+        <v/>
+      </c>
+      <c r="K783" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B784" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C784" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D784" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E784" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F784" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G784" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H784" t="str">
+        <v>N</v>
+      </c>
+      <c r="I784" t="str">
+        <v/>
+      </c>
+      <c r="J784" t="str">
+        <v/>
+      </c>
+      <c r="K784" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B785" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C785" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D785" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E785" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F785" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G785" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H785" t="str">
+        <v>N</v>
+      </c>
+      <c r="I785" t="str">
+        <v/>
+      </c>
+      <c r="J785" t="str">
+        <v/>
+      </c>
+      <c r="K785" t="str">
+        <v>S-muhgj7ed-k6bli</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K771"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K785"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-26T16:41:51.267Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -27386,7 +27386,7 @@
     </row>
     <row r="772">
       <c r="A772" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B772" t="str">
         <v>Night</v>
@@ -27421,7 +27421,7 @@
     </row>
     <row r="773">
       <c r="A773" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B773" t="str">
         <v>Night</v>
@@ -27456,7 +27456,7 @@
     </row>
     <row r="774">
       <c r="A774" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B774" t="str">
         <v>Night</v>
@@ -27491,7 +27491,7 @@
     </row>
     <row r="775">
       <c r="A775" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B775" t="str">
         <v>Night</v>
@@ -27526,7 +27526,7 @@
     </row>
     <row r="776">
       <c r="A776" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B776" t="str">
         <v>Night</v>
@@ -27561,7 +27561,7 @@
     </row>
     <row r="777">
       <c r="A777" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B777" t="str">
         <v>Night</v>
@@ -27596,7 +27596,7 @@
     </row>
     <row r="778">
       <c r="A778" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B778" t="str">
         <v>Night</v>
@@ -27631,7 +27631,7 @@
     </row>
     <row r="779">
       <c r="A779" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B779" t="str">
         <v>Night</v>
@@ -27666,7 +27666,7 @@
     </row>
     <row r="780">
       <c r="A780" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B780" t="str">
         <v>Night</v>
@@ -27701,7 +27701,7 @@
     </row>
     <row r="781">
       <c r="A781" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B781" t="str">
         <v>Night</v>
@@ -27736,7 +27736,7 @@
     </row>
     <row r="782">
       <c r="A782" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B782" t="str">
         <v>Night</v>
@@ -27771,7 +27771,7 @@
     </row>
     <row r="783">
       <c r="A783" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B783" t="str">
         <v>Night</v>
@@ -27806,7 +27806,7 @@
     </row>
     <row r="784">
       <c r="A784" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B784" t="str">
         <v>Night</v>
@@ -27841,7 +27841,7 @@
     </row>
     <row r="785">
       <c r="A785" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B785" t="str">
         <v>Night</v>

</xml_diff>

<commit_message>
Checklist log update 2026-09-27T07:23:53.686Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K785"/>
+  <dimension ref="A1:K799"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -27874,9 +27874,499 @@
         <v>S-muhgj7ed-k6bli</v>
       </c>
     </row>
+    <row r="786">
+      <c r="A786" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B786" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C786" t="str">
+        <v>06:15</v>
+      </c>
+      <c r="D786" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E786" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F786" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G786" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H786" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I786" t="str">
+        <v/>
+      </c>
+      <c r="J786" t="str">
+        <v/>
+      </c>
+      <c r="K786" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B787" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C787" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D787" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E787" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F787" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G787" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H787" t="str">
+        <v>N</v>
+      </c>
+      <c r="I787" t="str">
+        <v/>
+      </c>
+      <c r="J787" t="str">
+        <v/>
+      </c>
+      <c r="K787" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B788" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C788" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D788" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E788" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F788" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G788" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H788" t="str">
+        <v>N</v>
+      </c>
+      <c r="I788" t="str">
+        <v/>
+      </c>
+      <c r="J788" t="str">
+        <v/>
+      </c>
+      <c r="K788" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B789" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C789" t="str">
+        <v>07:15</v>
+      </c>
+      <c r="D789" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E789" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F789" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G789" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H789" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I789" t="str">
+        <v/>
+      </c>
+      <c r="J789" t="str">
+        <v/>
+      </c>
+      <c r="K789" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B790" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C790" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D790" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E790" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F790" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G790" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H790" t="str">
+        <v>N</v>
+      </c>
+      <c r="I790" t="str">
+        <v/>
+      </c>
+      <c r="J790" t="str">
+        <v/>
+      </c>
+      <c r="K790" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B791" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C791" t="str">
+        <v>10:30</v>
+      </c>
+      <c r="D791" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E791" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F791" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G791" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H791" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I791" t="str">
+        <v/>
+      </c>
+      <c r="J791" t="str">
+        <v/>
+      </c>
+      <c r="K791" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B792" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C792" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D792" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E792" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F792" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G792" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H792" t="str">
+        <v>N</v>
+      </c>
+      <c r="I792" t="str">
+        <v/>
+      </c>
+      <c r="J792" t="str">
+        <v/>
+      </c>
+      <c r="K792" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B793" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C793" t="str">
+        <v>15:43</v>
+      </c>
+      <c r="D793" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E793" t="str">
+        <v>KB</v>
+      </c>
+      <c r="F793" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G793" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H793" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I793" t="str">
+        <v>mill 1 purged as well</v>
+      </c>
+      <c r="J793" t="str">
+        <v/>
+      </c>
+      <c r="K793" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B794" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C794" t="str">
+        <v>17:21</v>
+      </c>
+      <c r="D794" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E794" t="str">
+        <v>AH</v>
+      </c>
+      <c r="F794" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G794" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H794" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I794" t="str">
+        <v/>
+      </c>
+      <c r="J794" t="str">
+        <v/>
+      </c>
+      <c r="K794" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B795" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C795" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D795" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E795" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F795" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G795" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H795" t="str">
+        <v>N</v>
+      </c>
+      <c r="I795" t="str">
+        <v/>
+      </c>
+      <c r="J795" t="str">
+        <v/>
+      </c>
+      <c r="K795" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B796" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C796" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="D796" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E796" t="str">
+        <v>AH</v>
+      </c>
+      <c r="F796" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G796" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H796" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I796" t="str">
+        <v/>
+      </c>
+      <c r="J796" t="str">
+        <v/>
+      </c>
+      <c r="K796" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B797" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C797" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D797" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E797" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F797" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G797" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H797" t="str">
+        <v>N</v>
+      </c>
+      <c r="I797" t="str">
+        <v/>
+      </c>
+      <c r="J797" t="str">
+        <v/>
+      </c>
+      <c r="K797" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B798" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C798" t="str">
+        <v>15:20</v>
+      </c>
+      <c r="D798" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E798" t="str">
+        <v>KB</v>
+      </c>
+      <c r="F798" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G798" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H798" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I798" t="str">
+        <v>Close to needing reordering</v>
+      </c>
+      <c r="J798" t="str">
+        <v/>
+      </c>
+      <c r="K798" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B799" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C799" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D799" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="E799" t="str">
+        <v>anthony kyle</v>
+      </c>
+      <c r="F799" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G799" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H799" t="str">
+        <v>N</v>
+      </c>
+      <c r="I799" t="str">
+        <v/>
+      </c>
+      <c r="J799" t="str">
+        <v/>
+      </c>
+      <c r="K799" t="str">
+        <v>S-muj2zvx1-to9hx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K785"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K799"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-27T11:29:18.191Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K799"/>
+  <dimension ref="A1:K813"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -28364,9 +28364,499 @@
         <v>S-muj2zvx1-to9hx</v>
       </c>
     </row>
+    <row r="800">
+      <c r="A800" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B800" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C800" t="str">
+        <v>18:30</v>
+      </c>
+      <c r="D800" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E800" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F800" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G800" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H800" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I800" t="str">
+        <v/>
+      </c>
+      <c r="J800" t="str">
+        <v/>
+      </c>
+      <c r="K800" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B801" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C801" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D801" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E801" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F801" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G801" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H801" t="str">
+        <v>N</v>
+      </c>
+      <c r="I801" t="str">
+        <v/>
+      </c>
+      <c r="J801" t="str">
+        <v/>
+      </c>
+      <c r="K801" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B802" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C802" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D802" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E802" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F802" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G802" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H802" t="str">
+        <v>N</v>
+      </c>
+      <c r="I802" t="str">
+        <v/>
+      </c>
+      <c r="J802" t="str">
+        <v/>
+      </c>
+      <c r="K802" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B803" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C803" t="str">
+        <v>18:30</v>
+      </c>
+      <c r="D803" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E803" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F803" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G803" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H803" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I803" t="str">
+        <v/>
+      </c>
+      <c r="J803" t="str">
+        <v/>
+      </c>
+      <c r="K803" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B804" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C804" t="str">
+        <v>18:30</v>
+      </c>
+      <c r="D804" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E804" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F804" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G804" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H804" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I804" t="str">
+        <v/>
+      </c>
+      <c r="J804" t="str">
+        <v/>
+      </c>
+      <c r="K804" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B805" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C805" t="str">
+        <v>18:30</v>
+      </c>
+      <c r="D805" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E805" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F805" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G805" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H805" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I805" t="str">
+        <v/>
+      </c>
+      <c r="J805" t="str">
+        <v/>
+      </c>
+      <c r="K805" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B806" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C806" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="D806" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E806" t="str">
+        <v>BA</v>
+      </c>
+      <c r="F806" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G806" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H806" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I806" t="str">
+        <v/>
+      </c>
+      <c r="J806" t="str">
+        <v/>
+      </c>
+      <c r="K806" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B807" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C807" t="str">
+        <v>03:00</v>
+      </c>
+      <c r="D807" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E807" t="str">
+        <v>KEN</v>
+      </c>
+      <c r="F807" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G807" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H807" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I807" t="str">
+        <v/>
+      </c>
+      <c r="J807" t="str">
+        <v/>
+      </c>
+      <c r="K807" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B808" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C808" t="str">
+        <v>05:30</v>
+      </c>
+      <c r="D808" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E808" t="str">
+        <v>KEN</v>
+      </c>
+      <c r="F808" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G808" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H808" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I808" t="str">
+        <v/>
+      </c>
+      <c r="J808" t="str">
+        <v/>
+      </c>
+      <c r="K808" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B809" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C809" t="str">
+        <v>05:30</v>
+      </c>
+      <c r="D809" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E809" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F809" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G809" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H809" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I809" t="str">
+        <v/>
+      </c>
+      <c r="J809" t="str">
+        <v/>
+      </c>
+      <c r="K809" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B810" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C810" t="str">
+        <v>05:00</v>
+      </c>
+      <c r="D810" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E810" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F810" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G810" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H810" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I810" t="str">
+        <v/>
+      </c>
+      <c r="J810" t="str">
+        <v/>
+      </c>
+      <c r="K810" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B811" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C811" t="str">
+        <v>18:30</v>
+      </c>
+      <c r="D811" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E811" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F811" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G811" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H811" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I811" t="str">
+        <v/>
+      </c>
+      <c r="J811" t="str">
+        <v/>
+      </c>
+      <c r="K811" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B812" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C812" t="str">
+        <v>21:30</v>
+      </c>
+      <c r="D812" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E812" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F812" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G812" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H812" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I812" t="str">
+        <v/>
+      </c>
+      <c r="J812" t="str">
+        <v/>
+      </c>
+      <c r="K812" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B813" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C813" t="str">
+        <v>05:00</v>
+      </c>
+      <c r="D813" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="E813" t="str">
+        <v>BA/Ken</v>
+      </c>
+      <c r="F813" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G813" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H813" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I813" t="str">
+        <v/>
+      </c>
+      <c r="J813" t="str">
+        <v/>
+      </c>
+      <c r="K813" t="str">
+        <v>S-muj2zu96-hvrt3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K799"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K813"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-28T01:29:47.526Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K813"/>
+  <dimension ref="A1:K827"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -28854,9 +28854,499 @@
         <v>S-muj2zu96-hvrt3</v>
       </c>
     </row>
+    <row r="814">
+      <c r="A814" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B814" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C814" t="str">
+        <v>06:11</v>
+      </c>
+      <c r="D814" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E814" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F814" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G814" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H814" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I814" t="str">
+        <v/>
+      </c>
+      <c r="J814" t="str">
+        <v/>
+      </c>
+      <c r="K814" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B815" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C815" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D815" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E815" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F815" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G815" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H815" t="str">
+        <v>N</v>
+      </c>
+      <c r="I815" t="str">
+        <v/>
+      </c>
+      <c r="J815" t="str">
+        <v/>
+      </c>
+      <c r="K815" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B816" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C816" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D816" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E816" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F816" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G816" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H816" t="str">
+        <v>N</v>
+      </c>
+      <c r="I816" t="str">
+        <v/>
+      </c>
+      <c r="J816" t="str">
+        <v/>
+      </c>
+      <c r="K816" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B817" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C817" t="str">
+        <v>09:00</v>
+      </c>
+      <c r="D817" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E817" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F817" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G817" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H817" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I817" t="str">
+        <v/>
+      </c>
+      <c r="J817" t="str">
+        <v/>
+      </c>
+      <c r="K817" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B818" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C818" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D818" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E818" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F818" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G818" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H818" t="str">
+        <v>N</v>
+      </c>
+      <c r="I818" t="str">
+        <v/>
+      </c>
+      <c r="J818" t="str">
+        <v/>
+      </c>
+      <c r="K818" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B819" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C819" t="str">
+        <v>09:21</v>
+      </c>
+      <c r="D819" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E819" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F819" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G819" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H819" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I819" t="str">
+        <v/>
+      </c>
+      <c r="J819" t="str">
+        <v/>
+      </c>
+      <c r="K819" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B820" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C820" t="str">
+        <v>11:29</v>
+      </c>
+      <c r="D820" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E820" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F820" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G820" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H820" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I820" t="str">
+        <v/>
+      </c>
+      <c r="J820" t="str">
+        <v/>
+      </c>
+      <c r="K820" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B821" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C821" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D821" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E821" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F821" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G821" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H821" t="str">
+        <v>N</v>
+      </c>
+      <c r="I821" t="str">
+        <v/>
+      </c>
+      <c r="J821" t="str">
+        <v/>
+      </c>
+      <c r="K821" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B822" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C822" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D822" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E822" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F822" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G822" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H822" t="str">
+        <v>N</v>
+      </c>
+      <c r="I822" t="str">
+        <v/>
+      </c>
+      <c r="J822" t="str">
+        <v/>
+      </c>
+      <c r="K822" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B823" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C823" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D823" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E823" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F823" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G823" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H823" t="str">
+        <v>N</v>
+      </c>
+      <c r="I823" t="str">
+        <v/>
+      </c>
+      <c r="J823" t="str">
+        <v/>
+      </c>
+      <c r="K823" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B824" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C824" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D824" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E824" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F824" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G824" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H824" t="str">
+        <v>N</v>
+      </c>
+      <c r="I824" t="str">
+        <v/>
+      </c>
+      <c r="J824" t="str">
+        <v/>
+      </c>
+      <c r="K824" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B825" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C825" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D825" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E825" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F825" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G825" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H825" t="str">
+        <v>N</v>
+      </c>
+      <c r="I825" t="str">
+        <v/>
+      </c>
+      <c r="J825" t="str">
+        <v/>
+      </c>
+      <c r="K825" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B826" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C826" t="str">
+        <v>11:29</v>
+      </c>
+      <c r="D826" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E826" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F826" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G826" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H826" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I826" t="str">
+        <v>20%</v>
+      </c>
+      <c r="J826" t="str">
+        <v/>
+      </c>
+      <c r="K826" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B827" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C827" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D827" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="E827" t="str">
+        <v>anthony Dylan Amber Rob</v>
+      </c>
+      <c r="F827" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G827" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H827" t="str">
+        <v>N</v>
+      </c>
+      <c r="I827" t="str">
+        <v/>
+      </c>
+      <c r="J827" t="str">
+        <v/>
+      </c>
+      <c r="K827" t="str">
+        <v>S-mukkitch-1vs62</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K813"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K827"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-29T08:08:50.985Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K827"/>
+  <dimension ref="A1:K841"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -29344,9 +29344,499 @@
         <v>S-mukkitch-1vs62</v>
       </c>
     </row>
+    <row r="828">
+      <c r="A828" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B828" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C828" t="str">
+        <v>22:14</v>
+      </c>
+      <c r="D828" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E828" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F828" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G828" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H828" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I828" t="str">
+        <v/>
+      </c>
+      <c r="J828" t="str">
+        <v/>
+      </c>
+      <c r="K828" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B829" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C829" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D829" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E829" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F829" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G829" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H829" t="str">
+        <v>N</v>
+      </c>
+      <c r="I829" t="str">
+        <v/>
+      </c>
+      <c r="J829" t="str">
+        <v/>
+      </c>
+      <c r="K829" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B830" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C830" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D830" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E830" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F830" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G830" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H830" t="str">
+        <v>N</v>
+      </c>
+      <c r="I830" t="str">
+        <v/>
+      </c>
+      <c r="J830" t="str">
+        <v/>
+      </c>
+      <c r="K830" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B831" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C831" t="str">
+        <v>23:59</v>
+      </c>
+      <c r="D831" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E831" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F831" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G831" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H831" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I831" t="str">
+        <v/>
+      </c>
+      <c r="J831" t="str">
+        <v/>
+      </c>
+      <c r="K831" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B832" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C832" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D832" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E832" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F832" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G832" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H832" t="str">
+        <v>N</v>
+      </c>
+      <c r="I832" t="str">
+        <v/>
+      </c>
+      <c r="J832" t="str">
+        <v/>
+      </c>
+      <c r="K832" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B833" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C833" t="str">
+        <v>22:14</v>
+      </c>
+      <c r="D833" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E833" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F833" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G833" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H833" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I833" t="str">
+        <v/>
+      </c>
+      <c r="J833" t="str">
+        <v/>
+      </c>
+      <c r="K833" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B834" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C834" t="str">
+        <v>22:14</v>
+      </c>
+      <c r="D834" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E834" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F834" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G834" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H834" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I834" t="str">
+        <v/>
+      </c>
+      <c r="J834" t="str">
+        <v/>
+      </c>
+      <c r="K834" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B835" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C835" t="str">
+        <v>03:01</v>
+      </c>
+      <c r="D835" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E835" t="str">
+        <v>TP</v>
+      </c>
+      <c r="F835" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G835" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H835" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I835" t="str">
+        <v/>
+      </c>
+      <c r="J835" t="str">
+        <v/>
+      </c>
+      <c r="K835" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B836" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C836" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D836" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E836" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F836" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G836" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H836" t="str">
+        <v>N</v>
+      </c>
+      <c r="I836" t="str">
+        <v/>
+      </c>
+      <c r="J836" t="str">
+        <v/>
+      </c>
+      <c r="K836" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B837" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C837" t="str">
+        <v>05:30</v>
+      </c>
+      <c r="D837" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E837" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="F837" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G837" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H837" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I837" t="str">
+        <v/>
+      </c>
+      <c r="J837" t="str">
+        <v/>
+      </c>
+      <c r="K837" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B838" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C838" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D838" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E838" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F838" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G838" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H838" t="str">
+        <v>N</v>
+      </c>
+      <c r="I838" t="str">
+        <v/>
+      </c>
+      <c r="J838" t="str">
+        <v/>
+      </c>
+      <c r="K838" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B839" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C839" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D839" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E839" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F839" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G839" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H839" t="str">
+        <v>N</v>
+      </c>
+      <c r="I839" t="str">
+        <v/>
+      </c>
+      <c r="J839" t="str">
+        <v/>
+      </c>
+      <c r="K839" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B840" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C840" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D840" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E840" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F840" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G840" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H840" t="str">
+        <v>N</v>
+      </c>
+      <c r="I840" t="str">
+        <v/>
+      </c>
+      <c r="J840" t="str">
+        <v/>
+      </c>
+      <c r="K840" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B841" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C841" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D841" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="E841" t="str">
+        <v>TP,KB</v>
+      </c>
+      <c r="F841" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G841" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H841" t="str">
+        <v>N</v>
+      </c>
+      <c r="I841" t="str">
+        <v/>
+      </c>
+      <c r="J841" t="str">
+        <v/>
+      </c>
+      <c r="K841" t="str">
+        <v>S-mume7f85-7uwip</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K827"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K841"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-29T19:42:33.999Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K841"/>
+  <dimension ref="A1:K855"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -29834,9 +29834,499 @@
         <v>S-mume7f85-7uwip</v>
       </c>
     </row>
+    <row r="842">
+      <c r="A842" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B842" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C842" t="str">
+        <v>18:09</v>
+      </c>
+      <c r="D842" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E842" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F842" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G842" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H842" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I842" t="str">
+        <v/>
+      </c>
+      <c r="J842" t="str">
+        <v/>
+      </c>
+      <c r="K842" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B843" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C843" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D843" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E843" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="F843" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G843" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H843" t="str">
+        <v>N</v>
+      </c>
+      <c r="I843" t="str">
+        <v/>
+      </c>
+      <c r="J843" t="str">
+        <v/>
+      </c>
+      <c r="K843" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B844" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C844" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D844" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E844" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="F844" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G844" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H844" t="str">
+        <v>N</v>
+      </c>
+      <c r="I844" t="str">
+        <v/>
+      </c>
+      <c r="J844" t="str">
+        <v/>
+      </c>
+      <c r="K844" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B845" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C845" t="str">
+        <v>18:10</v>
+      </c>
+      <c r="D845" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E845" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F845" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G845" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H845" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I845" t="str">
+        <v/>
+      </c>
+      <c r="J845" t="str">
+        <v/>
+      </c>
+      <c r="K845" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B846" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C846" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D846" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E846" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="F846" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G846" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H846" t="str">
+        <v>N</v>
+      </c>
+      <c r="I846" t="str">
+        <v/>
+      </c>
+      <c r="J846" t="str">
+        <v/>
+      </c>
+      <c r="K846" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B847" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C847" t="str">
+        <v>18:11</v>
+      </c>
+      <c r="D847" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E847" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F847" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G847" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H847" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I847" t="str">
+        <v/>
+      </c>
+      <c r="J847" t="str">
+        <v/>
+      </c>
+      <c r="K847" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B848" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C848" t="str">
+        <v>21:45</v>
+      </c>
+      <c r="D848" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E848" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F848" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G848" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H848" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I848" t="str">
+        <v/>
+      </c>
+      <c r="J848" t="str">
+        <v/>
+      </c>
+      <c r="K848" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B849" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C849" t="str">
+        <v>03:00</v>
+      </c>
+      <c r="D849" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E849" t="str">
+        <v>TP</v>
+      </c>
+      <c r="F849" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G849" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H849" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I849" t="str">
+        <v/>
+      </c>
+      <c r="J849" t="str">
+        <v/>
+      </c>
+      <c r="K849" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B850" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C850" t="str">
+        <v>05:20</v>
+      </c>
+      <c r="D850" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E850" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F850" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G850" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H850" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I850" t="str">
+        <v/>
+      </c>
+      <c r="J850" t="str">
+        <v/>
+      </c>
+      <c r="K850" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B851" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C851" t="str">
+        <v>05:42</v>
+      </c>
+      <c r="D851" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E851" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F851" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G851" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H851" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I851" t="str">
+        <v/>
+      </c>
+      <c r="J851" t="str">
+        <v/>
+      </c>
+      <c r="K851" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B852" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C852" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D852" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E852" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="F852" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G852" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H852" t="str">
+        <v>N</v>
+      </c>
+      <c r="I852" t="str">
+        <v/>
+      </c>
+      <c r="J852" t="str">
+        <v/>
+      </c>
+      <c r="K852" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B853" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C853" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D853" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E853" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="F853" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G853" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H853" t="str">
+        <v>N</v>
+      </c>
+      <c r="I853" t="str">
+        <v/>
+      </c>
+      <c r="J853" t="str">
+        <v/>
+      </c>
+      <c r="K853" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B854" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C854" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D854" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E854" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="F854" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G854" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H854" t="str">
+        <v>N</v>
+      </c>
+      <c r="I854" t="str">
+        <v/>
+      </c>
+      <c r="J854" t="str">
+        <v/>
+      </c>
+      <c r="K854" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B855" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C855" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D855" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="E855" t="str">
+        <v>TP, Ken</v>
+      </c>
+      <c r="F855" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G855" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H855" t="str">
+        <v>N</v>
+      </c>
+      <c r="I855" t="str">
+        <v/>
+      </c>
+      <c r="J855" t="str">
+        <v/>
+      </c>
+      <c r="K855" t="str">
+        <v>S-mumeafa2-u0r4a</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K841"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K855"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-30T00:50:56.257Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K855"/>
+  <dimension ref="A1:K869"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -30324,9 +30324,499 @@
         <v>S-mumeafa2-u0r4a</v>
       </c>
     </row>
+    <row r="856">
+      <c r="A856" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B856" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C856" t="str">
+        <v>06:25</v>
+      </c>
+      <c r="D856" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E856" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F856" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G856" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H856" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I856" t="str">
+        <v/>
+      </c>
+      <c r="J856" t="str">
+        <v/>
+      </c>
+      <c r="K856" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B857" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C857" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D857" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E857" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F857" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G857" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H857" t="str">
+        <v>N</v>
+      </c>
+      <c r="I857" t="str">
+        <v/>
+      </c>
+      <c r="J857" t="str">
+        <v/>
+      </c>
+      <c r="K857" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B858" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C858" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D858" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E858" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F858" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G858" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H858" t="str">
+        <v>N</v>
+      </c>
+      <c r="I858" t="str">
+        <v/>
+      </c>
+      <c r="J858" t="str">
+        <v/>
+      </c>
+      <c r="K858" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B859" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C859" t="str">
+        <v>06:26</v>
+      </c>
+      <c r="D859" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E859" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F859" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G859" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H859" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I859" t="str">
+        <v/>
+      </c>
+      <c r="J859" t="str">
+        <v/>
+      </c>
+      <c r="K859" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B860" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C860" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D860" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E860" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F860" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G860" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H860" t="str">
+        <v>N</v>
+      </c>
+      <c r="I860" t="str">
+        <v/>
+      </c>
+      <c r="J860" t="str">
+        <v/>
+      </c>
+      <c r="K860" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B861" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C861" t="str">
+        <v>06:35</v>
+      </c>
+      <c r="D861" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E861" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F861" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G861" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H861" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I861" t="str">
+        <v/>
+      </c>
+      <c r="J861" t="str">
+        <v/>
+      </c>
+      <c r="K861" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B862" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C862" t="str">
+        <v>09:50</v>
+      </c>
+      <c r="D862" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E862" t="str">
+        <v>dyl</v>
+      </c>
+      <c r="F862" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G862" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H862" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I862" t="str">
+        <v/>
+      </c>
+      <c r="J862" t="str">
+        <v/>
+      </c>
+      <c r="K862" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B863" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C863" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D863" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E863" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F863" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G863" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H863" t="str">
+        <v>N</v>
+      </c>
+      <c r="I863" t="str">
+        <v/>
+      </c>
+      <c r="J863" t="str">
+        <v/>
+      </c>
+      <c r="K863" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B864" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C864" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D864" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E864" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F864" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G864" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H864" t="str">
+        <v>N</v>
+      </c>
+      <c r="I864" t="str">
+        <v/>
+      </c>
+      <c r="J864" t="str">
+        <v/>
+      </c>
+      <c r="K864" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B865" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C865" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D865" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E865" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F865" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G865" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H865" t="str">
+        <v>N</v>
+      </c>
+      <c r="I865" t="str">
+        <v/>
+      </c>
+      <c r="J865" t="str">
+        <v/>
+      </c>
+      <c r="K865" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B866" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C866" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D866" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E866" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F866" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G866" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H866" t="str">
+        <v>N</v>
+      </c>
+      <c r="I866" t="str">
+        <v/>
+      </c>
+      <c r="J866" t="str">
+        <v/>
+      </c>
+      <c r="K866" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B867" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C867" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D867" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E867" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F867" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G867" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H867" t="str">
+        <v>N</v>
+      </c>
+      <c r="I867" t="str">
+        <v/>
+      </c>
+      <c r="J867" t="str">
+        <v/>
+      </c>
+      <c r="K867" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B868" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C868" t="str">
+        <v>06:30</v>
+      </c>
+      <c r="D868" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E868" t="str">
+        <v>ant</v>
+      </c>
+      <c r="F868" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G868" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H868" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I868" t="str">
+        <v>ordered. DH</v>
+      </c>
+      <c r="J868" t="str">
+        <v/>
+      </c>
+      <c r="K868" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="B869" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C869" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D869" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="E869" t="str">
+        <v>Anthoy Dylan</v>
+      </c>
+      <c r="F869" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G869" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H869" t="str">
+        <v>N</v>
+      </c>
+      <c r="I869" t="str">
+        <v/>
+      </c>
+      <c r="J869" t="str">
+        <v/>
+      </c>
+      <c r="K869" t="str">
+        <v>S-mun32nxo-1qix8</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K855"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K869"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-09-30T05:42:40.608Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -30682,13 +30682,13 @@
         <v>Day</v>
       </c>
       <c r="C866" t="str">
-        <v>(not entered)</v>
+        <v>13:29</v>
       </c>
       <c r="D866" t="str">
         <v>Anthoy Dylan</v>
       </c>
       <c r="E866" t="str">
-        <v>Anthoy Dylan</v>
+        <v>ant tim</v>
       </c>
       <c r="F866" t="str">
         <v>Once a Week</v>
@@ -30697,7 +30697,7 @@
         <v>Deep clean around mills</v>
       </c>
       <c r="H866" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I866" t="str">
         <v/>

</xml_diff>

<commit_message>
Checklist log update 2026-09-30T07:50:09.678Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -30612,13 +30612,13 @@
         <v>Day</v>
       </c>
       <c r="C864" t="str">
-        <v>(not entered)</v>
+        <v>17:30</v>
       </c>
       <c r="D864" t="str">
         <v>Anthoy Dylan</v>
       </c>
       <c r="E864" t="str">
-        <v>Anthoy Dylan</v>
+        <v>ant</v>
       </c>
       <c r="F864" t="str">
         <v>During Processing</v>
@@ -30627,7 +30627,7 @@
         <v>Inspect &amp; clean steam vent</v>
       </c>
       <c r="H864" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I864" t="str">
         <v/>
@@ -30647,13 +30647,13 @@
         <v>Day</v>
       </c>
       <c r="C865" t="str">
-        <v>(not entered)</v>
+        <v>17:49</v>
       </c>
       <c r="D865" t="str">
         <v>Anthoy Dylan</v>
       </c>
       <c r="E865" t="str">
-        <v>Anthoy Dylan</v>
+        <v>dylan</v>
       </c>
       <c r="F865" t="str">
         <v>During Processing</v>
@@ -30662,7 +30662,7 @@
         <v>Empty drop box at end of shift</v>
       </c>
       <c r="H865" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I865" t="str">
         <v/>

</xml_diff>

<commit_message>
Checklist log update 2026-09-30T19:53:39.159Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K869"/>
+  <dimension ref="A1:K883"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -30814,9 +30814,499 @@
         <v>S-mun32nxo-1qix8</v>
       </c>
     </row>
+    <row r="870">
+      <c r="A870" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B870" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C870" t="str">
+        <v>18:01</v>
+      </c>
+      <c r="D870" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E870" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F870" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G870" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H870" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I870" t="str">
+        <v/>
+      </c>
+      <c r="J870" t="str">
+        <v/>
+      </c>
+      <c r="K870" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B871" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C871" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D871" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E871" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F871" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G871" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H871" t="str">
+        <v>N</v>
+      </c>
+      <c r="I871" t="str">
+        <v/>
+      </c>
+      <c r="J871" t="str">
+        <v/>
+      </c>
+      <c r="K871" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B872" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C872" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D872" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E872" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F872" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G872" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H872" t="str">
+        <v>N</v>
+      </c>
+      <c r="I872" t="str">
+        <v/>
+      </c>
+      <c r="J872" t="str">
+        <v/>
+      </c>
+      <c r="K872" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B873" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C873" t="str">
+        <v>18:03</v>
+      </c>
+      <c r="D873" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E873" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F873" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G873" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H873" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I873" t="str">
+        <v/>
+      </c>
+      <c r="J873" t="str">
+        <v/>
+      </c>
+      <c r="K873" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B874" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C874" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D874" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E874" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F874" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G874" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H874" t="str">
+        <v>N</v>
+      </c>
+      <c r="I874" t="str">
+        <v/>
+      </c>
+      <c r="J874" t="str">
+        <v/>
+      </c>
+      <c r="K874" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B875" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C875" t="str">
+        <v>18:05</v>
+      </c>
+      <c r="D875" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E875" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F875" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G875" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H875" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I875" t="str">
+        <v/>
+      </c>
+      <c r="J875" t="str">
+        <v/>
+      </c>
+      <c r="K875" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B876" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C876" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="D876" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E876" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F876" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G876" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H876" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I876" t="str">
+        <v/>
+      </c>
+      <c r="J876" t="str">
+        <v/>
+      </c>
+      <c r="K876" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B877" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C877" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="D877" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E877" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F877" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G877" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H877" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I877" t="str">
+        <v/>
+      </c>
+      <c r="J877" t="str">
+        <v/>
+      </c>
+      <c r="K877" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B878" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C878" t="str">
+        <v>05:30</v>
+      </c>
+      <c r="D878" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E878" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F878" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G878" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H878" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I878" t="str">
+        <v/>
+      </c>
+      <c r="J878" t="str">
+        <v/>
+      </c>
+      <c r="K878" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B879" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C879" t="str">
+        <v>05:20</v>
+      </c>
+      <c r="D879" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E879" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F879" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G879" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H879" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I879" t="str">
+        <v/>
+      </c>
+      <c r="J879" t="str">
+        <v/>
+      </c>
+      <c r="K879" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B880" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C880" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D880" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E880" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F880" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G880" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H880" t="str">
+        <v>N</v>
+      </c>
+      <c r="I880" t="str">
+        <v/>
+      </c>
+      <c r="J880" t="str">
+        <v/>
+      </c>
+      <c r="K880" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B881" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C881" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D881" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E881" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F881" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G881" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H881" t="str">
+        <v>N</v>
+      </c>
+      <c r="I881" t="str">
+        <v/>
+      </c>
+      <c r="J881" t="str">
+        <v/>
+      </c>
+      <c r="K881" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B882" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C882" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D882" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E882" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F882" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G882" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H882" t="str">
+        <v>N</v>
+      </c>
+      <c r="I882" t="str">
+        <v/>
+      </c>
+      <c r="J882" t="str">
+        <v/>
+      </c>
+      <c r="K882" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B883" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C883" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D883" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E883" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F883" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G883" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H883" t="str">
+        <v>N</v>
+      </c>
+      <c r="I883" t="str">
+        <v/>
+      </c>
+      <c r="J883" t="str">
+        <v/>
+      </c>
+      <c r="K883" t="str">
+        <v>S-munt2sa4-umddf</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K869"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K883"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-10-01T08:02:05.980Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K883"/>
+  <dimension ref="A1:K897"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -31304,9 +31304,499 @@
         <v>S-munt2sa4-umddf</v>
       </c>
     </row>
+    <row r="884">
+      <c r="A884" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B884" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C884" t="str">
+        <v>18:01</v>
+      </c>
+      <c r="D884" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E884" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F884" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G884" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H884" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I884" t="str">
+        <v/>
+      </c>
+      <c r="J884" t="str">
+        <v/>
+      </c>
+      <c r="K884" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B885" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C885" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D885" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E885" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F885" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G885" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H885" t="str">
+        <v>N</v>
+      </c>
+      <c r="I885" t="str">
+        <v/>
+      </c>
+      <c r="J885" t="str">
+        <v/>
+      </c>
+      <c r="K885" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B886" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C886" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D886" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E886" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F886" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G886" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H886" t="str">
+        <v>N</v>
+      </c>
+      <c r="I886" t="str">
+        <v/>
+      </c>
+      <c r="J886" t="str">
+        <v/>
+      </c>
+      <c r="K886" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B887" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C887" t="str">
+        <v>18:03</v>
+      </c>
+      <c r="D887" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E887" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F887" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G887" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H887" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I887" t="str">
+        <v/>
+      </c>
+      <c r="J887" t="str">
+        <v/>
+      </c>
+      <c r="K887" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B888" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C888" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D888" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E888" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F888" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G888" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H888" t="str">
+        <v>N</v>
+      </c>
+      <c r="I888" t="str">
+        <v/>
+      </c>
+      <c r="J888" t="str">
+        <v/>
+      </c>
+      <c r="K888" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B889" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C889" t="str">
+        <v>18:05</v>
+      </c>
+      <c r="D889" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E889" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F889" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G889" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H889" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I889" t="str">
+        <v/>
+      </c>
+      <c r="J889" t="str">
+        <v/>
+      </c>
+      <c r="K889" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B890" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C890" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="D890" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E890" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F890" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G890" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H890" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I890" t="str">
+        <v/>
+      </c>
+      <c r="J890" t="str">
+        <v/>
+      </c>
+      <c r="K890" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B891" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C891" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="D891" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E891" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F891" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G891" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H891" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I891" t="str">
+        <v/>
+      </c>
+      <c r="J891" t="str">
+        <v/>
+      </c>
+      <c r="K891" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B892" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C892" t="str">
+        <v>05:30</v>
+      </c>
+      <c r="D892" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E892" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F892" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G892" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H892" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I892" t="str">
+        <v/>
+      </c>
+      <c r="J892" t="str">
+        <v/>
+      </c>
+      <c r="K892" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B893" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C893" t="str">
+        <v>05:20</v>
+      </c>
+      <c r="D893" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E893" t="str">
+        <v>Ken</v>
+      </c>
+      <c r="F893" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G893" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H893" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I893" t="str">
+        <v/>
+      </c>
+      <c r="J893" t="str">
+        <v/>
+      </c>
+      <c r="K893" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B894" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C894" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D894" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E894" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F894" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G894" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H894" t="str">
+        <v>N</v>
+      </c>
+      <c r="I894" t="str">
+        <v/>
+      </c>
+      <c r="J894" t="str">
+        <v/>
+      </c>
+      <c r="K894" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B895" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C895" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D895" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E895" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F895" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G895" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H895" t="str">
+        <v>N</v>
+      </c>
+      <c r="I895" t="str">
+        <v/>
+      </c>
+      <c r="J895" t="str">
+        <v/>
+      </c>
+      <c r="K895" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B896" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C896" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D896" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E896" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F896" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G896" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H896" t="str">
+        <v>N</v>
+      </c>
+      <c r="I896" t="str">
+        <v/>
+      </c>
+      <c r="J896" t="str">
+        <v/>
+      </c>
+      <c r="K896" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B897" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C897" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D897" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="E897" t="str">
+        <v>TP/Ken</v>
+      </c>
+      <c r="F897" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G897" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H897" t="str">
+        <v>N</v>
+      </c>
+      <c r="I897" t="str">
+        <v/>
+      </c>
+      <c r="J897" t="str">
+        <v/>
+      </c>
+      <c r="K897" t="str">
+        <v>S-mup8x5yq-5dbvp</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K883"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K897"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-10-01T18:58:43.902Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K897"/>
+  <dimension ref="A1:K911"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -31794,9 +31794,499 @@
         <v>S-mup8x5yq-5dbvp</v>
       </c>
     </row>
+    <row r="898">
+      <c r="A898" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B898" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C898" t="str">
+        <v>20:57</v>
+      </c>
+      <c r="D898" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E898" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F898" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G898" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H898" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I898" t="str">
+        <v/>
+      </c>
+      <c r="J898" t="str">
+        <v/>
+      </c>
+      <c r="K898" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B899" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C899" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D899" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E899" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F899" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G899" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H899" t="str">
+        <v>N</v>
+      </c>
+      <c r="I899" t="str">
+        <v/>
+      </c>
+      <c r="J899" t="str">
+        <v/>
+      </c>
+      <c r="K899" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B900" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C900" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D900" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E900" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F900" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G900" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H900" t="str">
+        <v>N</v>
+      </c>
+      <c r="I900" t="str">
+        <v/>
+      </c>
+      <c r="J900" t="str">
+        <v/>
+      </c>
+      <c r="K900" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B901" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C901" t="str">
+        <v>20:58</v>
+      </c>
+      <c r="D901" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E901" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F901" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G901" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H901" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I901" t="str">
+        <v/>
+      </c>
+      <c r="J901" t="str">
+        <v/>
+      </c>
+      <c r="K901" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B902" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C902" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D902" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E902" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F902" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G902" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H902" t="str">
+        <v>N</v>
+      </c>
+      <c r="I902" t="str">
+        <v/>
+      </c>
+      <c r="J902" t="str">
+        <v/>
+      </c>
+      <c r="K902" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B903" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C903" t="str">
+        <v>20:58</v>
+      </c>
+      <c r="D903" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E903" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F903" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G903" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H903" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I903" t="str">
+        <v/>
+      </c>
+      <c r="J903" t="str">
+        <v/>
+      </c>
+      <c r="K903" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B904" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C904" t="str">
+        <v>20:58</v>
+      </c>
+      <c r="D904" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E904" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F904" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G904" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H904" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I904" t="str">
+        <v/>
+      </c>
+      <c r="J904" t="str">
+        <v/>
+      </c>
+      <c r="K904" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B905" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C905" t="str">
+        <v>04:58</v>
+      </c>
+      <c r="D905" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E905" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F905" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G905" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H905" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I905" t="str">
+        <v/>
+      </c>
+      <c r="J905" t="str">
+        <v/>
+      </c>
+      <c r="K905" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B906" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C906" t="str">
+        <v>04:58</v>
+      </c>
+      <c r="D906" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E906" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F906" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G906" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H906" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I906" t="str">
+        <v/>
+      </c>
+      <c r="J906" t="str">
+        <v/>
+      </c>
+      <c r="K906" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B907" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C907" t="str">
+        <v>04:58</v>
+      </c>
+      <c r="D907" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E907" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F907" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G907" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H907" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I907" t="str">
+        <v/>
+      </c>
+      <c r="J907" t="str">
+        <v/>
+      </c>
+      <c r="K907" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B908" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C908" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D908" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E908" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F908" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G908" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H908" t="str">
+        <v>N</v>
+      </c>
+      <c r="I908" t="str">
+        <v/>
+      </c>
+      <c r="J908" t="str">
+        <v/>
+      </c>
+      <c r="K908" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B909" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C909" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D909" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E909" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F909" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G909" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H909" t="str">
+        <v>N</v>
+      </c>
+      <c r="I909" t="str">
+        <v/>
+      </c>
+      <c r="J909" t="str">
+        <v/>
+      </c>
+      <c r="K909" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B910" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C910" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D910" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E910" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F910" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G910" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H910" t="str">
+        <v>N</v>
+      </c>
+      <c r="I910" t="str">
+        <v/>
+      </c>
+      <c r="J910" t="str">
+        <v/>
+      </c>
+      <c r="K910" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B911" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C911" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D911" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E911" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F911" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G911" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H911" t="str">
+        <v>N</v>
+      </c>
+      <c r="I911" t="str">
+        <v/>
+      </c>
+      <c r="J911" t="str">
+        <v/>
+      </c>
+      <c r="K911" t="str">
+        <v>S-mupwcihh-1akf3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K897"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K911"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-10-02T06:49:24.310Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K911"/>
+  <dimension ref="A1:K925"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -32284,9 +32284,499 @@
         <v>S-mupwcihh-1akf3</v>
       </c>
     </row>
+    <row r="912">
+      <c r="A912" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B912" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C912" t="str">
+        <v>06:41</v>
+      </c>
+      <c r="D912" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E912" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F912" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G912" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H912" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I912" t="str">
+        <v/>
+      </c>
+      <c r="J912" t="str">
+        <v/>
+      </c>
+      <c r="K912" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B913" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C913" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D913" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E913" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F913" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G913" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H913" t="str">
+        <v>N</v>
+      </c>
+      <c r="I913" t="str">
+        <v/>
+      </c>
+      <c r="J913" t="str">
+        <v/>
+      </c>
+      <c r="K913" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B914" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C914" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D914" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E914" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F914" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G914" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H914" t="str">
+        <v>N</v>
+      </c>
+      <c r="I914" t="str">
+        <v/>
+      </c>
+      <c r="J914" t="str">
+        <v/>
+      </c>
+      <c r="K914" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B915" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C915" t="str">
+        <v>06:41</v>
+      </c>
+      <c r="D915" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E915" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F915" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G915" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H915" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I915" t="str">
+        <v/>
+      </c>
+      <c r="J915" t="str">
+        <v/>
+      </c>
+      <c r="K915" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B916" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C916" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D916" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E916" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F916" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G916" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H916" t="str">
+        <v>N</v>
+      </c>
+      <c r="I916" t="str">
+        <v/>
+      </c>
+      <c r="J916" t="str">
+        <v/>
+      </c>
+      <c r="K916" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B917" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C917" t="str">
+        <v>06:41</v>
+      </c>
+      <c r="D917" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E917" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F917" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G917" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H917" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I917" t="str">
+        <v/>
+      </c>
+      <c r="J917" t="str">
+        <v/>
+      </c>
+      <c r="K917" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B918" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C918" t="str">
+        <v>09:36</v>
+      </c>
+      <c r="D918" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E918" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F918" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G918" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H918" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I918" t="str">
+        <v/>
+      </c>
+      <c r="J918" t="str">
+        <v/>
+      </c>
+      <c r="K918" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B919" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C919" t="str">
+        <v>15:48</v>
+      </c>
+      <c r="D919" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E919" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F919" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G919" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H919" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I919" t="str">
+        <v/>
+      </c>
+      <c r="J919" t="str">
+        <v/>
+      </c>
+      <c r="K919" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B920" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C920" t="str">
+        <v>16:49</v>
+      </c>
+      <c r="D920" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E920" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F920" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G920" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H920" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I920" t="str">
+        <v/>
+      </c>
+      <c r="J920" t="str">
+        <v/>
+      </c>
+      <c r="K920" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B921" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C921" t="str">
+        <v>16:49</v>
+      </c>
+      <c r="D921" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E921" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F921" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G921" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H921" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I921" t="str">
+        <v/>
+      </c>
+      <c r="J921" t="str">
+        <v/>
+      </c>
+      <c r="K921" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B922" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C922" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D922" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E922" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F922" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G922" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H922" t="str">
+        <v>N</v>
+      </c>
+      <c r="I922" t="str">
+        <v/>
+      </c>
+      <c r="J922" t="str">
+        <v/>
+      </c>
+      <c r="K922" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B923" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C923" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D923" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E923" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F923" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G923" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H923" t="str">
+        <v>N</v>
+      </c>
+      <c r="I923" t="str">
+        <v/>
+      </c>
+      <c r="J923" t="str">
+        <v/>
+      </c>
+      <c r="K923" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B924" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C924" t="str">
+        <v>09:02</v>
+      </c>
+      <c r="D924" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E924" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F924" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G924" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H924" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I924" t="str">
+        <v>Full</v>
+      </c>
+      <c r="J924" t="str">
+        <v/>
+      </c>
+      <c r="K924" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B925" t="str">
+        <v>Day</v>
+      </c>
+      <c r="C925" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D925" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="E925" t="str">
+        <v>DH LS</v>
+      </c>
+      <c r="F925" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G925" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H925" t="str">
+        <v>N</v>
+      </c>
+      <c r="I925" t="str">
+        <v/>
+      </c>
+      <c r="J925" t="str">
+        <v/>
+      </c>
+      <c r="K925" t="str">
+        <v>S-mupwdwp0-2vc6z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K911"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K925"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-10-02T18:02:34.084Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K925"/>
+  <dimension ref="A1:K939"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -32774,9 +32774,499 @@
         <v>S-mupwdwp0-2vc6z</v>
       </c>
     </row>
+    <row r="926">
+      <c r="A926" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B926" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C926" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D926" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E926" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F926" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G926" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H926" t="str">
+        <v>N</v>
+      </c>
+      <c r="I926" t="str">
+        <v/>
+      </c>
+      <c r="J926" t="str">
+        <v/>
+      </c>
+      <c r="K926" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B927" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C927" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D927" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E927" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F927" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G927" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H927" t="str">
+        <v>N</v>
+      </c>
+      <c r="I927" t="str">
+        <v/>
+      </c>
+      <c r="J927" t="str">
+        <v/>
+      </c>
+      <c r="K927" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B928" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C928" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D928" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E928" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F928" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G928" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H928" t="str">
+        <v>N</v>
+      </c>
+      <c r="I928" t="str">
+        <v/>
+      </c>
+      <c r="J928" t="str">
+        <v/>
+      </c>
+      <c r="K928" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B929" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C929" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D929" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E929" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F929" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G929" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H929" t="str">
+        <v>N</v>
+      </c>
+      <c r="I929" t="str">
+        <v/>
+      </c>
+      <c r="J929" t="str">
+        <v/>
+      </c>
+      <c r="K929" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B930" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C930" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D930" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E930" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F930" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G930" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H930" t="str">
+        <v>N</v>
+      </c>
+      <c r="I930" t="str">
+        <v/>
+      </c>
+      <c r="J930" t="str">
+        <v/>
+      </c>
+      <c r="K930" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B931" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C931" t="str">
+        <v>19:23</v>
+      </c>
+      <c r="D931" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E931" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F931" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G931" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H931" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I931" t="str">
+        <v/>
+      </c>
+      <c r="J931" t="str">
+        <v/>
+      </c>
+      <c r="K931" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B932" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C932" t="str">
+        <v>20:58</v>
+      </c>
+      <c r="D932" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E932" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F932" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G932" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H932" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I932" t="str">
+        <v/>
+      </c>
+      <c r="J932" t="str">
+        <v/>
+      </c>
+      <c r="K932" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B933" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C933" t="str">
+        <v>03:23</v>
+      </c>
+      <c r="D933" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E933" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F933" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G933" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H933" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I933" t="str">
+        <v/>
+      </c>
+      <c r="J933" t="str">
+        <v/>
+      </c>
+      <c r="K933" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B934" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C934" t="str">
+        <v>04:02</v>
+      </c>
+      <c r="D934" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E934" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F934" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G934" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H934" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I934" t="str">
+        <v/>
+      </c>
+      <c r="J934" t="str">
+        <v/>
+      </c>
+      <c r="K934" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B935" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C935" t="str">
+        <v>04:02</v>
+      </c>
+      <c r="D935" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E935" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F935" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G935" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H935" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I935" t="str">
+        <v/>
+      </c>
+      <c r="J935" t="str">
+        <v/>
+      </c>
+      <c r="K935" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B936" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C936" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D936" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E936" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F936" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G936" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H936" t="str">
+        <v>N</v>
+      </c>
+      <c r="I936" t="str">
+        <v/>
+      </c>
+      <c r="J936" t="str">
+        <v/>
+      </c>
+      <c r="K936" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B937" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C937" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D937" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E937" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F937" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G937" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H937" t="str">
+        <v>N</v>
+      </c>
+      <c r="I937" t="str">
+        <v/>
+      </c>
+      <c r="J937" t="str">
+        <v/>
+      </c>
+      <c r="K937" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B938" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C938" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D938" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E938" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F938" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G938" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H938" t="str">
+        <v>N</v>
+      </c>
+      <c r="I938" t="str">
+        <v/>
+      </c>
+      <c r="J938" t="str">
+        <v/>
+      </c>
+      <c r="K938" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B939" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C939" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D939" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E939" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F939" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G939" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H939" t="str">
+        <v>N</v>
+      </c>
+      <c r="I939" t="str">
+        <v/>
+      </c>
+      <c r="J939" t="str">
+        <v/>
+      </c>
+      <c r="K939" t="str">
+        <v>S-mur9ta1z-ffi29</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K925"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K939"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-10-03T15:49:54.358Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K939"/>
+  <dimension ref="A1:K953"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -33264,9 +33264,499 @@
         <v>S-mur9ta1z-ffi29</v>
       </c>
     </row>
+    <row r="940">
+      <c r="A940" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B940" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C940" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D940" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E940" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F940" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G940" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H940" t="str">
+        <v>N</v>
+      </c>
+      <c r="I940" t="str">
+        <v/>
+      </c>
+      <c r="J940" t="str">
+        <v/>
+      </c>
+      <c r="K940" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B941" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C941" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D941" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E941" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F941" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G941" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H941" t="str">
+        <v>N</v>
+      </c>
+      <c r="I941" t="str">
+        <v/>
+      </c>
+      <c r="J941" t="str">
+        <v/>
+      </c>
+      <c r="K941" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B942" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C942" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D942" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E942" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F942" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G942" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H942" t="str">
+        <v>N</v>
+      </c>
+      <c r="I942" t="str">
+        <v/>
+      </c>
+      <c r="J942" t="str">
+        <v/>
+      </c>
+      <c r="K942" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B943" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C943" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D943" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E943" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F943" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G943" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H943" t="str">
+        <v>N</v>
+      </c>
+      <c r="I943" t="str">
+        <v/>
+      </c>
+      <c r="J943" t="str">
+        <v/>
+      </c>
+      <c r="K943" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B944" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C944" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D944" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E944" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F944" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G944" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H944" t="str">
+        <v>N</v>
+      </c>
+      <c r="I944" t="str">
+        <v/>
+      </c>
+      <c r="J944" t="str">
+        <v/>
+      </c>
+      <c r="K944" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B945" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C945" t="str">
+        <v>18:48</v>
+      </c>
+      <c r="D945" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E945" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F945" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G945" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H945" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I945" t="str">
+        <v/>
+      </c>
+      <c r="J945" t="str">
+        <v/>
+      </c>
+      <c r="K945" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B946" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C946" t="str">
+        <v>21:49</v>
+      </c>
+      <c r="D946" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E946" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F946" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G946" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H946" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I946" t="str">
+        <v/>
+      </c>
+      <c r="J946" t="str">
+        <v/>
+      </c>
+      <c r="K946" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B947" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C947" t="str">
+        <v>03:49</v>
+      </c>
+      <c r="D947" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E947" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F947" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G947" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H947" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I947" t="str">
+        <v/>
+      </c>
+      <c r="J947" t="str">
+        <v/>
+      </c>
+      <c r="K947" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B948" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C948" t="str">
+        <v>05:49</v>
+      </c>
+      <c r="D948" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E948" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F948" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G948" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H948" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I948" t="str">
+        <v/>
+      </c>
+      <c r="J948" t="str">
+        <v/>
+      </c>
+      <c r="K948" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B949" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C949" t="str">
+        <v>05:49</v>
+      </c>
+      <c r="D949" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E949" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F949" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G949" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H949" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I949" t="str">
+        <v/>
+      </c>
+      <c r="J949" t="str">
+        <v/>
+      </c>
+      <c r="K949" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B950" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C950" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D950" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E950" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F950" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G950" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H950" t="str">
+        <v>N</v>
+      </c>
+      <c r="I950" t="str">
+        <v/>
+      </c>
+      <c r="J950" t="str">
+        <v/>
+      </c>
+      <c r="K950" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B951" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C951" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D951" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E951" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F951" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G951" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H951" t="str">
+        <v>N</v>
+      </c>
+      <c r="I951" t="str">
+        <v/>
+      </c>
+      <c r="J951" t="str">
+        <v/>
+      </c>
+      <c r="K951" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B952" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C952" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D952" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E952" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F952" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G952" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H952" t="str">
+        <v>N</v>
+      </c>
+      <c r="I952" t="str">
+        <v/>
+      </c>
+      <c r="J952" t="str">
+        <v/>
+      </c>
+      <c r="K952" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B953" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C953" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D953" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="E953" t="str">
+        <v>tp ts</v>
+      </c>
+      <c r="F953" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G953" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H953" t="str">
+        <v>N</v>
+      </c>
+      <c r="I953" t="str">
+        <v/>
+      </c>
+      <c r="J953" t="str">
+        <v/>
+      </c>
+      <c r="K953" t="str">
+        <v>S-mus44gy5-y62id</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K939"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K953"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-10-03T20:48:26.994Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K953"/>
+  <dimension ref="A1:K967"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -33754,9 +33754,499 @@
         <v>S-mus44gy5-y62id</v>
       </c>
     </row>
+    <row r="954">
+      <c r="A954" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B954" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C954" t="str">
+        <v>06:41</v>
+      </c>
+      <c r="D954" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E954" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F954" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G954" t="str">
+        <v>Check Grecon is OK</v>
+      </c>
+      <c r="H954" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I954" t="str">
+        <v/>
+      </c>
+      <c r="J954" t="str">
+        <v/>
+      </c>
+      <c r="K954" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B955" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C955" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D955" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E955" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F955" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G955" t="str">
+        <v>Check fuel Hammermill Magnet</v>
+      </c>
+      <c r="H955" t="str">
+        <v>N</v>
+      </c>
+      <c r="I955" t="str">
+        <v/>
+      </c>
+      <c r="J955" t="str">
+        <v/>
+      </c>
+      <c r="K955" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B956" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C956" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D956" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E956" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F956" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G956" t="str">
+        <v>Check Dry Hammermill Magnet</v>
+      </c>
+      <c r="H956" t="str">
+        <v>N</v>
+      </c>
+      <c r="I956" t="str">
+        <v/>
+      </c>
+      <c r="J956" t="str">
+        <v/>
+      </c>
+      <c r="K956" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B957" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C957" t="str">
+        <v>06:41</v>
+      </c>
+      <c r="D957" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E957" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F957" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G957" t="str">
+        <v>Check Grecon Tank is on operational level</v>
+      </c>
+      <c r="H957" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I957" t="str">
+        <v/>
+      </c>
+      <c r="J957" t="str">
+        <v/>
+      </c>
+      <c r="K957" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B958" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C958" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D958" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E958" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F958" t="str">
+        <v>Before Startup</v>
+      </c>
+      <c r="G958" t="str">
+        <v>Check water sprayers are functioning correctly</v>
+      </c>
+      <c r="H958" t="str">
+        <v>N</v>
+      </c>
+      <c r="I958" t="str">
+        <v/>
+      </c>
+      <c r="J958" t="str">
+        <v/>
+      </c>
+      <c r="K958" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B959" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C959" t="str">
+        <v>06:41</v>
+      </c>
+      <c r="D959" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E959" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F959" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G959" t="str">
+        <v>Check Mill Adjustment Sheet is up to date</v>
+      </c>
+      <c r="H959" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I959" t="str">
+        <v/>
+      </c>
+      <c r="J959" t="str">
+        <v/>
+      </c>
+      <c r="K959" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B960" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C960" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D960" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E960" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F960" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G960" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H960" t="str">
+        <v>N</v>
+      </c>
+      <c r="I960" t="str">
+        <v/>
+      </c>
+      <c r="J960" t="str">
+        <v/>
+      </c>
+      <c r="K960" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B961" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C961" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D961" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E961" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F961" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G961" t="str">
+        <v>Purge mills — 200 pumps each</v>
+      </c>
+      <c r="H961" t="str">
+        <v>N</v>
+      </c>
+      <c r="I961" t="str">
+        <v/>
+      </c>
+      <c r="J961" t="str">
+        <v/>
+      </c>
+      <c r="K961" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B962" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C962" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D962" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E962" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F962" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G962" t="str">
+        <v>Inspect &amp; clean steam vent</v>
+      </c>
+      <c r="H962" t="str">
+        <v>N</v>
+      </c>
+      <c r="I962" t="str">
+        <v/>
+      </c>
+      <c r="J962" t="str">
+        <v/>
+      </c>
+      <c r="K962" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B963" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C963" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D963" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E963" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F963" t="str">
+        <v>During Processing</v>
+      </c>
+      <c r="G963" t="str">
+        <v>Empty drop box at end of shift</v>
+      </c>
+      <c r="H963" t="str">
+        <v>N</v>
+      </c>
+      <c r="I963" t="str">
+        <v/>
+      </c>
+      <c r="J963" t="str">
+        <v/>
+      </c>
+      <c r="K963" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B964" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C964" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D964" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E964" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F964" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G964" t="str">
+        <v>Deep clean around mills</v>
+      </c>
+      <c r="H964" t="str">
+        <v>N</v>
+      </c>
+      <c r="I964" t="str">
+        <v/>
+      </c>
+      <c r="J964" t="str">
+        <v/>
+      </c>
+      <c r="K964" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B965" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C965" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D965" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E965" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F965" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G965" t="str">
+        <v>Clean diverters / shavings 1 into 2 transition</v>
+      </c>
+      <c r="H965" t="str">
+        <v>N</v>
+      </c>
+      <c r="I965" t="str">
+        <v/>
+      </c>
+      <c r="J965" t="str">
+        <v/>
+      </c>
+      <c r="K965" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B966" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C966" t="str">
+        <v>06:41</v>
+      </c>
+      <c r="D966" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E966" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F966" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G966" t="str">
+        <v>Check drinking water tank level</v>
+      </c>
+      <c r="H966" t="str">
+        <v>N</v>
+      </c>
+      <c r="I966" t="str">
+        <v/>
+      </c>
+      <c r="J966" t="str">
+        <v/>
+      </c>
+      <c r="K966" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B967" t="str">
+        <v>Night</v>
+      </c>
+      <c r="C967" t="str">
+        <v>(not entered)</v>
+      </c>
+      <c r="D967" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="E967" t="str">
+        <v>DH AH</v>
+      </c>
+      <c r="F967" t="str">
+        <v>Once a Week</v>
+      </c>
+      <c r="G967" t="str">
+        <v>Empty all bins and wheel barrows</v>
+      </c>
+      <c r="H967" t="str">
+        <v>N</v>
+      </c>
+      <c r="I967" t="str">
+        <v/>
+      </c>
+      <c r="J967" t="str">
+        <v/>
+      </c>
+      <c r="K967" t="str">
+        <v>S-muskipfv-y2k9p</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K953"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K967"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist log update 2026-10-04T05:07:37.000Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -33972,7 +33972,7 @@
         <v>Night</v>
       </c>
       <c r="C960" t="str">
-        <v>(not entered)</v>
+        <v>09:20</v>
       </c>
       <c r="D960" t="str">
         <v>DH AH</v>
@@ -33987,7 +33987,7 @@
         <v>Purge mills — 200 pumps each</v>
       </c>
       <c r="H960" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I960" t="str">
         <v/>
@@ -34112,7 +34112,7 @@
         <v>Night</v>
       </c>
       <c r="C964" t="str">
-        <v>(not entered)</v>
+        <v>14:33</v>
       </c>
       <c r="D964" t="str">
         <v>DH AH</v>
@@ -34127,7 +34127,7 @@
         <v>Deep clean around mills</v>
       </c>
       <c r="H964" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I964" t="str">
         <v/>
@@ -34197,10 +34197,10 @@
         <v>Check drinking water tank level</v>
       </c>
       <c r="H966" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I966" t="str">
-        <v/>
+        <v>50%</v>
       </c>
       <c r="J966" t="str">
         <v/>

</xml_diff>

<commit_message>
Checklist log update 2026-10-04T07:51:59.340Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -34007,7 +34007,7 @@
         <v>Night</v>
       </c>
       <c r="C961" t="str">
-        <v>(not entered)</v>
+        <v>15:33</v>
       </c>
       <c r="D961" t="str">
         <v>DH AH</v>
@@ -34022,7 +34022,7 @@
         <v>Purge mills — 200 pumps each</v>
       </c>
       <c r="H961" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I961" t="str">
         <v/>
@@ -34042,7 +34042,7 @@
         <v>Night</v>
       </c>
       <c r="C962" t="str">
-        <v>(not entered)</v>
+        <v>17:51</v>
       </c>
       <c r="D962" t="str">
         <v>DH AH</v>
@@ -34057,7 +34057,7 @@
         <v>Inspect &amp; clean steam vent</v>
       </c>
       <c r="H962" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I962" t="str">
         <v/>
@@ -34077,7 +34077,7 @@
         <v>Night</v>
       </c>
       <c r="C963" t="str">
-        <v>(not entered)</v>
+        <v>17:51</v>
       </c>
       <c r="D963" t="str">
         <v>DH AH</v>
@@ -34092,7 +34092,7 @@
         <v>Empty drop box at end of shift</v>
       </c>
       <c r="H963" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="I963" t="str">
         <v/>

</xml_diff>

<commit_message>
Checklist log update 2026-10-07T05:02:07.167Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="510">
   <si>
     <t>Date</t>
   </si>
@@ -1535,6 +1535,15 @@
   </si>
   <si>
     <t>S-muxgjz0v-q3yxr</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>08:35</t>
+  </si>
+  <si>
+    <t>LS</t>
   </si>
 </sst>
 </file>
@@ -36017,7 +36026,7 @@
         <v>505</v>
       </c>
       <c r="E969" s="17" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F969" s="18" t="s">
         <v>16</v>
@@ -36052,7 +36061,7 @@
         <v>505</v>
       </c>
       <c r="E970" s="17" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F970" s="18" t="s">
         <v>16</v>
@@ -36081,7 +36090,7 @@
         <v>12</v>
       </c>
       <c r="C971" s="15" t="s">
-        <v>21</v>
+        <v>508</v>
       </c>
       <c r="D971" s="17" t="s">
         <v>505</v>
@@ -36095,8 +36104,8 @@
       <c r="G971" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="H971" s="8" t="s">
-        <v>23</v>
+      <c r="H971" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I971" s="17" t="s">
         <v>19</v>
@@ -36151,13 +36160,13 @@
         <v>12</v>
       </c>
       <c r="C973" s="15" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D973" s="17" t="s">
         <v>505</v>
       </c>
       <c r="E973" s="17" t="s">
-        <v>505</v>
+        <v>77</v>
       </c>
       <c r="F973" s="18" t="s">
         <v>28</v>
@@ -36165,8 +36174,8 @@
       <c r="G973" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="H973" s="8" t="s">
-        <v>23</v>
+      <c r="H973" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I973" s="17" t="s">
         <v>19</v>
@@ -36186,13 +36195,13 @@
         <v>12</v>
       </c>
       <c r="C974" s="15" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D974" s="17" t="s">
         <v>505</v>
       </c>
       <c r="E974" s="17" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="F974" s="18" t="s">
         <v>28</v>
@@ -36200,8 +36209,8 @@
       <c r="G974" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="H974" s="8" t="s">
-        <v>23</v>
+      <c r="H974" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I974" s="17" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-07T05:15:59.618Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="512">
   <si>
     <t>Date</t>
   </si>
@@ -1544,6 +1544,12 @@
   </si>
   <si>
     <t>LS</t>
+  </si>
+  <si>
+    <t>15:15</t>
+  </si>
+  <si>
+    <t>TR/BA</t>
   </si>
 </sst>
 </file>
@@ -36230,13 +36236,13 @@
         <v>12</v>
       </c>
       <c r="C975" s="15" t="s">
-        <v>21</v>
+        <v>510</v>
       </c>
       <c r="D975" s="17" t="s">
         <v>505</v>
       </c>
       <c r="E975" s="17" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="F975" s="18" t="s">
         <v>28</v>
@@ -36244,8 +36250,8 @@
       <c r="G975" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="H975" s="8" t="s">
-        <v>23</v>
+      <c r="H975" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I975" s="17" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-07T05:31:19.164Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="513">
   <si>
     <t>Date</t>
   </si>
@@ -1550,6 +1550,9 @@
   </si>
   <si>
     <t>TR/BA</t>
+  </si>
+  <si>
+    <t>15:36</t>
   </si>
 </sst>
 </file>
@@ -36411,13 +36414,13 @@
         <v>12</v>
       </c>
       <c r="C980" s="15" t="s">
-        <v>21</v>
+        <v>512</v>
       </c>
       <c r="D980" s="17" t="s">
         <v>505</v>
       </c>
       <c r="E980" s="17" t="s">
-        <v>505</v>
+        <v>287</v>
       </c>
       <c r="F980" s="18" t="s">
         <v>35</v>
@@ -36425,8 +36428,8 @@
       <c r="G980" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="H980" s="8" t="s">
-        <v>23</v>
+      <c r="H980" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I980" s="17" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-07T07:27:07.955Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="516">
   <si>
     <t>Date</t>
   </si>
@@ -1537,6 +1537,9 @@
     <t>S-muxgjz0v-q3yxr</t>
   </si>
   <si>
+    <t>16:11</t>
+  </si>
+  <si>
     <t>N/A</t>
   </si>
   <si>
@@ -1550,6 +1553,12 @@
   </si>
   <si>
     <t>TR/BA</t>
+  </si>
+  <si>
+    <t>17:26</t>
+  </si>
+  <si>
+    <t>17:27</t>
   </si>
   <si>
     <t>15:36</t>
@@ -36029,13 +36038,13 @@
         <v>12</v>
       </c>
       <c r="C969" s="15" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="D969" s="17" t="s">
         <v>505</v>
       </c>
       <c r="E969" s="17" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F969" s="18" t="s">
         <v>16</v>
@@ -36043,8 +36052,8 @@
       <c r="G969" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="H969" s="8" t="s">
-        <v>23</v>
+      <c r="H969" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I969" s="17" t="s">
         <v>19</v>
@@ -36070,7 +36079,7 @@
         <v>505</v>
       </c>
       <c r="E970" s="17" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F970" s="18" t="s">
         <v>16</v>
@@ -36099,7 +36108,7 @@
         <v>12</v>
       </c>
       <c r="C971" s="15" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D971" s="17" t="s">
         <v>505</v>
@@ -36210,7 +36219,7 @@
         <v>505</v>
       </c>
       <c r="E974" s="17" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F974" s="18" t="s">
         <v>28</v>
@@ -36239,13 +36248,13 @@
         <v>12</v>
       </c>
       <c r="C975" s="15" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D975" s="17" t="s">
         <v>505</v>
       </c>
       <c r="E975" s="17" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F975" s="18" t="s">
         <v>28</v>
@@ -36274,13 +36283,13 @@
         <v>12</v>
       </c>
       <c r="C976" s="15" t="s">
-        <v>21</v>
+        <v>513</v>
       </c>
       <c r="D976" s="17" t="s">
         <v>505</v>
       </c>
       <c r="E976" s="17" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="F976" s="18" t="s">
         <v>28</v>
@@ -36288,8 +36297,8 @@
       <c r="G976" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="H976" s="8" t="s">
-        <v>23</v>
+      <c r="H976" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I976" s="17" t="s">
         <v>19</v>
@@ -36309,13 +36318,13 @@
         <v>12</v>
       </c>
       <c r="C977" s="15" t="s">
-        <v>21</v>
+        <v>514</v>
       </c>
       <c r="D977" s="17" t="s">
         <v>505</v>
       </c>
       <c r="E977" s="17" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="F977" s="18" t="s">
         <v>28</v>
@@ -36323,8 +36332,8 @@
       <c r="G977" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="H977" s="8" t="s">
-        <v>23</v>
+      <c r="H977" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I977" s="17" t="s">
         <v>19</v>
@@ -36414,7 +36423,7 @@
         <v>12</v>
       </c>
       <c r="C980" s="15" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="D980" s="17" t="s">
         <v>505</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-07T19:45:07.594Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10791" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10945" uniqueCount="522">
   <si>
     <t>Date</t>
   </si>
@@ -1562,6 +1562,24 @@
   </si>
   <si>
     <t>15:36</t>
+  </si>
+  <si>
+    <t>2026-10-08</t>
+  </si>
+  <si>
+    <t>18:35</t>
+  </si>
+  <si>
+    <t>S-muxgjwva-8b4fj</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>21:12</t>
+  </si>
+  <si>
+    <t>23:12</t>
   </si>
 </sst>
 </file>
@@ -2137,7 +2155,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K981"/>
+  <dimension ref="A1:K995"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -36485,8 +36503,498 @@
         <v>506</v>
       </c>
     </row>
+    <row r="982" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A982" s="20" t="s">
+        <v>516</v>
+      </c>
+      <c r="B982" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C982" s="20" t="s">
+        <v>517</v>
+      </c>
+      <c r="D982" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="E982" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="F982" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G982" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H982" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I982" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J982" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K982" s="24" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="983" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A983" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B983" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C983" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D983" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E983" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="F983" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G983" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H983" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I983" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J983" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K983" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="984" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A984" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B984" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C984" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D984" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E984" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="F984" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G984" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H984" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I984" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J984" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K984" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="985" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A985" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B985" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C985" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D985" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E985" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F985" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G985" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H985" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I985" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J985" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K985" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="986" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A986" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B986" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C986" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D986" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E986" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F986" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G986" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H986" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I986" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J986" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K986" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="987" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A987" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B987" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C987" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="D987" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E987" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F987" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G987" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H987" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I987" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J987" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K987" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="988" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A988" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B988" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C988" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="D988" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E988" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F988" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G988" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H988" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I988" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J988" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K988" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="989" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A989" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B989" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C989" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D989" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E989" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F989" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G989" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H989" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I989" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J989" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K989" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="990" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A990" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B990" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C990" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D990" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E990" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F990" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G990" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H990" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I990" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J990" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K990" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="991" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A991" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B991" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C991" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D991" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E991" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F991" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G991" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H991" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I991" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J991" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K991" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="992" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A992" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B992" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C992" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D992" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E992" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F992" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G992" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H992" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I992" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J992" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K992" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="993" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A993" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B993" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C993" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D993" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E993" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F993" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G993" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H993" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I993" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J993" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K993" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="994" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A994" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B994" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C994" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D994" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E994" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F994" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G994" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H994" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I994" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J994" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K994" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="995" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A995" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B995" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C995" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D995" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E995" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F995" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G995" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H995" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I995" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J995" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K995" s="7" t="s">
+        <v>518</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K981"/>
+  <autoFilter ref="A1:K995"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-08T05:23:49.960Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10945" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11099" uniqueCount="525">
   <si>
     <t>Date</t>
   </si>
@@ -1580,6 +1580,15 @@
   </si>
   <si>
     <t>23:12</t>
+  </si>
+  <si>
+    <t>06:28</t>
+  </si>
+  <si>
+    <t>S-muyioktt-ru8be</t>
+  </si>
+  <si>
+    <t>15:23</t>
   </si>
 </sst>
 </file>
@@ -2155,7 +2164,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K995"/>
+  <dimension ref="A1:K1009"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -36993,8 +37002,498 @@
         <v>518</v>
       </c>
     </row>
+    <row r="996" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A996" s="9" t="s">
+        <v>516</v>
+      </c>
+      <c r="B996" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C996" s="9" t="s">
+        <v>522</v>
+      </c>
+      <c r="D996" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="E996" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="F996" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G996" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H996" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I996" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J996" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K996" s="14" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="997" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A997" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B997" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C997" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D997" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E997" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F997" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G997" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H997" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I997" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J997" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K997" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="998" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A998" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B998" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C998" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D998" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E998" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F998" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G998" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H998" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I998" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J998" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K998" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="999" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A999" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B999" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C999" s="15" t="s">
+        <v>522</v>
+      </c>
+      <c r="D999" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E999" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F999" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G999" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H999" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I999" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J999" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K999" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1000" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1000" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1000" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1000" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1000" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1000" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1000" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1000" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1000" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1000" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1000" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1000" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1001" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1001" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1001" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1001" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="D1001" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1001" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1001" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1001" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1001" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1001" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1001" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1001" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1002" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1002" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1002" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1002" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1002" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1002" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1002" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1002" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1002" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1002" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1002" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1002" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1003" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1003" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1003" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1003" s="15" t="s">
+        <v>524</v>
+      </c>
+      <c r="D1003" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1003" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1003" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1003" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1003" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1003" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1003" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1003" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1004" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1004" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1004" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1004" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1004" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1004" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1004" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1004" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1004" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1004" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1004" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1004" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1005" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1005" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1005" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1005" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1005" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1005" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1005" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1005" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1005" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1005" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1005" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1005" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1006" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1006" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1006" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1006" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1006" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1006" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1006" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1006" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1006" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1006" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1006" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1006" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1007" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1007" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1007" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1007" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1007" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1007" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1007" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1007" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1007" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1007" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1007" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1007" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1008" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1008" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1008" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1008" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1008" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1008" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1008" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1008" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1008" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1008" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1008" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1008" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="1009" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1009" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B1009" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1009" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1009" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1009" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1009" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1009" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1009" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1009" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1009" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1009" s="19" t="s">
+        <v>523</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K995"/>
+  <autoFilter ref="A1:K1009"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-08T20:01:36.723Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11099" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11253" uniqueCount="529">
   <si>
     <t>Date</t>
   </si>
@@ -1589,6 +1589,18 @@
   </si>
   <si>
     <t>15:23</t>
+  </si>
+  <si>
+    <t>2026-10-09</t>
+  </si>
+  <si>
+    <t>S-muzjbl5w-54dne</t>
+  </si>
+  <si>
+    <t>22:51</t>
+  </si>
+  <si>
+    <t>1/3 left</t>
   </si>
 </sst>
 </file>
@@ -2164,7 +2176,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1009"/>
+  <dimension ref="A1:K1023"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -37492,8 +37504,498 @@
         <v>523</v>
       </c>
     </row>
+    <row r="1010" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1010" s="20" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1010" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1010" s="20" t="s">
+        <v>517</v>
+      </c>
+      <c r="D1010" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1010" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="F1010" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1010" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1010" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1010" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1010" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1010" s="24" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1011" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1011" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1011" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1011" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1011" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1011" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="F1011" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1011" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1011" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1011" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1011" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1011" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1012" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1012" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1012" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1012" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1012" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1012" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="F1012" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1012" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1012" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1012" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1012" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1012" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1013" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1013" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1013" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1013" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1013" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1013" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1013" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1013" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1013" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1013" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1013" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1013" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1014" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1014" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1014" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1014" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1014" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1014" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1014" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1014" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1014" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1014" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1014" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1014" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1015" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1015" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1015" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1015" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1015" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1015" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1015" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1015" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1015" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1015" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1015" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1015" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1016" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1016" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1016" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1016" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1016" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1016" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1016" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1016" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1016" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1016" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1016" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1016" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1017" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1017" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1017" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1017" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1017" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1017" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1017" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1017" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1017" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1017" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1017" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1017" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1018" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1018" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1018" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1018" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1018" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1018" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1018" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1018" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1018" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1018" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1018" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1018" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1019" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1019" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1019" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1019" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1019" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1019" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1019" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1019" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1019" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1019" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1019" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1019" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1020" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1020" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1020" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1020" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1020" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1020" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1020" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1020" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1020" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1020" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1020" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1020" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1021" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1021" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1021" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1021" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1021" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1021" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1021" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1021" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1021" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1021" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1021" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1021" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1022" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1022" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1022" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1022" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="D1022" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1022" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1022" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1022" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1022" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1022" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="J1022" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1022" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="1023" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1023" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1023" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1023" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1023" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1023" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1023" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1023" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1023" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1023" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1023" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1023" s="7" t="s">
+        <v>526</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1009"/>
+  <autoFilter ref="A1:K1023"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-09T08:02:23.682Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11253" uniqueCount="529">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11407" uniqueCount="533">
   <si>
     <t>Date</t>
   </si>
@@ -1601,6 +1601,18 @@
   </si>
   <si>
     <t>1/3 left</t>
+  </si>
+  <si>
+    <t>S-muzyngub-wjlq1</t>
+  </si>
+  <si>
+    <t>06:03</t>
+  </si>
+  <si>
+    <t>09:03</t>
+  </si>
+  <si>
+    <t>15:39</t>
   </si>
 </sst>
 </file>
@@ -2176,7 +2188,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1023"/>
+  <dimension ref="A1:K1037"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -37994,8 +38006,498 @@
         <v>526</v>
       </c>
     </row>
+    <row r="1024" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1024" s="9" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1024" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1024" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1024" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1024" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1024" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1024" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1024" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1024" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1024" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1024" s="14" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1025" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1025" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1025" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1025" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1025" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1025" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1025" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1025" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1025" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1025" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1025" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1025" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1026" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1026" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1026" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1026" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1026" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1026" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1026" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1026" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1026" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1026" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1026" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1026" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1027" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1027" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1027" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1027" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1027" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1027" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1027" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1027" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1027" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1027" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1027" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1027" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1028" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1028" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1028" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1028" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1028" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1028" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1028" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1028" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1028" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1028" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1028" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1028" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1029" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1029" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1029" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1029" s="15" t="s">
+        <v>530</v>
+      </c>
+      <c r="D1029" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1029" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1029" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1029" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1029" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1029" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1029" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1029" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1030" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1030" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1030" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1030" s="15" t="s">
+        <v>531</v>
+      </c>
+      <c r="D1030" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1030" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1030" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1030" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1030" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1030" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1030" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1030" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1031" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1031" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1031" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1031" s="15" t="s">
+        <v>532</v>
+      </c>
+      <c r="D1031" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1031" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1031" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1031" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1031" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1031" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1031" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1031" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1032" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1032" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1032" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1032" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="D1032" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1032" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1032" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1032" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1032" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1032" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1032" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1032" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1033" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1033" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1033" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1033" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="D1033" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1033" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1033" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1033" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1033" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1033" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1033" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1033" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1034" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1034" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1034" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1034" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1034" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1034" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1034" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1034" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1034" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1034" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1034" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1034" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1035" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1035" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1035" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1035" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1035" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1035" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1035" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1035" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1035" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1035" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1035" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1035" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1036" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1036" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1036" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1036" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1036" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1036" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1036" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1036" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1036" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1036" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1036" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1036" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="1037" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1037" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1037" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1037" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1037" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1037" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1037" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1037" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1037" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1037" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1037" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1037" s="19" t="s">
+        <v>529</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1023"/>
+  <autoFilter ref="A1:K1037"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-09T08:34:11.068Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11407" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11561" uniqueCount="534">
   <si>
     <t>Date</t>
   </si>
@@ -1613,6 +1613,9 @@
   </si>
   <si>
     <t>15:39</t>
+  </si>
+  <si>
+    <t>S-muzynbl5-0cng4</t>
   </si>
 </sst>
 </file>
@@ -2188,7 +2191,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1037"/>
+  <dimension ref="A1:K1051"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -38496,8 +38499,498 @@
         <v>529</v>
       </c>
     </row>
+    <row r="1038" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1038" s="20" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1038" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1038" s="20" t="s">
+        <v>517</v>
+      </c>
+      <c r="D1038" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1038" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="F1038" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1038" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1038" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1038" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1038" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1038" s="24" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1039" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1039" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1039" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1039" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1039" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1039" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="F1039" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1039" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1039" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1039" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1039" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1039" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1040" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1040" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1040" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1040" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1040" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1040" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="F1040" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1040" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1040" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1040" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1040" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1040" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1041" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1041" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1041" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1041" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1041" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1041" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1041" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1041" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1041" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1041" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1041" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1041" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1042" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1042" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1042" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1042" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1042" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1042" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1042" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1042" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1042" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1042" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1042" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1042" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1043" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1043" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1043" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1043" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1043" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1043" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1043" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1043" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1043" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1043" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1043" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1043" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1044" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1044" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1044" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1044" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1044" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1044" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1044" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1044" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1044" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1044" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1044" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1044" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1045" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1045" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1045" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1045" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1045" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1045" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1045" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1045" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1045" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1045" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1045" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1045" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1046" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1046" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1046" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1046" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1046" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1046" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1046" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1046" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1046" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1046" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1046" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1046" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1047" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1047" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1047" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1047" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1047" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1047" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1047" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1047" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1047" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1047" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1047" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1047" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1048" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1048" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1048" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1048" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1048" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1048" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1048" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1048" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1048" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1048" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1048" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1048" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1049" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1049" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1049" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1049" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1049" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1049" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1049" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1049" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1049" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1049" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1049" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1049" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1050" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1050" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1050" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1050" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="D1050" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1050" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1050" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1050" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1050" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1050" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="J1050" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1050" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="1051" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1051" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1051" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1051" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1051" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1051" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1051" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1051" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1051" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1051" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1051" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1051" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1037"/>
+  <autoFilter ref="A1:K1051"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-09T20:05:49.470Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11561" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11715" uniqueCount="538">
   <si>
     <t>Date</t>
   </si>
@@ -1616,6 +1616,18 @@
   </si>
   <si>
     <t>S-muzynbl5-0cng4</t>
+  </si>
+  <si>
+    <t>2026-10-10</t>
+  </si>
+  <si>
+    <t>S-mv12jpxq-4ev4p</t>
+  </si>
+  <si>
+    <t>00:30</t>
+  </si>
+  <si>
+    <t>10:34</t>
   </si>
 </sst>
 </file>
@@ -2191,7 +2203,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1051"/>
+  <dimension ref="A1:K1065"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -38989,8 +39001,498 @@
         <v>533</v>
       </c>
     </row>
+    <row r="1052" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1052" s="9" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1052" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1052" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="D1052" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1052" s="11" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1052" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1052" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1052" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1052" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1052" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1052" s="14" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1053" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1053" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1053" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1053" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1053" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1053" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1053" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1053" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1053" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1053" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1053" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1053" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1054" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1054" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1054" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1054" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1054" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1054" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1054" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1054" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1054" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1054" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1054" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1054" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1055" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1055" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1055" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1055" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="D1055" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1055" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1055" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1055" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1055" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1055" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1055" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1055" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1056" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1056" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1056" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1056" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1056" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1056" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1056" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1056" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1056" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1056" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1056" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1056" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1057" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1057" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1057" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1057" s="15" t="s">
+        <v>536</v>
+      </c>
+      <c r="D1057" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1057" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1057" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1057" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1057" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1057" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1057" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1057" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1058" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1058" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1058" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1058" s="15" t="s">
+        <v>537</v>
+      </c>
+      <c r="D1058" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1058" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="F1058" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1058" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1058" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1058" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1058" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1058" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1059" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1059" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1059" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1059" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1059" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1059" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1059" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1059" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1059" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1059" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1059" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1059" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1060" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1060" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1060" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1060" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1060" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1060" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1060" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1060" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1060" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1060" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1060" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1060" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1061" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1061" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1061" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1061" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="D1061" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1061" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="F1061" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1061" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1061" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1061" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1061" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1061" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1062" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1062" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1062" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1062" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1062" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1062" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1062" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1062" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1062" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1062" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1062" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1062" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1063" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1063" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1063" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1063" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1063" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1063" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1063" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1063" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1063" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1063" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1063" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1063" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1064" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1064" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1064" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1064" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1064" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1064" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1064" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1064" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1064" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1064" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1064" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1064" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1065" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1065" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1065" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1065" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1065" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1065" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1065" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1065" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1065" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1065" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1065" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1065" s="19" t="s">
+        <v>535</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1051"/>
+  <autoFilter ref="A1:K1065"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-10T07:44:27.987Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11715" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11869" uniqueCount="541">
   <si>
     <t>Date</t>
   </si>
@@ -1628,6 +1628,15 @@
   </si>
   <si>
     <t>10:34</t>
+  </si>
+  <si>
+    <t>S-mv12jlxh-aemu1</t>
+  </si>
+  <si>
+    <t>15:07</t>
+  </si>
+  <si>
+    <t>17:43</t>
   </si>
 </sst>
 </file>
@@ -2203,7 +2212,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1065"/>
+  <dimension ref="A1:K1079"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -39491,8 +39500,498 @@
         <v>535</v>
       </c>
     </row>
+    <row r="1066" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1066" s="20" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1066" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1066" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="D1066" s="22" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1066" s="22" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1066" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1066" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1066" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1066" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1066" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1066" s="24" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1067" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1067" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1067" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1067" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1067" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1067" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1067" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1067" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1067" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1067" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1067" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1067" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1068" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1068" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1068" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1068" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1068" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1068" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1068" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1068" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1068" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1068" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1068" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1068" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1069" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1069" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1069" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1069" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D1069" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1069" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1069" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1069" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1069" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1069" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1069" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1069" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1070" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1070" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1070" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1070" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1070" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1070" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1070" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1070" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1070" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1070" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1070" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1070" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1071" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1071" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1071" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1071" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1071" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1071" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1071" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1071" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1071" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1071" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1071" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1071" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1072" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1072" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1072" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1072" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1072" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1072" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1072" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1072" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1072" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1072" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1072" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1072" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1073" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1073" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1073" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1073" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="D1073" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1073" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1073" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1073" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1073" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1073" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1073" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1073" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1074" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1074" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1074" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1074" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="D1074" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1074" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1074" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1074" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1074" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1074" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1074" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1074" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1075" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1075" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1075" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1075" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="D1075" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1075" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1075" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1075" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1075" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1075" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1075" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1075" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1076" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1076" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1076" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1076" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1076" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1076" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1076" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1076" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1076" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1076" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1076" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1076" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1077" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1077" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1077" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1077" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1077" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1077" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1077" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1077" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1077" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1077" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1077" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1077" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1078" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1078" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1078" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1078" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1078" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1078" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1078" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1078" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1078" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1078" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1078" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1078" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="1079" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1079" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B1079" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1079" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1079" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1079" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="F1079" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1079" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1079" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1079" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1079" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1079" s="7" t="s">
+        <v>538</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1065"/>
+  <autoFilter ref="A1:K1079"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-12T19:20:34.277Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11869" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12023" uniqueCount="548">
   <si>
     <t>Date</t>
   </si>
@@ -1637,6 +1637,27 @@
   </si>
   <si>
     <t>17:43</t>
+  </si>
+  <si>
+    <t>2026-10-13</t>
+  </si>
+  <si>
+    <t>18:14</t>
+  </si>
+  <si>
+    <t>DH KB</t>
+  </si>
+  <si>
+    <t>S-mv5gcnq1-4i6l5</t>
+  </si>
+  <si>
+    <t>03:24</t>
+  </si>
+  <si>
+    <t>21:34</t>
+  </si>
+  <si>
+    <t>37 %</t>
   </si>
 </sst>
 </file>
@@ -2212,7 +2233,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1079"/>
+  <dimension ref="A1:K1093"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -39990,8 +40011,498 @@
         <v>538</v>
       </c>
     </row>
+    <row r="1080" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1080" s="9" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1080" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1080" s="9" t="s">
+        <v>542</v>
+      </c>
+      <c r="D1080" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1080" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1080" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1080" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1080" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1080" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1080" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1080" s="14" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1081" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1081" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1081" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1081" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1081" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1081" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1081" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1081" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1081" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1081" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1081" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1081" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1082" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1082" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1082" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1082" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1082" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1082" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1082" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1082" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1082" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1082" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1082" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1082" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1083" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1083" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1083" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1083" s="15" t="s">
+        <v>542</v>
+      </c>
+      <c r="D1083" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1083" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1083" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1083" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1083" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1083" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1083" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1083" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1084" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1084" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1084" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1084" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1084" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1084" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1084" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1084" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1084" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1084" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1084" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1084" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1085" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1085" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1085" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1085" s="15" t="s">
+        <v>404</v>
+      </c>
+      <c r="D1085" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1085" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1085" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1085" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1085" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1085" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1085" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1085" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1086" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1086" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1086" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1086" s="15" t="s">
+        <v>301</v>
+      </c>
+      <c r="D1086" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1086" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1086" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1086" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1086" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1086" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1086" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1086" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1087" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1087" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1087" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1087" s="15" t="s">
+        <v>545</v>
+      </c>
+      <c r="D1087" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1087" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1087" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1087" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1087" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1087" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1087" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1087" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1088" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1088" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1088" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1088" s="15" t="s">
+        <v>460</v>
+      </c>
+      <c r="D1088" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1088" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1088" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1088" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1088" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1088" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1088" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1088" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1089" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1089" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1089" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1089" s="15" t="s">
+        <v>460</v>
+      </c>
+      <c r="D1089" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1089" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1089" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1089" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1089" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1089" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1089" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1089" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1090" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1090" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1090" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1090" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1090" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1090" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1090" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1090" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1090" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1090" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1090" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1090" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1091" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1091" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1091" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1091" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1091" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1091" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1091" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1091" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1091" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1091" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1091" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1091" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1092" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1092" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1092" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1092" s="15" t="s">
+        <v>546</v>
+      </c>
+      <c r="D1092" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1092" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1092" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1092" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1092" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1092" s="17" t="s">
+        <v>547</v>
+      </c>
+      <c r="J1092" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1092" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="1093" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1093" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1093" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1093" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1093" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1093" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1093" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1093" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1093" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1093" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1093" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1093" s="19" t="s">
+        <v>544</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1079"/>
+  <autoFilter ref="A1:K1093"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-13T07:46:44.896Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12023" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12177" uniqueCount="551">
   <si>
     <t>Date</t>
   </si>
@@ -1658,6 +1658,15 @@
   </si>
   <si>
     <t>37 %</t>
+  </si>
+  <si>
+    <t>TP/KEN</t>
+  </si>
+  <si>
+    <t>S-mv5gcimx-x393o</t>
+  </si>
+  <si>
+    <t>17:29</t>
   </si>
 </sst>
 </file>
@@ -2233,7 +2242,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1093"/>
+  <dimension ref="A1:K1107"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -40501,8 +40510,498 @@
         <v>544</v>
       </c>
     </row>
+    <row r="1094" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1094" s="20" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1094" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1094" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="D1094" s="22" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1094" s="22" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1094" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1094" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1094" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1094" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1094" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1094" s="24" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1095" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1095" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1095" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1095" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1095" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1095" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1095" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1095" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1095" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1095" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1095" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1095" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1096" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1096" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1096" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1096" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1096" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1096" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1096" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1096" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1096" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1096" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1096" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1096" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1097" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1097" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1097" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1097" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D1097" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1097" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1097" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1097" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1097" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1097" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1097" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1097" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1098" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1098" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1098" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1098" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1098" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1098" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1098" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1098" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1098" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1098" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1098" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1098" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1099" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1099" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1099" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1099" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="D1099" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1099" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1099" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1099" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1099" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1099" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1099" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1099" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1100" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1100" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1100" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1100" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1100" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1100" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1100" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1100" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1100" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1100" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1100" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1100" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1101" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1101" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1101" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1101" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1101" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1101" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1101" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1101" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1101" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1101" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1101" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1101" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1102" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1102" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1102" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1102" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="D1102" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1102" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1102" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1102" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1102" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1102" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1102" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1102" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1103" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1103" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1103" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1103" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="D1103" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1103" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="F1103" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1103" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1103" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1103" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1103" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1103" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1104" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1104" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1104" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1104" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1104" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1104" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1104" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1104" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1104" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1104" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1104" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1104" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1105" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1105" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1105" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1105" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1105" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1105" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1105" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1105" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1105" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1105" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1105" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1105" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1106" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1106" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1106" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1106" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1106" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1106" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1106" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1106" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1106" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1106" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1106" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1106" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1107" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1107" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1107" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1107" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1107" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1107" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1107" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1107" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1107" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1107" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1107" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1107" s="7" t="s">
+        <v>549</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1093"/>
+  <autoFilter ref="A1:K1107"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-13T19:22:35.838Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12177" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12331" uniqueCount="557">
   <si>
     <t>Date</t>
   </si>
@@ -1667,6 +1667,24 @@
   </si>
   <si>
     <t>17:29</t>
+  </si>
+  <si>
+    <t>2026-10-14</t>
+  </si>
+  <si>
+    <t>S-mv6gps4l-h2xs2</t>
+  </si>
+  <si>
+    <t>18:29</t>
+  </si>
+  <si>
+    <t>05:06</t>
+  </si>
+  <si>
+    <t>05:10</t>
+  </si>
+  <si>
+    <t>19:20</t>
   </si>
 </sst>
 </file>
@@ -2242,7 +2260,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1107"/>
+  <dimension ref="A1:K1121"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -41000,8 +41018,498 @@
         <v>549</v>
       </c>
     </row>
+    <row r="1108" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1108" s="9" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1108" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1108" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1108" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1108" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1108" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1108" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1108" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1108" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1108" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1108" s="14" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1109" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1109" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1109" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1109" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1109" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1109" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1109" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1109" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1109" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1109" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1109" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1109" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1110" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1110" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1110" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1110" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1110" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1110" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1110" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1110" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1110" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1110" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1110" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1110" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1111" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1111" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1111" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1111" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="D1111" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1111" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1111" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1111" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1111" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1111" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="J1111" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1111" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1112" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1112" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1112" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1112" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1112" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1112" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1112" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1112" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1112" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1112" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1112" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1112" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1113" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1113" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1113" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1113" s="15" t="s">
+        <v>553</v>
+      </c>
+      <c r="D1113" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1113" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1113" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1113" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1113" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1113" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1113" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1113" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1114" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1114" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1114" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1114" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1114" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1114" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1114" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1114" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1114" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1114" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1114" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1114" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1115" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1115" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1115" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1115" s="15" t="s">
+        <v>454</v>
+      </c>
+      <c r="D1115" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1115" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1115" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1115" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1115" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1115" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1115" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1115" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1116" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1116" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1116" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1116" s="15" t="s">
+        <v>407</v>
+      </c>
+      <c r="D1116" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1116" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1116" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1116" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1116" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1116" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1116" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1116" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1117" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1117" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1117" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1117" s="15" t="s">
+        <v>554</v>
+      </c>
+      <c r="D1117" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1117" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1117" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1117" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1117" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1117" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1117" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1117" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1118" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1118" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1118" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1118" s="15" t="s">
+        <v>555</v>
+      </c>
+      <c r="D1118" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1118" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1118" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1118" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1118" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1118" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1118" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1118" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1119" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1119" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1119" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1119" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1119" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1119" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1119" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1119" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1119" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1119" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1119" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1119" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1120" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1120" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1120" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1120" s="15" t="s">
+        <v>556</v>
+      </c>
+      <c r="D1120" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1120" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1120" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1120" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1120" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1120" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="J1120" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1120" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="1121" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1121" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1121" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1121" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1121" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1121" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1121" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1121" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1121" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1121" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1121" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1121" s="19" t="s">
+        <v>552</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1107"/>
+  <autoFilter ref="A1:K1121"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-14T08:03:56.728Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12331" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12485" uniqueCount="562">
   <si>
     <t>Date</t>
   </si>
@@ -1685,6 +1685,21 @@
   </si>
   <si>
     <t>19:20</t>
+  </si>
+  <si>
+    <t>S-mv74a44v-pswz8</t>
+  </si>
+  <si>
+    <t>14:59</t>
+  </si>
+  <si>
+    <t>Ken-</t>
+  </si>
+  <si>
+    <t>17:14</t>
+  </si>
+  <si>
+    <t>17:13</t>
   </si>
 </sst>
 </file>
@@ -2260,7 +2275,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1121"/>
+  <dimension ref="A1:K1135"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -41508,8 +41523,498 @@
         <v>552</v>
       </c>
     </row>
+    <row r="1122" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1122" s="20" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1122" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1122" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1122" s="22" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1122" s="22" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1122" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1122" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1122" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1122" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1122" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1122" s="24" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1123" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1123" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1123" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1123" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1123" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1123" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1123" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1123" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1123" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1123" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1123" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1123" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1124" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1124" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1124" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1124" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1124" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1124" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1124" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1124" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1124" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1124" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1124" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1124" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1125" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1125" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1125" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1125" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1125" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1125" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1125" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1125" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1125" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1125" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1125" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1125" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1126" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1126" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1126" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1126" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1126" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1126" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1126" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1126" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1126" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1126" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1126" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1126" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1127" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1127" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1127" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1127" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1127" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1127" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1127" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1127" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1127" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1127" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1127" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1127" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1128" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1128" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1128" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1128" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D1128" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1128" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1128" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1128" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1128" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1128" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1128" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1128" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1129" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1129" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1129" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1129" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="D1129" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1129" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="F1129" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1129" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1129" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1129" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1129" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1129" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1130" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1130" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1130" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1130" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="D1130" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1130" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="F1130" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1130" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1130" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1130" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1130" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1130" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1131" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1131" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1131" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1131" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="D1131" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1131" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1131" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1131" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1131" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1131" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1131" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1131" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1132" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1132" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1132" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1132" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1132" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1132" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1132" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1132" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1132" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1132" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1132" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1132" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1133" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1133" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1133" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1133" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1133" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1133" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1133" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1133" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1133" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1133" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1133" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1133" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1134" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1134" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1134" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1134" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1134" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1134" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1134" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1134" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1134" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1134" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1134" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1134" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1135" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1135" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1135" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1135" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1135" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="E1135" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F1135" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1135" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1135" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1135" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1135" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1135" s="7" t="s">
+        <v>557</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1121"/>
+  <autoFilter ref="A1:K1135"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-14T08:05:04.365Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12485" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12639" uniqueCount="565">
   <si>
     <t>Date</t>
   </si>
@@ -1700,6 +1700,15 @@
   </si>
   <si>
     <t>17:13</t>
+  </si>
+  <si>
+    <t>S-mv7tpytr-th6b4</t>
+  </si>
+  <si>
+    <t>18:08</t>
+  </si>
+  <si>
+    <t>18:07</t>
   </si>
 </sst>
 </file>
@@ -2275,7 +2284,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1135"/>
+  <dimension ref="A1:K1149"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -42013,8 +42022,498 @@
         <v>557</v>
       </c>
     </row>
+    <row r="1136" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1136" s="9" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1136" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1136" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="D1136" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1136" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1136" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1136" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1136" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1136" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1136" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1136" s="14" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1137" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1137" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1137" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1137" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1137" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1137" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1137" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1137" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1137" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1137" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1137" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1137" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1138" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1138" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1138" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1138" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1138" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1138" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1138" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1138" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1138" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1138" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1138" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1138" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1139" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1139" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1139" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1139" s="15" t="s">
+        <v>563</v>
+      </c>
+      <c r="D1139" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1139" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1139" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1139" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1139" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1139" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1139" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1139" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1140" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1140" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1140" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1140" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1140" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1140" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1140" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1140" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1140" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1140" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1140" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1140" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1141" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1141" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1141" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1141" s="15" t="s">
+        <v>564</v>
+      </c>
+      <c r="D1141" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1141" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1141" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1141" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1141" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1141" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1141" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1141" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1142" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1142" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1142" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1142" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1142" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1142" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1142" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1142" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1142" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1142" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1142" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1142" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1143" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1143" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1143" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1143" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1143" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1143" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1143" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1143" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1143" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1143" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1143" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1143" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1144" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1144" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1144" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1144" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1144" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1144" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1144" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1144" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1144" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1144" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1144" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1144" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1145" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1145" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1145" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1145" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1145" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1145" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1145" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1145" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1145" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1145" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1145" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1145" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1146" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1146" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1146" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1146" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1146" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1146" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1146" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1146" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1146" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1146" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1146" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1146" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1147" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1147" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1147" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1147" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1147" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1147" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1147" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1147" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1147" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1147" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1147" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1147" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1148" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1148" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1148" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1148" s="15" t="s">
+        <v>432</v>
+      </c>
+      <c r="D1148" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1148" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1148" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1148" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1148" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1148" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="J1148" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1148" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="1149" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1149" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1149" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1149" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1149" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1149" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="F1149" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1149" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1149" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1149" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1149" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1149" s="19" t="s">
+        <v>562</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1135"/>
+  <autoFilter ref="A1:K1149"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-15T07:18:45.737Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12639" uniqueCount="565">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12793" uniqueCount="570">
   <si>
     <t>Date</t>
   </si>
@@ -1709,6 +1709,21 @@
   </si>
   <si>
     <t>18:07</t>
+  </si>
+  <si>
+    <t>2026-10-15</t>
+  </si>
+  <si>
+    <t>TS TP CF GC PB TR AS</t>
+  </si>
+  <si>
+    <t>S-mv8ke03y-tst34</t>
+  </si>
+  <si>
+    <t>17:18</t>
+  </si>
+  <si>
+    <t>Spoke with Topher regarding 30% level</t>
   </si>
 </sst>
 </file>
@@ -2284,7 +2299,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1149"/>
+  <dimension ref="A1:K1163"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -42512,8 +42527,498 @@
         <v>562</v>
       </c>
     </row>
+    <row r="1150" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1150" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1150" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1150" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="D1150" s="22" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1150" s="22" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1150" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1150" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1150" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1150" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1150" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1150" s="24" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1151" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1151" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1151" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1151" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1151" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1151" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1151" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1151" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1151" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1151" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1151" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1151" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1152" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1152" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1152" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1152" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1152" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1152" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1152" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1152" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1152" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1152" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1152" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1152" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1153" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1153" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1153" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1153" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1153" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1153" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1153" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1153" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1153" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1153" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1153" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1153" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1154" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1154" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1154" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1154" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1154" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1154" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1154" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1154" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1154" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1154" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1154" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1154" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1155" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1155" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1155" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1155" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1155" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1155" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1155" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1155" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1155" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1155" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1155" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1155" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1156" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1156" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1156" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1156" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1156" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1156" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1156" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1156" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1156" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1156" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1156" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1156" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1157" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1157" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1157" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1157" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="D1157" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1157" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1157" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1157" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1157" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1157" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1157" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1157" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1158" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1158" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1158" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1158" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="D1158" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1158" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1158" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1158" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1158" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1158" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1158" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1158" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1159" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1159" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1159" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1159" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="D1159" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1159" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1159" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1159" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1159" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1159" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1159" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1159" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1160" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1160" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1160" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1160" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1160" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1160" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1160" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1160" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1160" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1160" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1160" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1160" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1161" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1161" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1161" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1161" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1161" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1161" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1161" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1161" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1161" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1161" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1161" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1161" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1162" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1162" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1162" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1162" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="D1162" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1162" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1162" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1162" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1162" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1162" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="J1162" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1162" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1163" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1163" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1163" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1163" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1163" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="E1163" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="F1163" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1163" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1163" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1163" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1163" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1163" s="7" t="s">
+        <v>567</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1149"/>
+  <autoFilter ref="A1:K1163"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-15T19:27:53.606Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12793" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12947" uniqueCount="578">
   <si>
     <t>Date</t>
   </si>
@@ -1724,6 +1724,30 @@
   </si>
   <si>
     <t>Spoke with Topher regarding 30% level</t>
+  </si>
+  <si>
+    <t>2026-10-16</t>
+  </si>
+  <si>
+    <t>LS DH</t>
+  </si>
+  <si>
+    <t>S-mv9usenx-3k6mk</t>
+  </si>
+  <si>
+    <t>21:51</t>
+  </si>
+  <si>
+    <t>DH</t>
+  </si>
+  <si>
+    <t>01:29</t>
+  </si>
+  <si>
+    <t>Early - with drum change</t>
+  </si>
+  <si>
+    <t>25%</t>
   </si>
 </sst>
 </file>
@@ -2299,7 +2323,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1163"/>
+  <dimension ref="A1:K1177"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -43017,8 +43041,498 @@
         <v>567</v>
       </c>
     </row>
+    <row r="1164" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1164" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1164" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1164" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1164" s="11" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1164" s="11" t="s">
+        <v>510</v>
+      </c>
+      <c r="F1164" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1164" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1164" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1164" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1164" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1164" s="14" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1165" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1165" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1165" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1165" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1165" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1165" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="F1165" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1165" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1165" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1165" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1165" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1165" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1166" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1166" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1166" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1166" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1166" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1166" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="F1166" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1166" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1166" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1166" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1166" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1166" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1167" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1167" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1167" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1167" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1167" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1167" s="17" t="s">
+        <v>510</v>
+      </c>
+      <c r="F1167" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1167" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1167" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1167" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1167" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1167" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1168" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1168" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1168" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1168" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1168" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1168" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="F1168" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1168" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1168" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1168" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1168" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1168" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1169" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1169" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1169" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1169" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1169" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1169" s="17" t="s">
+        <v>510</v>
+      </c>
+      <c r="F1169" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1169" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1169" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1169" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1169" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1169" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1170" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1170" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1170" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1170" s="15" t="s">
+        <v>573</v>
+      </c>
+      <c r="D1170" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1170" s="17" t="s">
+        <v>574</v>
+      </c>
+      <c r="F1170" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1170" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1170" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1170" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1170" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1170" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1171" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1171" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1171" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1171" s="15" t="s">
+        <v>575</v>
+      </c>
+      <c r="D1171" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1171" s="17" t="s">
+        <v>510</v>
+      </c>
+      <c r="F1171" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1171" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1171" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1171" s="17" t="s">
+        <v>576</v>
+      </c>
+      <c r="J1171" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1171" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1172" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1172" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1172" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1172" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1172" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1172" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="F1172" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1172" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1172" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1172" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1172" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1172" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1173" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1173" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1173" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1173" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1173" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1173" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="F1173" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1173" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1173" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1173" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1173" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1173" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1174" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1174" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1174" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1174" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1174" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1174" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="F1174" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1174" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1174" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1174" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1174" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1174" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1175" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1175" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1175" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1175" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1175" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1175" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="F1175" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1175" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1175" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1175" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1175" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1175" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1176" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1176" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1176" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1176" s="15" t="s">
+        <v>301</v>
+      </c>
+      <c r="D1176" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1176" s="17" t="s">
+        <v>574</v>
+      </c>
+      <c r="F1176" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1176" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1176" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1176" s="17" t="s">
+        <v>577</v>
+      </c>
+      <c r="J1176" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1176" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="1177" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1177" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1177" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1177" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1177" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="E1177" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="F1177" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1177" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1177" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1177" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1177" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1177" s="19" t="s">
+        <v>572</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1163"/>
+  <autoFilter ref="A1:K1177"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-16T01:22:18.890Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12947" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13101" uniqueCount="583">
   <si>
     <t>Date</t>
   </si>
@@ -1748,6 +1748,21 @@
   </si>
   <si>
     <t>25%</t>
+  </si>
+  <si>
+    <t>S-mv9us8vs-9klye</t>
+  </si>
+  <si>
+    <t>06:44</t>
+  </si>
+  <si>
+    <t>Tony</t>
+  </si>
+  <si>
+    <t>Checked at 6:40am Steam vent not cleaned by previous shift</t>
+  </si>
+  <si>
+    <t>Not emptied by previous shift</t>
   </si>
 </sst>
 </file>
@@ -2323,7 +2338,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K1177"/>
+  <dimension ref="A1:K1191"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -43531,8 +43546,498 @@
         <v>572</v>
       </c>
     </row>
+    <row r="1178" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1178" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1178" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1178" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="D1178" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1178" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1178" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1178" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1178" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1178" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1178" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1178" s="24" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1179" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1179" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1179" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1179" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1179" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1179" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1179" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1179" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1179" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1179" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1179" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1179" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1180" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1180" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1180" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1180" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1180" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1180" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1180" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1180" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1180" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1180" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1180" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1180" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1181" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1181" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1181" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1181" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1181" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1181" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1181" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1181" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1181" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1181" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1181" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1181" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1182" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1182" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1182" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1182" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1182" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1182" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1182" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1182" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1182" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1182" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1182" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1182" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1183" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1183" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1183" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1183" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D1183" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1183" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1183" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1183" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1183" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1183" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1183" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1183" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1184" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1184" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1184" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1184" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D1184" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1184" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1184" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1184" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1184" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1184" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1184" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1184" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1185" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1185" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1185" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1185" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1185" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1185" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1185" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1185" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1185" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1185" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1185" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1185" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1186" ht="34" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1186" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1186" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1186" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="D1186" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1186" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="F1186" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1186" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1186" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1186" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="J1186" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1186" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1187" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1187" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1187" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1187" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1187" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1187" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1187" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1187" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1187" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1187" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="J1187" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1187" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1188" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1188" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1188" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1188" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1188" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1188" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1188" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1188" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1188" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1188" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1188" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1188" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1189" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1189" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1189" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1189" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1189" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1189" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1189" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1189" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1189" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1189" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1189" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1189" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1190" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1190" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1190" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1190" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1190" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1190" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1190" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1190" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1190" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1190" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1190" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1190" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="1191" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1191" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1191" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1191" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1191" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1191" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1191" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1191" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1191" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1191" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1191" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1191" s="7" t="s">
+        <v>578</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1177"/>
+  <autoFilter ref="A1:K1191"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-16T01:24:03.374Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13101" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13101" uniqueCount="582">
   <si>
     <t>Date</t>
   </si>
@@ -1754,9 +1754,6 @@
   </si>
   <si>
     <t>06:44</t>
-  </si>
-  <si>
-    <t>Tony</t>
   </si>
   <si>
     <t>Checked at 6:40am Steam vent not cleaned by previous shift</t>
@@ -43560,7 +43557,7 @@
         <v>256</v>
       </c>
       <c r="E1178" s="22" t="s">
-        <v>256</v>
+        <v>157</v>
       </c>
       <c r="F1178" s="23" t="s">
         <v>16</v>
@@ -43735,7 +43732,7 @@
         <v>256</v>
       </c>
       <c r="E1183" s="4" t="s">
-        <v>256</v>
+        <v>157</v>
       </c>
       <c r="F1183" s="5" t="s">
         <v>28</v>
@@ -43770,7 +43767,7 @@
         <v>256</v>
       </c>
       <c r="E1184" s="4" t="s">
-        <v>256</v>
+        <v>157</v>
       </c>
       <c r="F1184" s="5" t="s">
         <v>28</v>
@@ -43840,7 +43837,7 @@
         <v>256</v>
       </c>
       <c r="E1186" s="4" t="s">
-        <v>580</v>
+        <v>157</v>
       </c>
       <c r="F1186" s="5" t="s">
         <v>28</v>
@@ -43852,7 +43849,7 @@
         <v>18</v>
       </c>
       <c r="I1186" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="J1186" s="4" t="s">
         <v>19</v>
@@ -43887,7 +43884,7 @@
         <v>23</v>
       </c>
       <c r="I1187" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="J1187" s="4" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-16T01:41:18.952Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13101" uniqueCount="582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13101" uniqueCount="583">
   <si>
     <t>Date</t>
   </si>
@@ -1751,6 +1751,9 @@
   </si>
   <si>
     <t>S-mv9us8vs-9klye</t>
+  </si>
+  <si>
+    <t>11:41</t>
   </si>
   <si>
     <t>06:44</t>
@@ -43656,7 +43659,7 @@
         <v>12</v>
       </c>
       <c r="C1181" s="2" t="s">
-        <v>21</v>
+        <v>579</v>
       </c>
       <c r="D1181" s="4" t="s">
         <v>256</v>
@@ -43670,8 +43673,8 @@
       <c r="G1181" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H1181" s="8" t="s">
-        <v>23</v>
+      <c r="H1181" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I1181" s="4" t="s">
         <v>19</v>
@@ -43796,7 +43799,7 @@
         <v>12</v>
       </c>
       <c r="C1185" s="2" t="s">
-        <v>21</v>
+        <v>579</v>
       </c>
       <c r="D1185" s="4" t="s">
         <v>256</v>
@@ -43810,8 +43813,8 @@
       <c r="G1185" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="H1185" s="8" t="s">
-        <v>23</v>
+      <c r="H1185" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I1185" s="4" t="s">
         <v>19</v>
@@ -43831,7 +43834,7 @@
         <v>12</v>
       </c>
       <c r="C1186" s="2" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="D1186" s="4" t="s">
         <v>256</v>
@@ -43849,7 +43852,7 @@
         <v>18</v>
       </c>
       <c r="I1186" s="4" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="J1186" s="4" t="s">
         <v>19</v>
@@ -43866,7 +43869,7 @@
         <v>12</v>
       </c>
       <c r="C1187" s="2" t="s">
-        <v>21</v>
+        <v>579</v>
       </c>
       <c r="D1187" s="4" t="s">
         <v>256</v>
@@ -43880,11 +43883,11 @@
       <c r="G1187" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H1187" s="8" t="s">
-        <v>23</v>
+      <c r="H1187" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="I1187" s="4" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="J1187" s="4" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-16T19:32:02.100Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14292" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14460" uniqueCount="588">
   <si>
     <t>Date</t>
   </si>
@@ -1766,6 +1766,18 @@
   </si>
   <si>
     <t>Not emptied by previous shift</t>
+  </si>
+  <si>
+    <t>2026-10-17</t>
+  </si>
+  <si>
+    <t>S-mv9xlbfs-73jzo</t>
+  </si>
+  <si>
+    <t>02:54</t>
+  </si>
+  <si>
+    <t>04:23</t>
   </si>
 </sst>
 </file>
@@ -2341,7 +2353,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1191"/>
+  <dimension ref="A1:L1205"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -47613,8 +47625,540 @@
         <v>571</v>
       </c>
     </row>
+    <row r="1192" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1192" s="9" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1192" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1192" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="D1192" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1192" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1192" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1192" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1192" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1192" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1192" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1192" s="14" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1192" s="9" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1193" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1193" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1193" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1193" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1193" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1193" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1193" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1193" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1193" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1193" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1193" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1193" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1193" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1194" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1194" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1194" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1194" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1194" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1194" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1194" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1194" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1194" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1194" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1194" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1194" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1194" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1195" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1195" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1195" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1195" s="15" t="s">
+        <v>312</v>
+      </c>
+      <c r="D1195" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1195" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1195" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1195" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1195" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1195" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1195" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1195" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1195" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1196" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1196" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1196" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1196" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1196" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1196" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1196" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1196" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1196" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1196" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1196" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1196" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1196" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1197" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1197" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1197" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1197" s="15" t="s">
+        <v>543</v>
+      </c>
+      <c r="D1197" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1197" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1197" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1197" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1197" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1197" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1197" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1197" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1197" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1198" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1198" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1198" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1198" s="15" t="s">
+        <v>478</v>
+      </c>
+      <c r="D1198" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1198" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1198" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1198" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1198" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1198" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1198" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1198" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1198" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1199" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1199" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1199" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1199" s="15" t="s">
+        <v>586</v>
+      </c>
+      <c r="D1199" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1199" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1199" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1199" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1199" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1199" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1199" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1199" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1199" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1200" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1200" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1200" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1200" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1200" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1200" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1200" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1200" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1200" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1200" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1200" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1200" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1200" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1201" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1201" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1201" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1201" s="15" t="s">
+        <v>587</v>
+      </c>
+      <c r="D1201" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1201" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1201" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1201" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1201" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1201" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1201" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1201" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1201" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1202" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1202" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1202" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1202" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1202" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1202" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1202" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1202" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1202" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1202" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1202" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1202" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1202" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1203" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1203" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1203" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1203" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1203" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1203" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1203" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1203" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1203" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1203" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1203" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1203" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1203" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1204" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1204" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1204" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1204" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1204" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1204" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1204" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1204" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1204" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1204" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1204" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1204" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1204" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="1205" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1205" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1205" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1205" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1205" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1205" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="F1205" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1205" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1205" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1205" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1205" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1205" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="L1205" s="15" t="s">
+        <v>571</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1191"/>
+  <autoFilter ref="A1:L1205"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-16T20:07:26.538Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14460" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14628" uniqueCount="589">
   <si>
     <t>Date</t>
   </si>
@@ -1778,6 +1778,9 @@
   </si>
   <si>
     <t>04:23</t>
+  </si>
+  <si>
+    <t>S-mvbdwpyn-pd567</t>
   </si>
 </sst>
 </file>
@@ -2353,7 +2356,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1205"/>
+  <dimension ref="A1:L1219"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -48157,8 +48160,540 @@
         <v>571</v>
       </c>
     </row>
+    <row r="1206" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1206" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1206" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1206" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="D1206" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1206" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1206" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1206" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1206" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1206" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1206" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1206" s="24" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1206" s="20" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1207" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1207" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1207" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1207" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1207" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1207" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1207" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1207" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1207" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1207" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1207" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1207" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1207" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1208" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1208" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1208" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1208" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1208" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1208" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1208" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1208" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1208" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1208" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1208" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1208" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1208" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1209" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1209" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1209" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1209" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D1209" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1209" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1209" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1209" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1209" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1209" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1209" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1209" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1209" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1210" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1210" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1210" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1210" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1210" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1210" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1210" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1210" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1210" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1210" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1210" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1210" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1210" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1211" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1211" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1211" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1211" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1211" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1211" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1211" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1211" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1211" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1211" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1211" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1211" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1211" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1212" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1212" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1212" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1212" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1212" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1212" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1212" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1212" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1212" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1212" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1212" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1212" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1212" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1213" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1213" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1213" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1213" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1213" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1213" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1213" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1213" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1213" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1213" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1213" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1213" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1213" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1214" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1214" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1214" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1214" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1214" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1214" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1214" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1214" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1214" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1214" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1214" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1214" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1214" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1215" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1215" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1215" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1215" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1215" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1215" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1215" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1215" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1215" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1215" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1215" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1215" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1215" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1216" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1216" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1216" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1216" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1216" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1216" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1216" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1216" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1216" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1216" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1216" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1216" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1216" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1217" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1217" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1217" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1217" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1217" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1217" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1217" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1217" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1217" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1217" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1217" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1217" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1217" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1218" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1218" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1218" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1218" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1218" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1218" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1218" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1218" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1218" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1218" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1218" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1218" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1218" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1219" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1219" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="B1219" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1219" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1219" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1219" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1219" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1219" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1219" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1219" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1219" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1219" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="L1219" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1205"/>
+  <autoFilter ref="A1:L1219"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-17T07:13:07.434Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14628" uniqueCount="589">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14628" uniqueCount="592">
   <si>
     <t>Date</t>
   </si>
@@ -1781,6 +1781,15 @@
   </si>
   <si>
     <t>S-mvbdwpyn-pd567</t>
+  </si>
+  <si>
+    <t>06:08</t>
+  </si>
+  <si>
+    <t>09:32</t>
+  </si>
+  <si>
+    <t>Not done on previous shift again.</t>
   </si>
 </sst>
 </file>
@@ -48358,7 +48367,7 @@
         <v>13</v>
       </c>
       <c r="C1211" s="2" t="s">
-        <v>22</v>
+        <v>589</v>
       </c>
       <c r="D1211" s="4" t="s">
         <v>236</v>
@@ -48372,8 +48381,8 @@
       <c r="G1211" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H1211" s="8" t="s">
-        <v>24</v>
+      <c r="H1211" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1211" s="4" t="s">
         <v>20</v>
@@ -48396,7 +48405,7 @@
         <v>13</v>
       </c>
       <c r="C1212" s="2" t="s">
-        <v>22</v>
+        <v>590</v>
       </c>
       <c r="D1212" s="4" t="s">
         <v>236</v>
@@ -48410,8 +48419,8 @@
       <c r="G1212" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H1212" s="8" t="s">
-        <v>24</v>
+      <c r="H1212" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1212" s="4" t="s">
         <v>20</v>
@@ -48434,7 +48443,7 @@
         <v>13</v>
       </c>
       <c r="C1213" s="2" t="s">
-        <v>22</v>
+        <v>384</v>
       </c>
       <c r="D1213" s="4" t="s">
         <v>236</v>
@@ -48448,8 +48457,8 @@
       <c r="G1213" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H1213" s="8" t="s">
-        <v>24</v>
+      <c r="H1213" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1213" s="4" t="s">
         <v>20</v>
@@ -48472,7 +48481,7 @@
         <v>13</v>
       </c>
       <c r="C1214" s="2" t="s">
-        <v>22</v>
+        <v>562</v>
       </c>
       <c r="D1214" s="4" t="s">
         <v>236</v>
@@ -48486,11 +48495,11 @@
       <c r="G1214" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H1214" s="8" t="s">
-        <v>24</v>
+      <c r="H1214" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1214" s="4" t="s">
-        <v>20</v>
+        <v>591</v>
       </c>
       <c r="J1214" s="4" t="s">
         <v>20</v>
@@ -48510,7 +48519,7 @@
         <v>13</v>
       </c>
       <c r="C1215" s="2" t="s">
-        <v>22</v>
+        <v>562</v>
       </c>
       <c r="D1215" s="4" t="s">
         <v>236</v>
@@ -48524,8 +48533,8 @@
       <c r="G1215" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H1215" s="8" t="s">
-        <v>24</v>
+      <c r="H1215" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1215" s="4" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-17T19:35:36.946Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14628" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14796" uniqueCount="596">
   <si>
     <t>Date</t>
   </si>
@@ -1790,6 +1790,18 @@
   </si>
   <si>
     <t>Not done on previous shift again.</t>
+  </si>
+  <si>
+    <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>S-mvbecv3e-sbtlj</t>
+  </si>
+  <si>
+    <t>03:58</t>
+  </si>
+  <si>
+    <t>Had issues arise, missed initial 3am slot</t>
   </si>
 </sst>
 </file>
@@ -2365,7 +2377,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1219"/>
+  <dimension ref="A1:L1233"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -48701,8 +48713,540 @@
         <v>584</v>
       </c>
     </row>
+    <row r="1220" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1220" s="9" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1220" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1220" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="D1220" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1220" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1220" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1220" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1220" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1220" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1220" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1220" s="14" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1220" s="9" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1221" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1221" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1221" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1221" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1221" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1221" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1221" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1221" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1221" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1221" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1221" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1221" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1221" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1222" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1222" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1222" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1222" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1222" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1222" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1222" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1222" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1222" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1222" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1222" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1222" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1222" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1223" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1223" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1223" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1223" s="15" t="s">
+        <v>351</v>
+      </c>
+      <c r="D1223" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1223" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1223" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1223" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1223" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1223" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1223" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1223" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1223" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1224" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1224" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1224" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1224" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1224" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1224" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1224" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1224" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1224" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1224" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1224" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1224" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1224" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1225" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1225" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1225" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1225" s="15" t="s">
+        <v>351</v>
+      </c>
+      <c r="D1225" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1225" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1225" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1225" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1225" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1225" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1225" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1225" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1225" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1226" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1226" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1226" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1226" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="D1226" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1226" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1226" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1226" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1226" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1226" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1226" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1226" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1226" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1227" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1227" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1227" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1227" s="15" t="s">
+        <v>594</v>
+      </c>
+      <c r="D1227" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1227" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1227" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1227" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1227" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1227" s="17" t="s">
+        <v>595</v>
+      </c>
+      <c r="J1227" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1227" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1227" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1228" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1228" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1228" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1228" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="D1228" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1228" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1228" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1228" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1228" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1228" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1228" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1228" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1228" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1229" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1229" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1229" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1229" s="15" t="s">
+        <v>481</v>
+      </c>
+      <c r="D1229" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1229" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1229" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1229" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1229" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1229" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1229" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1229" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1229" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1230" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1230" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1230" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1230" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1230" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1230" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1230" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1230" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1230" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1230" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1230" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1230" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1230" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1231" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1231" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1231" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1231" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1231" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1231" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1231" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1231" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1231" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1231" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1231" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1231" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1231" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1232" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1232" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1232" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1232" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1232" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1232" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1232" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1232" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1232" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1232" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1232" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1232" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1232" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="1233" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1233" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="B1233" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1233" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1233" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1233" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1233" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1233" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1233" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1233" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1233" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1233" s="19" t="s">
+        <v>593</v>
+      </c>
+      <c r="L1233" s="15" t="s">
+        <v>584</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1219"/>
+  <autoFilter ref="A1:L1233"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-19T00:12:29.256Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14796" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14964" uniqueCount="606">
   <si>
     <t>Date</t>
   </si>
@@ -1802,6 +1802,36 @@
   </si>
   <si>
     <t>Had issues arise, missed initial 3am slot</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>18:12</t>
+  </si>
+  <si>
+    <t>S-mvef71ll-1m8uy</t>
+  </si>
+  <si>
+    <t>18:13</t>
+  </si>
+  <si>
+    <t>21:27</t>
+  </si>
+  <si>
+    <t>03:12</t>
+  </si>
+  <si>
+    <t>05:08</t>
+  </si>
+  <si>
+    <t>05:07</t>
+  </si>
+  <si>
+    <t>20:18</t>
+  </si>
+  <si>
+    <t>20:47</t>
   </si>
 </sst>
 </file>
@@ -2377,7 +2407,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1233"/>
+  <dimension ref="A1:L1247"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -49245,8 +49275,540 @@
         <v>584</v>
       </c>
     </row>
+    <row r="1234" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1234" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1234" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1234" s="20" t="s">
+        <v>597</v>
+      </c>
+      <c r="D1234" s="22" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1234" s="22" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1234" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1234" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1234" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1234" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1234" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1234" s="24" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1234" s="20" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1235" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1235" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1235" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1235" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1235" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1235" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1235" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1235" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1235" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1235" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1235" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1235" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1235" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1236" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1236" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1236" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1236" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1236" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1236" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1236" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1236" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1236" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1236" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1236" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1236" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1236" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1237" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1237" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1237" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1237" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="D1237" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1237" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1237" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1237" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1237" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1237" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1237" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1237" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1237" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1238" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1238" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1238" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1238" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1238" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1238" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1238" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1238" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1238" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1238" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1238" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1238" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1238" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1239" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1239" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1239" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1239" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="D1239" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1239" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1239" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1239" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1239" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1239" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1239" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1239" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1239" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1240" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1240" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1240" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1240" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="D1240" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1240" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1240" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1240" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1240" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1240" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1240" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1240" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1240" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1241" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1241" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1241" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1241" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="D1241" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1241" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1241" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1241" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1241" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1241" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1241" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1241" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1241" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1242" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1242" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1242" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1242" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="D1242" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1242" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1242" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1242" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1242" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1242" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1242" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1242" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1242" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1243" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1243" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1243" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1243" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="D1243" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1243" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1243" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1243" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1243" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1243" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1243" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1243" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1243" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1244" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1244" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1244" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1244" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1244" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1244" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1244" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1244" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1244" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1244" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1244" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1244" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1244" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1245" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1245" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1245" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1245" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="D1245" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1245" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1245" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1245" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1245" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1245" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1245" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1245" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1245" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1246" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1246" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1246" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1246" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="D1246" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1246" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1246" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1246" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1246" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1246" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="J1246" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1246" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1246" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1247" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1247" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1247" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1247" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1247" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="E1247" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="F1247" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1247" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1247" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1247" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1247" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1247" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="L1247" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1233"/>
+  <autoFilter ref="A1:L1247"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-19T07:05:54.622Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14964" uniqueCount="606">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15132" uniqueCount="611">
   <si>
     <t>Date</t>
   </si>
@@ -1832,6 +1832,21 @@
   </si>
   <si>
     <t>20:47</t>
+  </si>
+  <si>
+    <t>09:01</t>
+  </si>
+  <si>
+    <t>Tony</t>
+  </si>
+  <si>
+    <t>S-mvec97pn-lxwij</t>
+  </si>
+  <si>
+    <t>16:58</t>
+  </si>
+  <si>
+    <t>17:05</t>
   </si>
 </sst>
 </file>
@@ -2407,7 +2422,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1247"/>
+  <dimension ref="A1:L1261"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -49807,8 +49822,540 @@
         <v>596</v>
       </c>
     </row>
+    <row r="1248" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1248" s="9" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1248" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1248" s="9" t="s">
+        <v>606</v>
+      </c>
+      <c r="D1248" s="11" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1248" s="11" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1248" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1248" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1248" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1248" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1248" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1248" s="14" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1248" s="9" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1249" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1249" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1249" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1249" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1249" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1249" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1249" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1249" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1249" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1249" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1249" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1249" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1249" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1250" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1250" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1250" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1250" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1250" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1250" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1250" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1250" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1250" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1250" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1250" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1250" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1250" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1251" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1251" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1251" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1251" s="15" t="s">
+        <v>467</v>
+      </c>
+      <c r="D1251" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1251" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1251" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1251" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1251" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1251" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1251" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1251" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1251" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1252" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1252" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1252" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1252" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1252" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1252" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1252" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1252" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1252" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1252" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1252" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1252" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1252" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1253" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1253" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1253" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1253" s="15" t="s">
+        <v>606</v>
+      </c>
+      <c r="D1253" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1253" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1253" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1253" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1253" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1253" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1253" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1253" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1253" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1254" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1254" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1254" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1254" s="15" t="s">
+        <v>606</v>
+      </c>
+      <c r="D1254" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1254" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1254" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1254" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1254" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1254" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1254" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1254" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1254" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1255" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1255" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1255" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1255" s="15" t="s">
+        <v>609</v>
+      </c>
+      <c r="D1255" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1255" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1255" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1255" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1255" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1255" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1255" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1255" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1255" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1256" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1256" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1256" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1256" s="15" t="s">
+        <v>610</v>
+      </c>
+      <c r="D1256" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1256" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1256" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1256" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1256" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1256" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1256" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1256" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1256" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1257" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1257" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1257" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1257" s="15" t="s">
+        <v>610</v>
+      </c>
+      <c r="D1257" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1257" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1257" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1257" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1257" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1257" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1257" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1257" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1257" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1258" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1258" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1258" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1258" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1258" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1258" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1258" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1258" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1258" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1258" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1258" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1258" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1258" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1259" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1259" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1259" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1259" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1259" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1259" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1259" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1259" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1259" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1259" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1259" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1259" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1259" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1260" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1260" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1260" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1260" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1260" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1260" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1260" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1260" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1260" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1260" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1260" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1260" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1260" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1261" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1261" s="15" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1261" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1261" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1261" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1261" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1261" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1261" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1261" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1261" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1261" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1261" s="19" t="s">
+        <v>608</v>
+      </c>
+      <c r="L1261" s="15" t="s">
+        <v>596</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1247"/>
+  <autoFilter ref="A1:L1261"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-19T11:11:08.954Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15132" uniqueCount="611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15300" uniqueCount="615">
   <si>
     <t>Date</t>
   </si>
@@ -1847,6 +1847,18 @@
   </si>
   <si>
     <t>17:05</t>
+  </si>
+  <si>
+    <t>Ben/Luke</t>
+  </si>
+  <si>
+    <t>S-mvei2sr7-sclo4</t>
+  </si>
+  <si>
+    <t>18:41</t>
+  </si>
+  <si>
+    <t>21:10</t>
   </si>
 </sst>
 </file>
@@ -2422,7 +2434,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1261"/>
+  <dimension ref="A1:L1275"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -50354,8 +50366,540 @@
         <v>596</v>
       </c>
     </row>
+    <row r="1262" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1262" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1262" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1262" s="20" t="s">
+        <v>325</v>
+      </c>
+      <c r="D1262" s="22" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1262" s="22" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1262" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1262" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1262" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1262" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1262" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1262" s="24" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1262" s="20" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1263" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1263" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1263" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1263" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1263" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1263" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1263" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1263" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1263" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1263" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1263" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1263" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1263" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1264" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1264" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1264" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1264" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1264" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1264" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1264" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1264" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1264" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1264" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1264" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1264" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1264" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1265" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1265" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1265" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1265" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="D1265" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1265" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1265" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1265" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1265" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1265" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1265" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1265" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1265" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1266" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1266" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1266" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1266" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1266" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1266" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1266" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1266" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1266" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1266" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1266" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1266" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1266" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1267" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1267" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1267" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1267" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="D1267" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1267" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1267" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1267" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1267" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1267" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1267" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1267" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1267" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1268" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1268" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1268" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1268" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="D1268" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1268" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1268" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1268" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1268" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1268" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1268" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1268" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1268" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1269" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1269" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1269" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1269" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1269" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1269" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1269" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1269" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1269" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1269" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1269" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1269" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1269" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1270" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1270" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1270" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1270" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1270" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1270" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1270" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1270" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1270" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1270" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1270" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1270" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1270" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1271" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1271" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1271" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1271" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1271" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1271" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1271" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1271" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1271" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1271" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1271" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1271" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1271" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1272" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1272" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1272" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1272" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1272" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1272" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1272" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1272" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1272" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1272" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1272" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1272" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1272" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1273" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1273" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1273" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1273" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1273" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1273" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1273" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1273" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1273" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1273" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1273" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1273" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1273" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1274" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1274" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1274" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1274" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1274" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1274" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1274" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1274" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1274" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1274" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1274" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1274" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1274" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="1275" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1275" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1275" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1275" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1275" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="E1275" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="F1275" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1275" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1275" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1275" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1275" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1275" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="L1275" s="2" t="s">
+        <v>596</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1261"/>
+  <autoFilter ref="A1:L1275"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-19T18:48:18.781Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15300" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15300" uniqueCount="618">
   <si>
     <t>Date</t>
   </si>
@@ -1849,6 +1849,9 @@
     <t>17:05</t>
   </si>
   <si>
+    <t>2026-10-20</t>
+  </si>
+  <si>
     <t>Ben/Luke</t>
   </si>
   <si>
@@ -1859,6 +1862,12 @@
   </si>
   <si>
     <t>21:10</t>
+  </si>
+  <si>
+    <t>03:02</t>
+  </si>
+  <si>
+    <t>04:48</t>
   </si>
 </sst>
 </file>
@@ -50368,7 +50377,7 @@
     </row>
     <row r="1262" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1262" s="20" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1262" s="10" t="s">
         <v>42</v>
@@ -50377,10 +50386,10 @@
         <v>325</v>
       </c>
       <c r="D1262" s="22" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1262" s="22" t="s">
-        <v>611</v>
+        <v>511</v>
       </c>
       <c r="F1262" s="23" t="s">
         <v>17</v>
@@ -50398,7 +50407,7 @@
         <v>20</v>
       </c>
       <c r="K1262" s="24" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1262" s="20" t="s">
         <v>596</v>
@@ -50406,7 +50415,7 @@
     </row>
     <row r="1263" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1263" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1263" s="16" t="s">
         <v>42</v>
@@ -50415,10 +50424,10 @@
         <v>22</v>
       </c>
       <c r="D1263" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1263" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F1263" s="5" t="s">
         <v>17</v>
@@ -50436,7 +50445,7 @@
         <v>20</v>
       </c>
       <c r="K1263" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1263" s="2" t="s">
         <v>596</v>
@@ -50444,7 +50453,7 @@
     </row>
     <row r="1264" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1264" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1264" s="16" t="s">
         <v>42</v>
@@ -50453,10 +50462,10 @@
         <v>22</v>
       </c>
       <c r="D1264" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1264" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F1264" s="5" t="s">
         <v>17</v>
@@ -50474,7 +50483,7 @@
         <v>20</v>
       </c>
       <c r="K1264" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1264" s="2" t="s">
         <v>596</v>
@@ -50482,7 +50491,7 @@
     </row>
     <row r="1265" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1265" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1265" s="16" t="s">
         <v>42</v>
@@ -50491,10 +50500,10 @@
         <v>405</v>
       </c>
       <c r="D1265" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1265" s="4" t="s">
-        <v>611</v>
+        <v>511</v>
       </c>
       <c r="F1265" s="5" t="s">
         <v>17</v>
@@ -50512,7 +50521,7 @@
         <v>20</v>
       </c>
       <c r="K1265" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1265" s="2" t="s">
         <v>596</v>
@@ -50520,7 +50529,7 @@
     </row>
     <row r="1266" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1266" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1266" s="16" t="s">
         <v>42</v>
@@ -50529,10 +50538,10 @@
         <v>22</v>
       </c>
       <c r="D1266" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1266" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F1266" s="5" t="s">
         <v>17</v>
@@ -50550,7 +50559,7 @@
         <v>20</v>
       </c>
       <c r="K1266" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1266" s="2" t="s">
         <v>596</v>
@@ -50558,19 +50567,19 @@
     </row>
     <row r="1267" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1267" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1267" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1267" s="2" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="D1267" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1267" s="4" t="s">
-        <v>611</v>
+        <v>511</v>
       </c>
       <c r="F1267" s="5" t="s">
         <v>29</v>
@@ -50588,7 +50597,7 @@
         <v>20</v>
       </c>
       <c r="K1267" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1267" s="2" t="s">
         <v>596</v>
@@ -50596,16 +50605,16 @@
     </row>
     <row r="1268" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1268" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1268" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1268" s="2" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D1268" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1268" s="4" t="s">
         <v>16</v>
@@ -50626,7 +50635,7 @@
         <v>20</v>
       </c>
       <c r="K1268" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1268" s="2" t="s">
         <v>596</v>
@@ -50634,19 +50643,19 @@
     </row>
     <row r="1269" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1269" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1269" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1269" s="2" t="s">
-        <v>22</v>
+        <v>616</v>
       </c>
       <c r="D1269" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1269" s="4" t="s">
-        <v>611</v>
+        <v>511</v>
       </c>
       <c r="F1269" s="5" t="s">
         <v>29</v>
@@ -50654,8 +50663,8 @@
       <c r="G1269" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H1269" s="8" t="s">
-        <v>24</v>
+      <c r="H1269" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1269" s="4" t="s">
         <v>20</v>
@@ -50664,7 +50673,7 @@
         <v>20</v>
       </c>
       <c r="K1269" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1269" s="2" t="s">
         <v>596</v>
@@ -50672,19 +50681,19 @@
     </row>
     <row r="1270" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1270" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1270" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1270" s="2" t="s">
-        <v>22</v>
+        <v>617</v>
       </c>
       <c r="D1270" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1270" s="4" t="s">
-        <v>611</v>
+        <v>511</v>
       </c>
       <c r="F1270" s="5" t="s">
         <v>29</v>
@@ -50692,8 +50701,8 @@
       <c r="G1270" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H1270" s="8" t="s">
-        <v>24</v>
+      <c r="H1270" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1270" s="4" t="s">
         <v>20</v>
@@ -50702,7 +50711,7 @@
         <v>20</v>
       </c>
       <c r="K1270" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1270" s="2" t="s">
         <v>596</v>
@@ -50710,19 +50719,19 @@
     </row>
     <row r="1271" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1271" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1271" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1271" s="2" t="s">
-        <v>22</v>
+        <v>165</v>
       </c>
       <c r="D1271" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1271" s="4" t="s">
-        <v>611</v>
+        <v>511</v>
       </c>
       <c r="F1271" s="5" t="s">
         <v>29</v>
@@ -50730,8 +50739,8 @@
       <c r="G1271" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H1271" s="8" t="s">
-        <v>24</v>
+      <c r="H1271" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1271" s="4" t="s">
         <v>20</v>
@@ -50740,7 +50749,7 @@
         <v>20</v>
       </c>
       <c r="K1271" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1271" s="2" t="s">
         <v>596</v>
@@ -50748,7 +50757,7 @@
     </row>
     <row r="1272" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1272" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1272" s="16" t="s">
         <v>42</v>
@@ -50757,10 +50766,10 @@
         <v>22</v>
       </c>
       <c r="D1272" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1272" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F1272" s="5" t="s">
         <v>36</v>
@@ -50778,7 +50787,7 @@
         <v>20</v>
       </c>
       <c r="K1272" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1272" s="2" t="s">
         <v>596</v>
@@ -50786,7 +50795,7 @@
     </row>
     <row r="1273" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1273" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1273" s="16" t="s">
         <v>42</v>
@@ -50795,10 +50804,10 @@
         <v>22</v>
       </c>
       <c r="D1273" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1273" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F1273" s="5" t="s">
         <v>36</v>
@@ -50816,7 +50825,7 @@
         <v>20</v>
       </c>
       <c r="K1273" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1273" s="2" t="s">
         <v>596</v>
@@ -50824,7 +50833,7 @@
     </row>
     <row r="1274" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1274" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1274" s="16" t="s">
         <v>42</v>
@@ -50833,10 +50842,10 @@
         <v>22</v>
       </c>
       <c r="D1274" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1274" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F1274" s="5" t="s">
         <v>36</v>
@@ -50854,7 +50863,7 @@
         <v>20</v>
       </c>
       <c r="K1274" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1274" s="2" t="s">
         <v>596</v>
@@ -50862,7 +50871,7 @@
     </row>
     <row r="1275" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1275" s="2" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="B1275" s="16" t="s">
         <v>42</v>
@@ -50871,10 +50880,10 @@
         <v>22</v>
       </c>
       <c r="D1275" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E1275" s="4" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F1275" s="5" t="s">
         <v>36</v>
@@ -50892,7 +50901,7 @@
         <v>20</v>
       </c>
       <c r="K1275" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="L1275" s="2" t="s">
         <v>596</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-20T05:53:58.627Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15300" uniqueCount="618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15468" uniqueCount="624">
   <si>
     <t>Date</t>
   </si>
@@ -1868,6 +1868,24 @@
   </si>
   <si>
     <t>04:48</t>
+  </si>
+  <si>
+    <t>06:51</t>
+  </si>
+  <si>
+    <t>ts tr</t>
+  </si>
+  <si>
+    <t>S-mvflyhru-bni9r</t>
+  </si>
+  <si>
+    <t>07:11</t>
+  </si>
+  <si>
+    <t>15:53</t>
+  </si>
+  <si>
+    <t>tr</t>
   </si>
 </sst>
 </file>
@@ -2443,7 +2461,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1275"/>
+  <dimension ref="A1:L1289"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -50907,8 +50925,540 @@
         <v>596</v>
       </c>
     </row>
+    <row r="1276" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1276" s="9" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1276" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1276" s="9" t="s">
+        <v>618</v>
+      </c>
+      <c r="D1276" s="11" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1276" s="11" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1276" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1276" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1276" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1276" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1276" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1276" s="14" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1276" s="9" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1277" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1277" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1277" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1277" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1277" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1277" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1277" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1277" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1277" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1277" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1277" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1277" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1277" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1278" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1278" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1278" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1278" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1278" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1278" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1278" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1278" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1278" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1278" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1278" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1278" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1278" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1279" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1279" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1279" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1279" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1279" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1279" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1279" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1279" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1279" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1279" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1279" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1279" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1279" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1280" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1280" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1280" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1280" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1280" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1280" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1280" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1280" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1280" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1280" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1280" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1280" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1280" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1281" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1281" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1281" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1281" s="15" t="s">
+        <v>621</v>
+      </c>
+      <c r="D1281" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1281" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="F1281" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1281" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1281" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1281" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1281" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1281" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1281" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1282" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1282" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1282" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1282" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1282" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1282" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="F1282" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1282" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1282" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1282" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1282" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1282" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1282" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1283" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1283" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1283" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1283" s="15" t="s">
+        <v>622</v>
+      </c>
+      <c r="D1283" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1283" s="17" t="s">
+        <v>623</v>
+      </c>
+      <c r="F1283" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1283" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1283" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1283" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1283" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1283" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1283" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1284" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1284" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1284" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1284" s="15" t="s">
+        <v>622</v>
+      </c>
+      <c r="D1284" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1284" s="17" t="s">
+        <v>623</v>
+      </c>
+      <c r="F1284" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1284" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1284" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1284" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1284" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1284" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1284" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1285" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1285" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1285" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1285" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1285" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1285" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1285" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1285" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1285" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1285" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1285" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1285" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1285" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1286" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1286" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1286" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1286" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1286" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1286" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1286" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1286" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1286" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1286" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1286" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1286" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1286" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1287" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1287" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1287" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1287" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1287" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1287" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1287" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1287" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1287" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1287" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1287" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1287" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1287" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1288" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1288" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1288" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1288" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1288" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1288" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1288" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1288" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1288" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1288" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1288" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1288" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1288" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1289" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1289" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B1289" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1289" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1289" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="E1289" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="F1289" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1289" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1289" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1289" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1289" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1289" s="19" t="s">
+        <v>620</v>
+      </c>
+      <c r="L1289" s="15" t="s">
+        <v>611</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1275"/>
+  <autoFilter ref="A1:L1289"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-20T07:09:22.770Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15468" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15468" uniqueCount="626">
   <si>
     <t>Date</t>
   </si>
@@ -1879,6 +1879,9 @@
     <t>S-mvflyhru-bni9r</t>
   </si>
   <si>
+    <t>16:10</t>
+  </si>
+  <si>
     <t>07:11</t>
   </si>
   <si>
@@ -1886,6 +1889,9 @@
   </si>
   <si>
     <t>tr</t>
+  </si>
+  <si>
+    <t>17:09</t>
   </si>
 </sst>
 </file>
@@ -51047,7 +51053,7 @@
         <v>13</v>
       </c>
       <c r="C1279" s="15" t="s">
-        <v>22</v>
+        <v>621</v>
       </c>
       <c r="D1279" s="17" t="s">
         <v>619</v>
@@ -51061,8 +51067,8 @@
       <c r="G1279" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="H1279" s="8" t="s">
-        <v>24</v>
+      <c r="H1279" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1279" s="17" t="s">
         <v>20</v>
@@ -51123,7 +51129,7 @@
         <v>13</v>
       </c>
       <c r="C1281" s="15" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="D1281" s="17" t="s">
         <v>619</v>
@@ -51199,13 +51205,13 @@
         <v>13</v>
       </c>
       <c r="C1283" s="15" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D1283" s="17" t="s">
         <v>619</v>
       </c>
       <c r="E1283" s="17" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F1283" s="18" t="s">
         <v>29</v>
@@ -51237,13 +51243,13 @@
         <v>13</v>
       </c>
       <c r="C1284" s="15" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D1284" s="17" t="s">
         <v>619</v>
       </c>
       <c r="E1284" s="17" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F1284" s="18" t="s">
         <v>29</v>
@@ -51275,13 +51281,13 @@
         <v>13</v>
       </c>
       <c r="C1285" s="15" t="s">
-        <v>22</v>
+        <v>625</v>
       </c>
       <c r="D1285" s="17" t="s">
         <v>619</v>
       </c>
       <c r="E1285" s="17" t="s">
-        <v>619</v>
+        <v>288</v>
       </c>
       <c r="F1285" s="18" t="s">
         <v>29</v>
@@ -51289,8 +51295,8 @@
       <c r="G1285" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="H1285" s="8" t="s">
-        <v>24</v>
+      <c r="H1285" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1285" s="17" t="s">
         <v>20</v>
@@ -51389,13 +51395,13 @@
         <v>13</v>
       </c>
       <c r="C1288" s="15" t="s">
-        <v>22</v>
+        <v>625</v>
       </c>
       <c r="D1288" s="17" t="s">
         <v>619</v>
       </c>
       <c r="E1288" s="17" t="s">
-        <v>619</v>
+        <v>288</v>
       </c>
       <c r="F1288" s="18" t="s">
         <v>36</v>
@@ -51403,8 +51409,8 @@
       <c r="G1288" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="H1288" s="8" t="s">
-        <v>24</v>
+      <c r="H1288" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1288" s="17" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-21T03:56:04.568Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15468" uniqueCount="626">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="631">
   <si>
     <t>Date</t>
   </si>
@@ -1892,6 +1892,21 @@
   </si>
   <si>
     <t>17:09</t>
+  </si>
+  <si>
+    <t>2026-10-21</t>
+  </si>
+  <si>
+    <t>S-mvheq8oo-60m22</t>
+  </si>
+  <si>
+    <t>07:16</t>
+  </si>
+  <si>
+    <t>13:55</t>
+  </si>
+  <si>
+    <t>Water Delivered</t>
   </si>
 </sst>
 </file>
@@ -2467,7 +2482,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1289"/>
+  <dimension ref="A1:L1303"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -51463,8 +51478,540 @@
         <v>611</v>
       </c>
     </row>
+    <row r="1290" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1290" s="20" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1290" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1290" s="20" t="s">
+        <v>346</v>
+      </c>
+      <c r="D1290" s="22" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1290" s="22" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1290" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1290" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1290" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1290" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1290" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1290" s="24" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1290" s="20" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1291" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1291" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1291" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1291" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1291" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1291" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1291" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1291" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1291" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1291" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1291" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1291" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1291" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1292" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1292" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1292" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1292" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1292" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1292" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1292" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1292" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1292" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1292" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1292" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1292" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1292" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1293" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1293" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1293" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1293" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="D1293" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1293" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1293" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1293" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1293" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1293" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1293" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1293" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1293" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1294" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1294" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1294" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1294" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1294" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1294" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1294" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1294" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1294" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1294" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1294" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1294" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1294" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1295" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1295" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1295" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1295" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="D1295" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1295" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1295" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1295" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1295" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1295" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1295" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1295" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1295" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1296" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1296" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1296" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1296" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="D1296" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1296" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1296" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1296" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1296" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1296" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1296" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1296" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1296" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1297" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1297" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1297" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1297" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1297" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1297" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1297" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1297" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1297" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1297" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1297" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1297" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1297" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1298" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1298" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1298" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1298" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1298" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1298" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1298" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1298" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1298" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1298" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1298" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1298" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1298" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1299" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1299" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1299" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1299" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1299" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1299" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1299" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1299" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1299" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1299" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1299" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1299" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1299" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1300" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1300" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1300" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1300" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1300" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1300" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1300" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1300" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1300" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1300" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1300" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1300" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1300" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1301" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1301" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1301" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1301" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1301" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1301" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1301" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1301" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1301" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1301" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1301" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1301" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1301" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1302" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1302" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1302" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1302" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="D1302" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1302" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1302" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1302" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1302" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1302" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="J1302" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1302" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1302" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1303" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1303" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1303" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1303" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1303" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="E1303" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="F1303" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1303" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1303" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1303" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1303" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1303" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="L1303" s="2" t="s">
+        <v>626</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1289"/>
+  <autoFilter ref="A1:L1303"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-21T06:04:26.880Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="634">
   <si>
     <t>Date</t>
   </si>
@@ -1898,6 +1898,15 @@
   </si>
   <si>
     <t>S-mvheq8oo-60m22</t>
+  </si>
+  <si>
+    <t>na</t>
+  </si>
+  <si>
+    <t>16:03</t>
+  </si>
+  <si>
+    <t>Check and Clean The Filters in Behind Water Sprayers Nozzels</t>
   </si>
   <si>
     <t>07:16</t>
@@ -51492,7 +51501,7 @@
         <v>607</v>
       </c>
       <c r="E1290" s="22" t="s">
-        <v>607</v>
+        <v>158</v>
       </c>
       <c r="F1290" s="23" t="s">
         <v>17</v>
@@ -51542,7 +51551,7 @@
         <v>24</v>
       </c>
       <c r="I1291" s="4" t="s">
-        <v>20</v>
+        <v>628</v>
       </c>
       <c r="J1291" s="4" t="s">
         <v>20</v>
@@ -51580,7 +51589,7 @@
         <v>24</v>
       </c>
       <c r="I1292" s="4" t="s">
-        <v>20</v>
+        <v>628</v>
       </c>
       <c r="J1292" s="4" t="s">
         <v>20</v>
@@ -51606,7 +51615,7 @@
         <v>607</v>
       </c>
       <c r="E1293" s="4" t="s">
-        <v>607</v>
+        <v>158</v>
       </c>
       <c r="F1293" s="5" t="s">
         <v>17</v>
@@ -51630,7 +51639,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="1294" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1294" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1294" s="2" t="s">
         <v>626</v>
       </c>
@@ -51638,22 +51647,22 @@
         <v>13</v>
       </c>
       <c r="C1294" s="2" t="s">
-        <v>22</v>
+        <v>629</v>
       </c>
       <c r="D1294" s="4" t="s">
         <v>607</v>
       </c>
       <c r="E1294" s="4" t="s">
-        <v>607</v>
+        <v>288</v>
       </c>
       <c r="F1294" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G1294" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1294" s="8" t="s">
-        <v>24</v>
+        <v>630</v>
+      </c>
+      <c r="H1294" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1294" s="4" t="s">
         <v>20</v>
@@ -51676,7 +51685,7 @@
         <v>13</v>
       </c>
       <c r="C1295" s="2" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D1295" s="4" t="s">
         <v>607</v>
@@ -51752,13 +51761,13 @@
         <v>13</v>
       </c>
       <c r="C1297" s="2" t="s">
-        <v>22</v>
+        <v>629</v>
       </c>
       <c r="D1297" s="4" t="s">
         <v>607</v>
       </c>
       <c r="E1297" s="4" t="s">
-        <v>607</v>
+        <v>288</v>
       </c>
       <c r="F1297" s="5" t="s">
         <v>29</v>
@@ -51766,8 +51775,8 @@
       <c r="G1297" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H1297" s="8" t="s">
-        <v>24</v>
+      <c r="H1297" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1297" s="4" t="s">
         <v>20</v>
@@ -51828,7 +51837,7 @@
         <v>13</v>
       </c>
       <c r="C1299" s="2" t="s">
-        <v>22</v>
+        <v>629</v>
       </c>
       <c r="D1299" s="4" t="s">
         <v>607</v>
@@ -51842,8 +51851,8 @@
       <c r="G1299" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H1299" s="8" t="s">
-        <v>24</v>
+      <c r="H1299" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1299" s="4" t="s">
         <v>20</v>
@@ -51942,7 +51951,7 @@
         <v>13</v>
       </c>
       <c r="C1302" s="2" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="D1302" s="4" t="s">
         <v>607</v>
@@ -51960,7 +51969,7 @@
         <v>19</v>
       </c>
       <c r="I1302" s="4" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="J1302" s="4" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-21T06:20:17.490Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="634">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="635">
   <si>
     <t>Date</t>
   </si>
@@ -1895,6 +1895,9 @@
   </si>
   <si>
     <t>2026-10-21</t>
+  </si>
+  <si>
+    <t>Tony tim</t>
   </si>
   <si>
     <t>S-mvheq8oo-60m22</t>
@@ -51498,7 +51501,7 @@
         <v>346</v>
       </c>
       <c r="D1290" s="22" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1290" s="22" t="s">
         <v>158</v>
@@ -51519,7 +51522,7 @@
         <v>20</v>
       </c>
       <c r="K1290" s="24" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1290" s="20" t="s">
         <v>626</v>
@@ -51536,10 +51539,10 @@
         <v>22</v>
       </c>
       <c r="D1291" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1291" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1291" s="5" t="s">
         <v>17</v>
@@ -51551,13 +51554,13 @@
         <v>24</v>
       </c>
       <c r="I1291" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="J1291" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1291" s="7" t="s">
         <v>628</v>
-      </c>
-      <c r="J1291" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K1291" s="7" t="s">
-        <v>627</v>
       </c>
       <c r="L1291" s="2" t="s">
         <v>626</v>
@@ -51574,10 +51577,10 @@
         <v>22</v>
       </c>
       <c r="D1292" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1292" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1292" s="5" t="s">
         <v>17</v>
@@ -51589,13 +51592,13 @@
         <v>24</v>
       </c>
       <c r="I1292" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="J1292" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1292" s="7" t="s">
         <v>628</v>
-      </c>
-      <c r="J1292" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K1292" s="7" t="s">
-        <v>627</v>
       </c>
       <c r="L1292" s="2" t="s">
         <v>626</v>
@@ -51612,7 +51615,7 @@
         <v>346</v>
       </c>
       <c r="D1293" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1293" s="4" t="s">
         <v>158</v>
@@ -51633,7 +51636,7 @@
         <v>20</v>
       </c>
       <c r="K1293" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1293" s="2" t="s">
         <v>626</v>
@@ -51647,10 +51650,10 @@
         <v>13</v>
       </c>
       <c r="C1294" s="2" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D1294" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1294" s="4" t="s">
         <v>288</v>
@@ -51659,7 +51662,7 @@
         <v>17</v>
       </c>
       <c r="G1294" s="4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="H1294" s="6" t="s">
         <v>19</v>
@@ -51671,7 +51674,7 @@
         <v>20</v>
       </c>
       <c r="K1294" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1294" s="2" t="s">
         <v>626</v>
@@ -51685,13 +51688,13 @@
         <v>13</v>
       </c>
       <c r="C1295" s="2" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D1295" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1295" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1295" s="5" t="s">
         <v>29</v>
@@ -51709,7 +51712,7 @@
         <v>20</v>
       </c>
       <c r="K1295" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1295" s="2" t="s">
         <v>626</v>
@@ -51726,10 +51729,10 @@
         <v>532</v>
       </c>
       <c r="D1296" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1296" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1296" s="5" t="s">
         <v>29</v>
@@ -51747,7 +51750,7 @@
         <v>20</v>
       </c>
       <c r="K1296" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1296" s="2" t="s">
         <v>626</v>
@@ -51761,10 +51764,10 @@
         <v>13</v>
       </c>
       <c r="C1297" s="2" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D1297" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1297" s="4" t="s">
         <v>288</v>
@@ -51785,7 +51788,7 @@
         <v>20</v>
       </c>
       <c r="K1297" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1297" s="2" t="s">
         <v>626</v>
@@ -51802,10 +51805,10 @@
         <v>22</v>
       </c>
       <c r="D1298" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1298" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1298" s="5" t="s">
         <v>29</v>
@@ -51823,7 +51826,7 @@
         <v>20</v>
       </c>
       <c r="K1298" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1298" s="2" t="s">
         <v>626</v>
@@ -51837,13 +51840,13 @@
         <v>13</v>
       </c>
       <c r="C1299" s="2" t="s">
-        <v>629</v>
+        <v>22</v>
       </c>
       <c r="D1299" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1299" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1299" s="5" t="s">
         <v>29</v>
@@ -51851,8 +51854,8 @@
       <c r="G1299" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H1299" s="6" t="s">
-        <v>19</v>
+      <c r="H1299" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="I1299" s="4" t="s">
         <v>20</v>
@@ -51861,7 +51864,7 @@
         <v>20</v>
       </c>
       <c r="K1299" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1299" s="2" t="s">
         <v>626</v>
@@ -51878,10 +51881,10 @@
         <v>22</v>
       </c>
       <c r="D1300" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1300" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1300" s="5" t="s">
         <v>36</v>
@@ -51899,7 +51902,7 @@
         <v>20</v>
       </c>
       <c r="K1300" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1300" s="2" t="s">
         <v>626</v>
@@ -51916,10 +51919,10 @@
         <v>22</v>
       </c>
       <c r="D1301" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1301" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1301" s="5" t="s">
         <v>36</v>
@@ -51937,7 +51940,7 @@
         <v>20</v>
       </c>
       <c r="K1301" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1301" s="2" t="s">
         <v>626</v>
@@ -51951,13 +51954,13 @@
         <v>13</v>
       </c>
       <c r="C1302" s="2" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="D1302" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1302" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1302" s="5" t="s">
         <v>36</v>
@@ -51969,13 +51972,13 @@
         <v>19</v>
       </c>
       <c r="I1302" s="4" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="J1302" s="4" t="s">
         <v>20</v>
       </c>
       <c r="K1302" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1302" s="2" t="s">
         <v>626</v>
@@ -51992,10 +51995,10 @@
         <v>22</v>
       </c>
       <c r="D1303" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="E1303" s="4" t="s">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="F1303" s="5" t="s">
         <v>36</v>
@@ -52013,7 +52016,7 @@
         <v>20</v>
       </c>
       <c r="K1303" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="L1303" s="2" t="s">
         <v>626</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-21T06:35:04.701Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="636">
   <si>
     <t>Date</t>
   </si>
@@ -1913,6 +1913,9 @@
   </si>
   <si>
     <t>07:16</t>
+  </si>
+  <si>
+    <t>16:34</t>
   </si>
   <si>
     <t>13:55</t>
@@ -51802,13 +51805,13 @@
         <v>13</v>
       </c>
       <c r="C1298" s="2" t="s">
-        <v>22</v>
+        <v>633</v>
       </c>
       <c r="D1298" s="4" t="s">
         <v>627</v>
       </c>
       <c r="E1298" s="4" t="s">
-        <v>627</v>
+        <v>288</v>
       </c>
       <c r="F1298" s="5" t="s">
         <v>29</v>
@@ -51816,8 +51819,8 @@
       <c r="G1298" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H1298" s="8" t="s">
-        <v>24</v>
+      <c r="H1298" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1298" s="4" t="s">
         <v>20</v>
@@ -51954,7 +51957,7 @@
         <v>13</v>
       </c>
       <c r="C1302" s="2" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D1302" s="4" t="s">
         <v>627</v>
@@ -51972,7 +51975,7 @@
         <v>19</v>
       </c>
       <c r="I1302" s="4" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="J1302" s="4" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-21T06:38:30.134Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="637">
   <si>
     <t>Date</t>
   </si>
@@ -1916,6 +1916,9 @@
   </si>
   <si>
     <t>16:34</t>
+  </si>
+  <si>
+    <t>16:38</t>
   </si>
   <si>
     <t>13:55</t>
@@ -51843,13 +51846,13 @@
         <v>13</v>
       </c>
       <c r="C1299" s="2" t="s">
-        <v>22</v>
+        <v>634</v>
       </c>
       <c r="D1299" s="4" t="s">
         <v>627</v>
       </c>
       <c r="E1299" s="4" t="s">
-        <v>627</v>
+        <v>288</v>
       </c>
       <c r="F1299" s="5" t="s">
         <v>29</v>
@@ -51857,8 +51860,8 @@
       <c r="G1299" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H1299" s="8" t="s">
-        <v>24</v>
+      <c r="H1299" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1299" s="4" t="s">
         <v>20</v>
@@ -51957,7 +51960,7 @@
         <v>13</v>
       </c>
       <c r="C1302" s="2" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D1302" s="4" t="s">
         <v>627</v>
@@ -51975,7 +51978,7 @@
         <v>19</v>
       </c>
       <c r="I1302" s="4" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="J1302" s="4" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-21T08:03:40.514Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15636" uniqueCount="637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15804" uniqueCount="639">
   <si>
     <t>Date</t>
   </si>
@@ -1925,6 +1925,12 @@
   </si>
   <si>
     <t>Water Delivered</t>
+  </si>
+  <si>
+    <t>18:02</t>
+  </si>
+  <si>
+    <t>S-mvheq5pl-wjfi7</t>
   </si>
 </sst>
 </file>
@@ -2500,7 +2506,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1303"/>
+  <dimension ref="A1:L1317"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -52028,8 +52034,540 @@
         <v>626</v>
       </c>
     </row>
+    <row r="1304" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1304" s="9" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1304" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1304" s="9" t="s">
+        <v>637</v>
+      </c>
+      <c r="D1304" s="11" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1304" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1304" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1304" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1304" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1304" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1304" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1304" s="14" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1304" s="9" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1305" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1305" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1305" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1305" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1305" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1305" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1305" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1305" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1305" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1305" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1305" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1305" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1305" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1306" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1306" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1306" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1306" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1306" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1306" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1306" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1306" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1306" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1306" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1306" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1306" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1306" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1307" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1307" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1307" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1307" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1307" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1307" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1307" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1307" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1307" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1307" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1307" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1307" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1307" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1308" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1308" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1308" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1308" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1308" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1308" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1308" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1308" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1308" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1308" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1308" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1308" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1308" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1309" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1309" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1309" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1309" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1309" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1309" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1309" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1309" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1309" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1309" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1309" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1309" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1309" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1310" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1310" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1310" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1310" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1310" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1310" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1310" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1310" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1310" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1310" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1310" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1310" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1310" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1311" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1311" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1311" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1311" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1311" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1311" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1311" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1311" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1311" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1311" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1311" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1311" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1311" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1312" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1312" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1312" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1312" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1312" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1312" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1312" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1312" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1312" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1312" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1312" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1312" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1312" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1313" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1313" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1313" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1313" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1313" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1313" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1313" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1313" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1313" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1313" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1313" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1313" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1313" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1314" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1314" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1314" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1314" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1314" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1314" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1314" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1314" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1314" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1314" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1314" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1314" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1314" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1315" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1315" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1315" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1315" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1315" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1315" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1315" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1315" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1315" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1315" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1315" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1315" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1315" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1316" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1316" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1316" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1316" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1316" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1316" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1316" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1316" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1316" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1316" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1316" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1316" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1316" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="1317" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1317" s="15" t="s">
+        <v>626</v>
+      </c>
+      <c r="B1317" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1317" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1317" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E1317" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F1317" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1317" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1317" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1317" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1317" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1317" s="19" t="s">
+        <v>638</v>
+      </c>
+      <c r="L1317" s="15" t="s">
+        <v>626</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1303"/>
+  <autoFilter ref="A1:L1317"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-22T17:19:36.718Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15804" uniqueCount="639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15972" uniqueCount="645">
   <si>
     <t>Date</t>
   </si>
@@ -1931,6 +1931,24 @@
   </si>
   <si>
     <t>S-mvheq5pl-wjfi7</t>
+  </si>
+  <si>
+    <t>2026-10-23</t>
+  </si>
+  <si>
+    <t>18:22</t>
+  </si>
+  <si>
+    <t>Ben/Ken</t>
+  </si>
+  <si>
+    <t>S-mvj97zeq-nklwi</t>
+  </si>
+  <si>
+    <t>2026-10-22</t>
+  </si>
+  <si>
+    <t>03:19</t>
   </si>
 </sst>
 </file>
@@ -2506,7 +2524,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1317"/>
+  <dimension ref="A1:L1331"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -52566,8 +52584,540 @@
         <v>626</v>
       </c>
     </row>
+    <row r="1318" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1318" s="20" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1318" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1318" s="20" t="s">
+        <v>640</v>
+      </c>
+      <c r="D1318" s="22" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1318" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1318" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1318" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1318" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1318" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1318" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1318" s="24" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1318" s="20" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1319" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1319" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1319" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1319" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1319" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1319" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1319" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1319" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1319" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1319" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1319" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1319" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1319" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1320" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1320" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1320" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1320" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1320" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1320" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1320" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1320" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1320" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1320" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1320" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1320" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1320" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1321" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1321" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1321" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1321" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1321" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1321" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1321" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1321" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1321" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1321" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1321" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1321" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1321" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1322" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1322" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1322" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1322" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1322" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1322" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1322" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1322" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1322" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1322" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1322" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1322" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1322" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1323" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1323" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1323" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1323" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1323" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1323" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1323" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1323" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1323" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1323" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1323" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1323" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1323" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1324" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1324" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1324" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1324" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1324" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1324" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1324" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1324" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1324" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1324" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1324" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1324" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1324" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1325" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1325" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1325" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1325" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="D1325" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1325" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1325" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1325" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1325" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1325" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1325" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1325" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1325" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1326" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1326" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1326" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1326" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1326" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1326" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1326" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1326" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1326" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1326" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1326" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1326" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1326" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1327" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1327" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1327" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1327" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1327" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1327" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1327" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1327" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1327" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1327" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1327" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1327" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1327" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1328" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1328" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1328" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1328" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1328" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1328" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1328" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1328" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1328" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1328" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1328" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1328" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1328" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1329" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1329" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1329" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1329" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1329" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1329" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1329" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1329" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1329" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1329" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1329" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1329" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1329" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1330" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1330" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1330" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1330" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1330" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1330" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1330" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1330" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1330" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1330" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1330" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1330" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1330" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="1331" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1331" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1331" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1331" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1331" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="E1331" s="4" t="s">
+        <v>641</v>
+      </c>
+      <c r="F1331" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1331" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1331" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1331" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1331" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1331" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="L1331" s="2" t="s">
+        <v>643</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1317"/>
+  <autoFilter ref="A1:L1331"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-22T19:35:00.573Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15972" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15972" uniqueCount="646">
   <si>
     <t>Date</t>
   </si>
@@ -1949,6 +1949,9 @@
   </si>
   <si>
     <t>03:19</t>
+  </si>
+  <si>
+    <t>05:09</t>
   </si>
 </sst>
 </file>
@@ -52896,13 +52899,13 @@
         <v>42</v>
       </c>
       <c r="C1326" s="2" t="s">
-        <v>22</v>
+        <v>645</v>
       </c>
       <c r="D1326" s="4" t="s">
         <v>641</v>
       </c>
       <c r="E1326" s="4" t="s">
-        <v>641</v>
+        <v>431</v>
       </c>
       <c r="F1326" s="5" t="s">
         <v>29</v>
@@ -52910,8 +52913,8 @@
       <c r="G1326" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H1326" s="8" t="s">
-        <v>24</v>
+      <c r="H1326" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1326" s="4" t="s">
         <v>20</v>
@@ -52934,13 +52937,13 @@
         <v>42</v>
       </c>
       <c r="C1327" s="2" t="s">
-        <v>22</v>
+        <v>645</v>
       </c>
       <c r="D1327" s="4" t="s">
         <v>641</v>
       </c>
       <c r="E1327" s="4" t="s">
-        <v>641</v>
+        <v>16</v>
       </c>
       <c r="F1327" s="5" t="s">
         <v>29</v>
@@ -52948,8 +52951,8 @@
       <c r="G1327" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H1327" s="8" t="s">
-        <v>24</v>
+      <c r="H1327" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1327" s="4" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-22T21:05:00.803Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15972" uniqueCount="646">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16140" uniqueCount="650">
   <si>
     <t>Date</t>
   </si>
@@ -1952,6 +1952,18 @@
   </si>
   <si>
     <t>05:09</t>
+  </si>
+  <si>
+    <t>06:54</t>
+  </si>
+  <si>
+    <t>Anthony  Kyle</t>
+  </si>
+  <si>
+    <t>anthoy</t>
+  </si>
+  <si>
+    <t>S-mvk0rb1h-1nj2g</t>
   </si>
 </sst>
 </file>
@@ -2527,7 +2539,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1331"/>
+  <dimension ref="A1:L1345"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -53119,8 +53131,540 @@
         <v>643</v>
       </c>
     </row>
+    <row r="1332" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1332" s="9" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1332" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1332" s="9" t="s">
+        <v>646</v>
+      </c>
+      <c r="D1332" s="11" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1332" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="F1332" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1332" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1332" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1332" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1332" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1332" s="14" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1332" s="9" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1333" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1333" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1333" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1333" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1333" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1333" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1333" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1333" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1333" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1333" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="J1333" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1333" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1333" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1334" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1334" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1334" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1334" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1334" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1334" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1334" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1334" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1334" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1334" s="17" t="s">
+        <v>629</v>
+      </c>
+      <c r="J1334" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1334" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1334" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1335" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1335" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1335" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1335" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1335" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1335" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1335" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1335" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1335" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1335" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1335" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1335" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1335" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1336" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1336" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1336" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1336" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1336" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1336" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1336" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1336" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1336" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1336" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1336" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1336" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1336" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1337" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1337" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1337" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1337" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1337" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1337" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1337" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1337" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1337" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1337" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1337" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1337" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1337" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1338" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1338" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1338" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1338" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1338" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1338" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1338" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1338" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1338" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1338" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1338" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1338" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1338" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1339" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1339" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1339" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1339" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1339" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1339" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1339" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1339" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1339" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1339" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1339" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1339" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1339" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1340" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1340" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1340" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1340" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1340" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1340" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1340" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1340" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1340" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1340" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1340" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1340" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1340" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1341" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1341" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1341" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1341" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1341" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1341" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1341" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1341" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1341" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1341" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1341" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1341" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1341" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1342" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1342" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1342" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1342" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1342" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1342" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1342" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1342" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1342" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1342" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1342" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1342" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1342" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1343" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1343" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1343" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1343" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1343" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1343" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1343" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1343" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1343" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1343" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1343" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1343" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1343" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1344" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1344" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1344" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1344" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1344" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1344" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1344" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1344" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1344" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1344" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1344" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1344" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1344" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1345" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1345" s="15" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1345" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1345" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1345" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="E1345" s="17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F1345" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1345" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1345" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1345" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1345" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1345" s="19" t="s">
+        <v>649</v>
+      </c>
+      <c r="L1345" s="15" t="s">
+        <v>639</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1331"/>
+  <autoFilter ref="A1:L1345"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-23T08:15:53.853Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16140" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16140" uniqueCount="649">
   <si>
     <t>Date</t>
   </si>
@@ -1958,9 +1958,6 @@
   </si>
   <si>
     <t>Anthony  Kyle</t>
-  </si>
-  <si>
-    <t>anthoy</t>
   </si>
   <si>
     <t>S-mvk0rb1h-1nj2g</t>
@@ -53145,7 +53142,7 @@
         <v>647</v>
       </c>
       <c r="E1332" s="11" t="s">
-        <v>648</v>
+        <v>45</v>
       </c>
       <c r="F1332" s="12" t="s">
         <v>17</v>
@@ -53163,7 +53160,7 @@
         <v>20</v>
       </c>
       <c r="K1332" s="14" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1332" s="9" t="s">
         <v>639</v>
@@ -53201,7 +53198,7 @@
         <v>20</v>
       </c>
       <c r="K1333" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1333" s="15" t="s">
         <v>639</v>
@@ -53239,7 +53236,7 @@
         <v>20</v>
       </c>
       <c r="K1334" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1334" s="15" t="s">
         <v>639</v>
@@ -53277,7 +53274,7 @@
         <v>20</v>
       </c>
       <c r="K1335" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1335" s="15" t="s">
         <v>639</v>
@@ -53315,7 +53312,7 @@
         <v>20</v>
       </c>
       <c r="K1336" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1336" s="15" t="s">
         <v>639</v>
@@ -53329,13 +53326,13 @@
         <v>13</v>
       </c>
       <c r="C1337" s="15" t="s">
-        <v>22</v>
+        <v>300</v>
       </c>
       <c r="D1337" s="17" t="s">
         <v>647</v>
       </c>
       <c r="E1337" s="17" t="s">
-        <v>647</v>
+        <v>427</v>
       </c>
       <c r="F1337" s="18" t="s">
         <v>29</v>
@@ -53343,8 +53340,8 @@
       <c r="G1337" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="H1337" s="8" t="s">
-        <v>24</v>
+      <c r="H1337" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1337" s="17" t="s">
         <v>20</v>
@@ -53353,7 +53350,7 @@
         <v>20</v>
       </c>
       <c r="K1337" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1337" s="15" t="s">
         <v>639</v>
@@ -53367,13 +53364,13 @@
         <v>13</v>
       </c>
       <c r="C1338" s="15" t="s">
-        <v>22</v>
+        <v>615</v>
       </c>
       <c r="D1338" s="17" t="s">
         <v>647</v>
       </c>
       <c r="E1338" s="17" t="s">
-        <v>647</v>
+        <v>283</v>
       </c>
       <c r="F1338" s="18" t="s">
         <v>29</v>
@@ -53381,8 +53378,8 @@
       <c r="G1338" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="H1338" s="8" t="s">
-        <v>24</v>
+      <c r="H1338" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1338" s="17" t="s">
         <v>20</v>
@@ -53391,7 +53388,7 @@
         <v>20</v>
       </c>
       <c r="K1338" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1338" s="15" t="s">
         <v>639</v>
@@ -53405,13 +53402,13 @@
         <v>13</v>
       </c>
       <c r="C1339" s="15" t="s">
-        <v>22</v>
+        <v>425</v>
       </c>
       <c r="D1339" s="17" t="s">
         <v>647</v>
       </c>
       <c r="E1339" s="17" t="s">
-        <v>647</v>
+        <v>283</v>
       </c>
       <c r="F1339" s="18" t="s">
         <v>29</v>
@@ -53419,8 +53416,8 @@
       <c r="G1339" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="H1339" s="8" t="s">
-        <v>24</v>
+      <c r="H1339" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1339" s="17" t="s">
         <v>20</v>
@@ -53429,7 +53426,7 @@
         <v>20</v>
       </c>
       <c r="K1339" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1339" s="15" t="s">
         <v>639</v>
@@ -53467,7 +53464,7 @@
         <v>20</v>
       </c>
       <c r="K1340" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1340" s="15" t="s">
         <v>639</v>
@@ -53505,7 +53502,7 @@
         <v>20</v>
       </c>
       <c r="K1341" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1341" s="15" t="s">
         <v>639</v>
@@ -53543,7 +53540,7 @@
         <v>20</v>
       </c>
       <c r="K1342" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1342" s="15" t="s">
         <v>639</v>
@@ -53581,7 +53578,7 @@
         <v>20</v>
       </c>
       <c r="K1343" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1343" s="15" t="s">
         <v>639</v>
@@ -53619,7 +53616,7 @@
         <v>20</v>
       </c>
       <c r="K1344" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1344" s="15" t="s">
         <v>639</v>
@@ -53657,7 +53654,7 @@
         <v>20</v>
       </c>
       <c r="K1345" s="19" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="L1345" s="15" t="s">
         <v>639</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-23T11:59:52.678Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16140" uniqueCount="649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16308" uniqueCount="653">
   <si>
     <t>Date</t>
   </si>
@@ -1961,6 +1961,18 @@
   </si>
   <si>
     <t>S-mvk0rb1h-1nj2g</t>
+  </si>
+  <si>
+    <t>18:21</t>
+  </si>
+  <si>
+    <t>S-mvkpa4i8-s7v03</t>
+  </si>
+  <si>
+    <t>18:36</t>
+  </si>
+  <si>
+    <t>21:59</t>
   </si>
 </sst>
 </file>
@@ -2536,7 +2548,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1345"/>
+  <dimension ref="A1:L1359"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -53660,8 +53672,540 @@
         <v>639</v>
       </c>
     </row>
+    <row r="1346" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1346" s="20" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1346" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1346" s="20" t="s">
+        <v>649</v>
+      </c>
+      <c r="D1346" s="22" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1346" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1346" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1346" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1346" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1346" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1346" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1346" s="24" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1346" s="20" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1347" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1347" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1347" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1347" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1347" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1347" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1347" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1347" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1347" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1347" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1347" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1347" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1347" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1348" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1348" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1348" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1348" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1348" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1348" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1348" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1348" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1348" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1348" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1348" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1348" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1348" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1349" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1349" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1349" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1349" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="D1349" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1349" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1349" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1349" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1349" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1349" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1349" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1349" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1349" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1350" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1350" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1350" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1350" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1350" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1350" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1350" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1350" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1350" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1350" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1350" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1350" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1350" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1351" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1351" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1351" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1351" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="D1351" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1351" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1351" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1351" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1351" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1351" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1351" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1351" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1351" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1352" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1352" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1352" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1352" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="D1352" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1352" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1352" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1352" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1352" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1352" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1352" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1352" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1352" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1353" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1353" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1353" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1353" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1353" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1353" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1353" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1353" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1353" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1353" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1353" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1353" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1353" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1354" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1354" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1354" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1354" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1354" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1354" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1354" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1354" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1354" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1354" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1354" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1354" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1354" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1355" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1355" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1355" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1355" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1355" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1355" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1355" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1355" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1355" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1355" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1355" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1355" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1355" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1356" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1356" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1356" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1356" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1356" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1356" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1356" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1356" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1356" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1356" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1356" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1356" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1356" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1357" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1357" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1357" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1357" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1357" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1357" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1357" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1357" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1357" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1357" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1357" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1357" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1357" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1358" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1358" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1358" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1358" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1358" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1358" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1358" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1358" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1358" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1358" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1358" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1358" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1358" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1359" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1359" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B1359" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1359" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1359" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1359" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1359" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1359" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1359" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1359" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1359" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1359" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="L1359" s="2" t="s">
+        <v>639</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1345"/>
+  <autoFilter ref="A1:L1359"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-23T19:17:33.118Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16308" uniqueCount="653">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16308" uniqueCount="656">
   <si>
     <t>Date</t>
   </si>
@@ -1963,6 +1963,9 @@
     <t>S-mvk0rb1h-1nj2g</t>
   </si>
   <si>
+    <t>2026-10-24</t>
+  </si>
+  <si>
     <t>18:21</t>
   </si>
   <si>
@@ -1973,6 +1976,12 @@
   </si>
   <si>
     <t>21:59</t>
+  </si>
+  <si>
+    <t>03:31</t>
+  </si>
+  <si>
+    <t>05:17</t>
   </si>
 </sst>
 </file>
@@ -53674,13 +53683,13 @@
     </row>
     <row r="1346" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1346" s="20" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1346" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C1346" s="20" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D1346" s="22" t="s">
         <v>430</v>
@@ -53704,7 +53713,7 @@
         <v>20</v>
       </c>
       <c r="K1346" s="24" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1346" s="20" t="s">
         <v>639</v>
@@ -53712,7 +53721,7 @@
     </row>
     <row r="1347" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1347" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1347" s="16" t="s">
         <v>42</v>
@@ -53742,7 +53751,7 @@
         <v>20</v>
       </c>
       <c r="K1347" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1347" s="2" t="s">
         <v>639</v>
@@ -53750,7 +53759,7 @@
     </row>
     <row r="1348" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1348" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1348" s="16" t="s">
         <v>42</v>
@@ -53780,7 +53789,7 @@
         <v>20</v>
       </c>
       <c r="K1348" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1348" s="2" t="s">
         <v>639</v>
@@ -53788,13 +53797,13 @@
     </row>
     <row r="1349" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1349" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1349" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1349" s="2" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D1349" s="4" t="s">
         <v>430</v>
@@ -53818,7 +53827,7 @@
         <v>20</v>
       </c>
       <c r="K1349" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1349" s="2" t="s">
         <v>639</v>
@@ -53826,7 +53835,7 @@
     </row>
     <row r="1350" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1350" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1350" s="16" t="s">
         <v>42</v>
@@ -53856,7 +53865,7 @@
         <v>20</v>
       </c>
       <c r="K1350" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1350" s="2" t="s">
         <v>639</v>
@@ -53864,13 +53873,13 @@
     </row>
     <row r="1351" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1351" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1351" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1351" s="2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D1351" s="4" t="s">
         <v>430</v>
@@ -53894,7 +53903,7 @@
         <v>20</v>
       </c>
       <c r="K1351" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1351" s="2" t="s">
         <v>639</v>
@@ -53902,13 +53911,13 @@
     </row>
     <row r="1352" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1352" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1352" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1352" s="2" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="D1352" s="4" t="s">
         <v>430</v>
@@ -53932,7 +53941,7 @@
         <v>20</v>
       </c>
       <c r="K1352" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1352" s="2" t="s">
         <v>639</v>
@@ -53940,19 +53949,19 @@
     </row>
     <row r="1353" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1353" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1353" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1353" s="2" t="s">
-        <v>22</v>
+        <v>654</v>
       </c>
       <c r="D1353" s="4" t="s">
         <v>430</v>
       </c>
       <c r="E1353" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F1353" s="5" t="s">
         <v>29</v>
@@ -53960,8 +53969,8 @@
       <c r="G1353" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H1353" s="8" t="s">
-        <v>24</v>
+      <c r="H1353" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1353" s="4" t="s">
         <v>20</v>
@@ -53970,7 +53979,7 @@
         <v>20</v>
       </c>
       <c r="K1353" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1353" s="2" t="s">
         <v>639</v>
@@ -53978,19 +53987,19 @@
     </row>
     <row r="1354" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1354" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1354" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1354" s="2" t="s">
-        <v>22</v>
+        <v>655</v>
       </c>
       <c r="D1354" s="4" t="s">
         <v>430</v>
       </c>
       <c r="E1354" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F1354" s="5" t="s">
         <v>29</v>
@@ -53998,8 +54007,8 @@
       <c r="G1354" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H1354" s="8" t="s">
-        <v>24</v>
+      <c r="H1354" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1354" s="4" t="s">
         <v>20</v>
@@ -54008,7 +54017,7 @@
         <v>20</v>
       </c>
       <c r="K1354" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1354" s="2" t="s">
         <v>639</v>
@@ -54016,19 +54025,19 @@
     </row>
     <row r="1355" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1355" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1355" s="16" t="s">
         <v>42</v>
       </c>
       <c r="C1355" s="2" t="s">
-        <v>22</v>
+        <v>655</v>
       </c>
       <c r="D1355" s="4" t="s">
         <v>430</v>
       </c>
       <c r="E1355" s="4" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F1355" s="5" t="s">
         <v>29</v>
@@ -54036,8 +54045,8 @@
       <c r="G1355" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H1355" s="8" t="s">
-        <v>24</v>
+      <c r="H1355" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1355" s="4" t="s">
         <v>20</v>
@@ -54046,7 +54055,7 @@
         <v>20</v>
       </c>
       <c r="K1355" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1355" s="2" t="s">
         <v>639</v>
@@ -54054,7 +54063,7 @@
     </row>
     <row r="1356" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1356" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1356" s="16" t="s">
         <v>42</v>
@@ -54084,7 +54093,7 @@
         <v>20</v>
       </c>
       <c r="K1356" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1356" s="2" t="s">
         <v>639</v>
@@ -54092,7 +54101,7 @@
     </row>
     <row r="1357" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1357" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1357" s="16" t="s">
         <v>42</v>
@@ -54122,7 +54131,7 @@
         <v>20</v>
       </c>
       <c r="K1357" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1357" s="2" t="s">
         <v>639</v>
@@ -54130,7 +54139,7 @@
     </row>
     <row r="1358" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1358" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1358" s="16" t="s">
         <v>42</v>
@@ -54160,7 +54169,7 @@
         <v>20</v>
       </c>
       <c r="K1358" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1358" s="2" t="s">
         <v>639</v>
@@ -54168,7 +54177,7 @@
     </row>
     <row r="1359" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1359" s="2" t="s">
-        <v>639</v>
+        <v>649</v>
       </c>
       <c r="B1359" s="16" t="s">
         <v>42</v>
@@ -54198,7 +54207,7 @@
         <v>20</v>
       </c>
       <c r="K1359" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="L1359" s="2" t="s">
         <v>639</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-24T19:47:01.302Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16308" uniqueCount="656">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16476" uniqueCount="659">
   <si>
     <t>Date</t>
   </si>
@@ -1982,6 +1982,15 @@
   </si>
   <si>
     <t>05:17</t>
+  </si>
+  <si>
+    <t>2026-10-25</t>
+  </si>
+  <si>
+    <t>S-mvm4803m-egbsn</t>
+  </si>
+  <si>
+    <t>05:46</t>
   </si>
 </sst>
 </file>
@@ -2557,7 +2566,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1359"/>
+  <dimension ref="A1:L1373"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -54213,8 +54222,540 @@
         <v>639</v>
       </c>
     </row>
+    <row r="1360" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1360" s="9" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1360" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1360" s="9" t="s">
+        <v>565</v>
+      </c>
+      <c r="D1360" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1360" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1360" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1360" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1360" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1360" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1360" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1360" s="14" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1360" s="9" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1361" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1361" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1361" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1361" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1361" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1361" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1361" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1361" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1361" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1361" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1361" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1361" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1361" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1362" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1362" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1362" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1362" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1362" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1362" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1362" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1362" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1362" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1362" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1362" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1362" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1362" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1363" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1363" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1363" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1363" s="15" t="s">
+        <v>565</v>
+      </c>
+      <c r="D1363" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1363" s="17" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1363" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1363" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1363" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1363" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1363" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1363" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1363" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1364" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1364" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1364" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1364" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1364" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1364" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1364" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1364" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1364" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1364" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1364" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1364" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1364" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1365" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1365" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1365" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1365" s="15" t="s">
+        <v>564</v>
+      </c>
+      <c r="D1365" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1365" s="17" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1365" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1365" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1365" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1365" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1365" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1365" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1365" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1366" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1366" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1366" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1366" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1366" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1366" s="17" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1366" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1366" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1366" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1366" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1366" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1366" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1366" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1367" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1367" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1367" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1367" s="15" t="s">
+        <v>601</v>
+      </c>
+      <c r="D1367" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1367" s="17" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1367" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1367" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1367" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1367" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1367" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1367" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1367" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1368" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1368" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1368" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1368" s="15" t="s">
+        <v>658</v>
+      </c>
+      <c r="D1368" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1368" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1368" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1368" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1368" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1368" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1368" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1368" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1368" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1369" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1369" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1369" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1369" s="15" t="s">
+        <v>658</v>
+      </c>
+      <c r="D1369" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1369" s="17" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1369" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1369" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1369" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1369" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1369" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1369" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1369" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1370" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1370" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1370" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1370" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1370" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1370" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1370" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1370" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1370" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1370" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1370" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1370" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1370" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1371" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1371" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1371" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1371" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1371" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1371" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1371" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1371" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1371" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1371" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1371" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1371" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1371" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1372" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1372" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1372" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1372" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1372" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1372" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1372" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1372" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1372" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1372" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1372" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1372" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1372" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="1373" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1373" s="15" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1373" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1373" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1373" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="E1373" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="F1373" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1373" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1373" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1373" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1373" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1373" s="19" t="s">
+        <v>657</v>
+      </c>
+      <c r="L1373" s="15" t="s">
+        <v>649</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1359"/>
+  <autoFilter ref="A1:L1373"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-25T08:30:55.825Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16476" uniqueCount="659">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16644" uniqueCount="664">
   <si>
     <t>Date</t>
   </si>
@@ -1991,6 +1991,21 @@
   </si>
   <si>
     <t>05:46</t>
+  </si>
+  <si>
+    <t>06:09</t>
+  </si>
+  <si>
+    <t>Anthony   Kyle</t>
+  </si>
+  <si>
+    <t>S-mvmt8lxx-qc1ox</t>
+  </si>
+  <si>
+    <t>09:07</t>
+  </si>
+  <si>
+    <t>10:38</t>
   </si>
 </sst>
 </file>
@@ -2566,7 +2581,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1373"/>
+  <dimension ref="A1:L1387"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -54754,8 +54769,540 @@
         <v>649</v>
       </c>
     </row>
+    <row r="1374" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1374" s="20" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1374" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1374" s="20" t="s">
+        <v>659</v>
+      </c>
+      <c r="D1374" s="22" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1374" s="22" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1374" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1374" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1374" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1374" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1374" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1374" s="24" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1374" s="20" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1375" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1375" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1375" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1375" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1375" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1375" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1375" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1375" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1375" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1375" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1375" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1375" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1375" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1376" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1376" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1376" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1376" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1376" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1376" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1376" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1376" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1376" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1376" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1376" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1376" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1376" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1377" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1377" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1377" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1377" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="D1377" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1377" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1377" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1377" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1377" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1377" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1377" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1377" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1377" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1378" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1378" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1378" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1378" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1378" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1378" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1378" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1378" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1378" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1378" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1378" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1378" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1378" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1379" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1379" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1379" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1379" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="D1379" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1379" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="F1379" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1379" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1379" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1379" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1379" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1379" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1379" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1380" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1380" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1380" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1380" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1380" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1380" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="F1380" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1380" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1380" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1380" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1380" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1380" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1380" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1381" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1381" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1381" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1381" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1381" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1381" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1381" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1381" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1381" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1381" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1381" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1381" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1381" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1382" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1382" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1382" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1382" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1382" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1382" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1382" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1382" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1382" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1382" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1382" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1382" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1382" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1383" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1383" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1383" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1383" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1383" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1383" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1383" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1383" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1383" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1383" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1383" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1383" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1383" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1384" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1384" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1384" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1384" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="D1384" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1384" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="F1384" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1384" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1384" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1384" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1384" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1384" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1384" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1385" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1385" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1385" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1385" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1385" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1385" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1385" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1385" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1385" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1385" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1385" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1385" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1385" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1386" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1386" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1386" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1386" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1386" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1386" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1386" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1386" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1386" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1386" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1386" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1386" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1386" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="1387" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1387" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1387" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1387" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1387" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="E1387" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="F1387" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1387" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1387" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1387" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1387" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1387" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L1387" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1373"/>
+  <autoFilter ref="A1:L1387"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-26T01:30:55.043Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16644" uniqueCount="664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16812" uniqueCount="671">
   <si>
     <t>Date</t>
   </si>
@@ -2006,6 +2006,27 @@
   </si>
   <si>
     <t>10:38</t>
+  </si>
+  <si>
+    <t>2026-10-26</t>
+  </si>
+  <si>
+    <t>S-mvof7s86-jl7wm</t>
+  </si>
+  <si>
+    <t>06:55</t>
+  </si>
+  <si>
+    <t>08:42</t>
+  </si>
+  <si>
+    <t>09:55</t>
+  </si>
+  <si>
+    <t>drum has been changed</t>
+  </si>
+  <si>
+    <t>10:09</t>
   </si>
 </sst>
 </file>
@@ -2581,7 +2602,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1387"/>
+  <dimension ref="A1:L1401"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -55301,8 +55322,540 @@
         <v>656</v>
       </c>
     </row>
+    <row r="1388" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1388" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1388" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1388" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="D1388" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1388" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1388" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1388" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1388" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1388" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1388" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1388" s="14" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1388" s="9" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1389" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1389" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1389" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1389" s="15" t="s">
+        <v>306</v>
+      </c>
+      <c r="D1389" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1389" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1389" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1389" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1389" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1389" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1389" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1389" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1389" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1390" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1390" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1390" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1390" s="15" t="s">
+        <v>306</v>
+      </c>
+      <c r="D1390" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1390" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1390" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1390" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1390" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1390" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1390" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1390" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1390" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1391" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1391" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1391" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1391" s="15" t="s">
+        <v>666</v>
+      </c>
+      <c r="D1391" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1391" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1391" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1391" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1391" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1391" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1391" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1391" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1391" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1392" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1392" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1392" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1392" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1392" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1392" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1392" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1392" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1392" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1392" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1392" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1392" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1392" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1393" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1393" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1393" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1393" s="15" t="s">
+        <v>667</v>
+      </c>
+      <c r="D1393" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1393" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1393" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1393" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1393" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1393" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1393" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1393" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1393" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1394" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1394" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1394" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1394" s="15" t="s">
+        <v>668</v>
+      </c>
+      <c r="D1394" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1394" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1394" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1394" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1394" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1394" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1394" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1394" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1394" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1395" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1395" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1395" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1395" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1395" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1395" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1395" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1395" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1395" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1395" s="17" t="s">
+        <v>669</v>
+      </c>
+      <c r="J1395" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1395" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1395" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1396" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1396" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1396" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1396" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1396" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1396" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1396" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1396" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1396" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1396" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1396" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1396" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1396" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1397" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1397" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1397" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1397" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1397" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1397" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1397" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1397" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1397" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1397" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1397" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1397" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1397" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1398" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1398" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1398" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1398" s="15" t="s">
+        <v>668</v>
+      </c>
+      <c r="D1398" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1398" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1398" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1398" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1398" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1398" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1398" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1398" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1398" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1399" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1399" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1399" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1399" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1399" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1399" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1399" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1399" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1399" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1399" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1399" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1399" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1399" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1400" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1400" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1400" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1400" s="15" t="s">
+        <v>670</v>
+      </c>
+      <c r="D1400" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1400" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1400" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1400" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1400" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1400" s="17" t="s">
+        <v>488</v>
+      </c>
+      <c r="J1400" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1400" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1400" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1401" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1401" s="15" t="s">
+        <v>664</v>
+      </c>
+      <c r="B1401" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1401" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1401" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1401" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1401" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1401" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1401" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1401" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1401" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1401" s="19" t="s">
+        <v>665</v>
+      </c>
+      <c r="L1401" s="15" t="s">
+        <v>664</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1387"/>
+  <autoFilter ref="A1:L1401"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-26T07:58:53.772Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16812" uniqueCount="671">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16812" uniqueCount="672">
   <si>
     <t>Date</t>
   </si>
@@ -2021,6 +2021,9 @@
   </si>
   <si>
     <t>09:55</t>
+  </si>
+  <si>
+    <t>15:40</t>
   </si>
   <si>
     <t>drum has been changed</t>
@@ -55596,7 +55599,7 @@
         <v>13</v>
       </c>
       <c r="C1395" s="15" t="s">
-        <v>22</v>
+        <v>669</v>
       </c>
       <c r="D1395" s="17" t="s">
         <v>313</v>
@@ -55610,11 +55613,11 @@
       <c r="G1395" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="H1395" s="8" t="s">
-        <v>24</v>
+      <c r="H1395" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="I1395" s="17" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="J1395" s="17" t="s">
         <v>20</v>
@@ -55786,7 +55789,7 @@
         <v>13</v>
       </c>
       <c r="C1400" s="15" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="D1400" s="17" t="s">
         <v>313</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-26T18:30:27.431Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16812" uniqueCount="672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16980" uniqueCount="677">
   <si>
     <t>Date</t>
   </si>
@@ -2030,6 +2030,21 @@
   </si>
   <si>
     <t>10:09</t>
+  </si>
+  <si>
+    <t>2026-10-27</t>
+  </si>
+  <si>
+    <t>17:59</t>
+  </si>
+  <si>
+    <t>S-mvow7k9h-sj4jg</t>
+  </si>
+  <si>
+    <t>21:37</t>
+  </si>
+  <si>
+    <t>04:29</t>
   </si>
 </sst>
 </file>
@@ -2605,7 +2620,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1401"/>
+  <dimension ref="A1:L1415"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -55857,8 +55872,540 @@
         <v>664</v>
       </c>
     </row>
+    <row r="1402" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1402" s="20" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1402" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1402" s="20" t="s">
+        <v>673</v>
+      </c>
+      <c r="D1402" s="22" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1402" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1402" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1402" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1402" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1402" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1402" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1402" s="24" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1402" s="20" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1403" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1403" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1403" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1403" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1403" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1403" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1403" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1403" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1403" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1403" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1403" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1403" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1403" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1404" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1404" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1404" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1404" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1404" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1404" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1404" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1404" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1404" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1404" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1404" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1404" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1404" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1405" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1405" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1405" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1405" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="D1405" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1405" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1405" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1405" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1405" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1405" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1405" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1405" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1405" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1406" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1406" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1406" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1406" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1406" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1406" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1406" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1406" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1406" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1406" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1406" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1406" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1406" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1407" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1407" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1407" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1407" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="D1407" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1407" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1407" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1407" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1407" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1407" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1407" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1407" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1407" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1408" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1408" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1408" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1408" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="D1408" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1408" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1408" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1408" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1408" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1408" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1408" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1408" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1408" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1409" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1409" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1409" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1409" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D1409" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1409" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1409" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1409" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1409" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1409" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1409" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1409" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1409" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1410" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1410" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1410" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1410" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="D1410" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1410" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1410" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1410" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1410" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1410" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1410" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1410" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1410" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1411" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1411" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1411" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1411" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="D1411" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1411" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1411" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1411" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1411" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1411" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1411" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1411" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1411" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1412" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1412" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1412" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1412" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1412" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1412" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1412" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1412" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1412" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1412" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1412" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1412" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1412" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1413" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1413" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1413" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1413" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1413" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1413" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1413" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1413" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1413" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1413" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1413" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1413" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1413" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1414" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1414" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1414" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1414" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1414" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1414" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1414" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1414" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1414" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1414" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1414" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1414" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1414" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1415" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1415" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1415" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1415" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1415" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1415" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1415" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1415" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1415" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1415" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1415" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1415" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="L1415" s="2" t="s">
+        <v>664</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1401"/>
+  <autoFilter ref="A1:L1415"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-27T07:58:58.285Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16980" uniqueCount="677">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17148" uniqueCount="683">
   <si>
     <t>Date</t>
   </si>
@@ -2045,6 +2045,24 @@
   </si>
   <si>
     <t>04:29</t>
+  </si>
+  <si>
+    <t>S-mvps1y9c-gnm9z</t>
+  </si>
+  <si>
+    <t>06:47</t>
+  </si>
+  <si>
+    <t>09:44</t>
+  </si>
+  <si>
+    <t>15:44</t>
+  </si>
+  <si>
+    <t>15:56</t>
+  </si>
+  <si>
+    <t>07:25</t>
   </si>
 </sst>
 </file>
@@ -2620,7 +2638,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1415"/>
+  <dimension ref="A1:L1429"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -56404,8 +56422,540 @@
         <v>664</v>
       </c>
     </row>
+    <row r="1416" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1416" s="9" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1416" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1416" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1416" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1416" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1416" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1416" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1416" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1416" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1416" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1416" s="14" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1416" s="9" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1417" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1417" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1417" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1417" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1417" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1417" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1417" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1417" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1417" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1417" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1417" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1417" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1417" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1418" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1418" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1418" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1418" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1418" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1418" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1418" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1418" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1418" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1418" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1418" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1418" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1418" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1419" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1419" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1419" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1419" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1419" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1419" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1419" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1419" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1419" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1419" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1419" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1419" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1419" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1420" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1420" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1420" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1420" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1420" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1420" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1420" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1420" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1420" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1420" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1420" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1420" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1420" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1421" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1421" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1421" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1421" s="15" t="s">
+        <v>678</v>
+      </c>
+      <c r="D1421" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1421" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1421" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1421" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1421" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1421" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1421" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1421" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1421" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1422" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1422" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1422" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1422" s="15" t="s">
+        <v>679</v>
+      </c>
+      <c r="D1422" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1422" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1422" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1422" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1422" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1422" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1422" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1422" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1422" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1423" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1423" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1423" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1423" s="15" t="s">
+        <v>680</v>
+      </c>
+      <c r="D1423" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1423" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1423" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1423" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1423" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1423" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1423" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1423" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1423" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1424" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1424" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1424" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1424" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1424" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1424" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1424" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1424" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1424" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1424" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1424" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1424" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1424" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1425" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1425" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1425" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1425" s="15" t="s">
+        <v>681</v>
+      </c>
+      <c r="D1425" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1425" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1425" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1425" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1425" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1425" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1425" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1425" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1425" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1426" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1426" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1426" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1426" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1426" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1426" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1426" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1426" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1426" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1426" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1426" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1426" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1426" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1427" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1427" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1427" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1427" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1427" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1427" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1427" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1427" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1427" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1427" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1427" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1427" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1427" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1428" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1428" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1428" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1428" s="15" t="s">
+        <v>682</v>
+      </c>
+      <c r="D1428" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1428" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1428" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1428" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1428" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1428" s="17" t="s">
+        <v>488</v>
+      </c>
+      <c r="J1428" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1428" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1428" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1429" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1429" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="B1429" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1429" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1429" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E1429" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F1429" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1429" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1429" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1429" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1429" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1429" s="19" t="s">
+        <v>677</v>
+      </c>
+      <c r="L1429" s="15" t="s">
+        <v>672</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1415"/>
+  <autoFilter ref="A1:L1429"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-27T17:54:00.973Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17148" uniqueCount="683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17316" uniqueCount="688">
   <si>
     <t>Date</t>
   </si>
@@ -2063,6 +2063,21 @@
   </si>
   <si>
     <t>07:25</t>
+  </si>
+  <si>
+    <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>S-mvps1wlk-jkvnl</t>
+  </si>
+  <si>
+    <t>21:16</t>
+  </si>
+  <si>
+    <t>02:53</t>
+  </si>
+  <si>
+    <t>04:53</t>
   </si>
 </sst>
 </file>
@@ -2638,7 +2653,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1429"/>
+  <dimension ref="A1:L1443"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -56954,8 +56969,540 @@
         <v>672</v>
       </c>
     </row>
+    <row r="1430" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1430" s="20" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1430" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1430" s="20" t="s">
+        <v>673</v>
+      </c>
+      <c r="D1430" s="22" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1430" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1430" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1430" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1430" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1430" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1430" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1430" s="24" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1430" s="20" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1431" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1431" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1431" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1431" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1431" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1431" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1431" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1431" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1431" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1431" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1431" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1431" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1431" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1432" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1432" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1432" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1432" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1432" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1432" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1432" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1432" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1432" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1432" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1432" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1432" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1432" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1433" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1433" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1433" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1433" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="D1433" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1433" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1433" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1433" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1433" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1433" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1433" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1433" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1433" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1434" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1434" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1434" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1434" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1434" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1434" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1434" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1434" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1434" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1434" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1434" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1434" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1434" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1435" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1435" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1435" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1435" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="D1435" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1435" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1435" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1435" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1435" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1435" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1435" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1435" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1435" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1436" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1436" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1436" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1436" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="D1436" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1436" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1436" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1436" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1436" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1436" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1436" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1436" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1436" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1437" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1437" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1437" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1437" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="D1437" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1437" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1437" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1437" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1437" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1437" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1437" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1437" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1437" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1438" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1438" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1438" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1438" s="2" t="s">
+        <v>687</v>
+      </c>
+      <c r="D1438" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1438" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1438" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1438" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1438" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1438" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1438" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1438" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1438" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1439" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1439" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1439" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1439" s="2" t="s">
+        <v>687</v>
+      </c>
+      <c r="D1439" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1439" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1439" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1439" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1439" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1439" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1439" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1439" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1439" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1440" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1440" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1440" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1440" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1440" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1440" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1440" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1440" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1440" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1440" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1440" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1440" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1440" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1441" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1441" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1441" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1441" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1441" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1441" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1441" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1441" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1441" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1441" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1441" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1441" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1441" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1442" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1442" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1442" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1442" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1442" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1442" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1442" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1442" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1442" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1442" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1442" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1442" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1442" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="1443" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1443" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1443" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1443" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1443" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1443" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1443" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1443" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1443" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1443" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1443" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1443" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="L1443" s="2" t="s">
+        <v>672</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1429"/>
+  <autoFilter ref="A1:L1443"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-27T19:24:06.126Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -57287,7 +57287,7 @@
         <v>472</v>
       </c>
       <c r="E1438" s="4" t="s">
-        <v>472</v>
+        <v>222</v>
       </c>
       <c r="F1438" s="5" t="s">
         <v>29</v>
@@ -57325,7 +57325,7 @@
         <v>472</v>
       </c>
       <c r="E1439" s="4" t="s">
-        <v>472</v>
+        <v>222</v>
       </c>
       <c r="F1439" s="5" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Checklist log update 2026-10-28T08:05:09.067Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17316" uniqueCount="688">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17484" uniqueCount="694">
   <si>
     <t>Date</t>
   </si>
@@ -2078,6 +2078,24 @@
   </si>
   <si>
     <t>04:53</t>
+  </si>
+  <si>
+    <t>Anthony  Tim</t>
+  </si>
+  <si>
+    <t>S-mvqziz34-d6ejj</t>
+  </si>
+  <si>
+    <t>06:13</t>
+  </si>
+  <si>
+    <t>good full</t>
+  </si>
+  <si>
+    <t>09:41</t>
+  </si>
+  <si>
+    <t>ok</t>
   </si>
 </sst>
 </file>
@@ -2653,7 +2671,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1443"/>
+  <dimension ref="A1:L1457"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -57501,8 +57519,540 @@
         <v>672</v>
       </c>
     </row>
+    <row r="1444" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1444" s="9" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1444" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1444" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1444" s="11" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1444" s="11" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1444" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1444" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1444" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1444" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1444" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1444" s="14" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1444" s="9" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1445" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1445" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1445" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1445" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1445" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1445" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1445" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1445" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1445" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1445" s="17" t="s">
+        <v>520</v>
+      </c>
+      <c r="J1445" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1445" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1445" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1446" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1446" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1446" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1446" s="15" t="s">
+        <v>690</v>
+      </c>
+      <c r="D1446" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1446" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1446" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1446" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1446" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1446" s="17" t="s">
+        <v>520</v>
+      </c>
+      <c r="J1446" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1446" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1446" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1447" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1447" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1447" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1447" s="15" t="s">
+        <v>690</v>
+      </c>
+      <c r="D1447" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1447" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1447" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1447" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1447" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1447" s="17" t="s">
+        <v>691</v>
+      </c>
+      <c r="J1447" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1447" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1447" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1448" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1448" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1448" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1448" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1448" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1448" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1448" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1448" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1448" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1448" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1448" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1448" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1448" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1449" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1449" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1449" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1449" s="15" t="s">
+        <v>690</v>
+      </c>
+      <c r="D1449" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1449" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1449" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1449" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1449" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1449" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1449" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1449" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1449" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1450" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1450" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1450" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1450" s="15" t="s">
+        <v>692</v>
+      </c>
+      <c r="D1450" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1450" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1450" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1450" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1450" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1450" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1450" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1450" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1450" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1451" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1451" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1451" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1451" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1451" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1451" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1451" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1451" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1451" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1451" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1451" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1451" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1451" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1452" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1452" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1452" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1452" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1452" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1452" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1452" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1452" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1452" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1452" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1452" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1452" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1452" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1453" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1453" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1453" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1453" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1453" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1453" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1453" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1453" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1453" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1453" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1453" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1453" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1453" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1454" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1454" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1454" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1454" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1454" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1454" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1454" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1454" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1454" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1454" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1454" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1454" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1454" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1455" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1455" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1455" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1455" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1455" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1455" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1455" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1455" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1455" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1455" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1455" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1455" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1455" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1456" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1456" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1456" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1456" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1456" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1456" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1456" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1456" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1456" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1456" s="17" t="s">
+        <v>693</v>
+      </c>
+      <c r="J1456" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1456" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1456" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1457" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1457" s="15" t="s">
+        <v>683</v>
+      </c>
+      <c r="B1457" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1457" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1457" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1457" s="17" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1457" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1457" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1457" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1457" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1457" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1457" s="19" t="s">
+        <v>689</v>
+      </c>
+      <c r="L1457" s="15" t="s">
+        <v>683</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1443"/>
+  <autoFilter ref="A1:L1457"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-28T19:04:32.220Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17484" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17652" uniqueCount="699">
   <si>
     <t>Date</t>
   </si>
@@ -2096,6 +2096,21 @@
   </si>
   <si>
     <t>ok</t>
+  </si>
+  <si>
+    <t>2026-10-29</t>
+  </si>
+  <si>
+    <t>18:06</t>
+  </si>
+  <si>
+    <t>S-mvrtxync-vqt5a</t>
+  </si>
+  <si>
+    <t>05:04</t>
+  </si>
+  <si>
+    <t>03:13</t>
   </si>
 </sst>
 </file>
@@ -2671,7 +2686,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1457"/>
+  <dimension ref="A1:L1471"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -58051,8 +58066,540 @@
         <v>683</v>
       </c>
     </row>
+    <row r="1458" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1458" s="20" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1458" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1458" s="20" t="s">
+        <v>695</v>
+      </c>
+      <c r="D1458" s="22" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1458" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1458" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1458" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1458" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1458" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1458" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1458" s="24" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1458" s="20" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1459" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1459" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1459" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1459" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1459" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1459" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1459" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1459" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1459" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1459" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1459" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1459" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1459" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1460" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1460" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1460" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1460" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1460" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1460" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1460" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1460" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1460" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1460" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1460" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1460" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1460" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1461" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1461" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1461" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1461" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1461" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1461" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1461" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1461" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1461" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1461" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1461" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1461" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1461" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1462" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1462" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1462" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1462" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1462" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1462" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1462" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1462" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1462" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1462" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1462" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1462" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1462" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1463" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1463" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1463" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1463" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="D1463" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1463" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1463" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1463" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1463" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1463" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1463" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1463" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1463" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1464" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1464" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1464" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1464" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D1464" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1464" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1464" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1464" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1464" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1464" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1464" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1464" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1464" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1465" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1465" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1465" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1465" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="D1465" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1465" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F1465" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1465" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1465" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1465" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1465" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1465" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1465" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1466" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1466" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1466" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1466" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="D1466" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1466" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1466" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1466" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1466" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1466" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1466" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1466" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1466" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1467" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1467" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1467" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1467" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="D1467" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1467" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1467" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1467" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1467" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1467" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1467" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1467" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1467" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1468" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1468" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1468" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1468" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D1468" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1468" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1468" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1468" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1468" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1468" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1468" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1468" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1468" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1469" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1469" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1469" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1469" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1469" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1469" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1469" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1469" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1469" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1469" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1469" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1469" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1469" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1470" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1470" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1470" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1470" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1470" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1470" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1470" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1470" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1470" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1470" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1470" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1470" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1470" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="1471" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1471" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1471" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1471" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1471" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1471" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="F1471" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1471" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1471" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1471" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1471" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1471" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="L1471" s="2" t="s">
+        <v>683</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1457"/>
+  <autoFilter ref="A1:L1471"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-28T20:27:40.502Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -58101,7 +58101,7 @@
         <v>696</v>
       </c>
       <c r="L1458" s="20" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1459" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58139,7 +58139,7 @@
         <v>696</v>
       </c>
       <c r="L1459" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1460" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58177,7 +58177,7 @@
         <v>696</v>
       </c>
       <c r="L1460" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1461" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58215,7 +58215,7 @@
         <v>696</v>
       </c>
       <c r="L1461" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1462" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58253,7 +58253,7 @@
         <v>696</v>
       </c>
       <c r="L1462" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1463" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58291,7 +58291,7 @@
         <v>696</v>
       </c>
       <c r="L1463" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1464" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58329,7 +58329,7 @@
         <v>696</v>
       </c>
       <c r="L1464" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1465" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58367,7 +58367,7 @@
         <v>696</v>
       </c>
       <c r="L1465" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1466" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58405,7 +58405,7 @@
         <v>696</v>
       </c>
       <c r="L1466" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1467" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58443,7 +58443,7 @@
         <v>696</v>
       </c>
       <c r="L1467" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1468" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58481,7 +58481,7 @@
         <v>696</v>
       </c>
       <c r="L1468" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1469" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58519,7 +58519,7 @@
         <v>696</v>
       </c>
       <c r="L1469" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1470" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58557,7 +58557,7 @@
         <v>696</v>
       </c>
       <c r="L1470" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="1471" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -58595,7 +58595,7 @@
         <v>696</v>
       </c>
       <c r="L1471" s="2" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checklist log update 2026-10-29T08:01:30.146Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17652" uniqueCount="699">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17820" uniqueCount="705">
   <si>
     <t>Date</t>
   </si>
@@ -2111,6 +2111,24 @@
   </si>
   <si>
     <t>03:13</t>
+  </si>
+  <si>
+    <t>06:27</t>
+  </si>
+  <si>
+    <t>S-mvskg7q9-p6kq4</t>
+  </si>
+  <si>
+    <t>06:34</t>
+  </si>
+  <si>
+    <t>09:42</t>
+  </si>
+  <si>
+    <t>15:09</t>
+  </si>
+  <si>
+    <t>17:12</t>
   </si>
 </sst>
 </file>
@@ -2686,7 +2704,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1471"/>
+  <dimension ref="A1:L1485"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -58598,8 +58616,540 @@
         <v>694</v>
       </c>
     </row>
+    <row r="1472" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1472" s="9" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1472" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1472" s="9" t="s">
+        <v>699</v>
+      </c>
+      <c r="D1472" s="11" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1472" s="11" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1472" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1472" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1472" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1472" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1472" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1472" s="14" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1472" s="9" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1473" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1473" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1473" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1473" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1473" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1473" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1473" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1473" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1473" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1473" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1473" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1473" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1473" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1474" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1474" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1474" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1474" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1474" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1474" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1474" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1474" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1474" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1474" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1474" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1474" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1474" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1475" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1475" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1475" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1475" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1475" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1475" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1475" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1475" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1475" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1475" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1475" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1475" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1475" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1476" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1476" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1476" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1476" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1476" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1476" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1476" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1476" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1476" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1476" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1476" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1476" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1476" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1477" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1477" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1477" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1477" s="15" t="s">
+        <v>701</v>
+      </c>
+      <c r="D1477" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1477" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1477" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1477" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1477" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1477" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1477" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1477" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1477" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1478" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1478" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1478" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1478" s="15" t="s">
+        <v>702</v>
+      </c>
+      <c r="D1478" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1478" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1478" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1478" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1478" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1478" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1478" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1478" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1478" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1479" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1479" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1479" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1479" s="15" t="s">
+        <v>703</v>
+      </c>
+      <c r="D1479" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1479" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1479" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1479" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1479" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1479" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1479" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1479" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1479" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1480" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1480" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1480" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1480" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1480" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1480" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1480" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1480" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1480" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1480" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1480" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1480" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1480" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1481" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1481" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1481" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1481" s="15" t="s">
+        <v>704</v>
+      </c>
+      <c r="D1481" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1481" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1481" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1481" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1481" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1481" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1481" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1481" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1481" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1482" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1482" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1482" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1482" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1482" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1482" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1482" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1482" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1482" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1482" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1482" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1482" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1482" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1483" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1483" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1483" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1483" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1483" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1483" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1483" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1483" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1483" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1483" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1483" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1483" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1483" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1484" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1484" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1484" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1484" s="15" t="s">
+        <v>699</v>
+      </c>
+      <c r="D1484" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1484" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1484" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1484" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1484" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1484" s="17" t="s">
+        <v>488</v>
+      </c>
+      <c r="J1484" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1484" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1484" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1485" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1485" s="15" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1485" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1485" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1485" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1485" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1485" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1485" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1485" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1485" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1485" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1485" s="19" t="s">
+        <v>700</v>
+      </c>
+      <c r="L1485" s="15" t="s">
+        <v>694</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1471"/>
+  <autoFilter ref="A1:L1485"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-29T19:17:42.367Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17820" uniqueCount="705">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17988" uniqueCount="707">
   <si>
     <t>Date</t>
   </si>
@@ -2129,6 +2129,12 @@
   </si>
   <si>
     <t>17:12</t>
+  </si>
+  <si>
+    <t>2026-10-30</t>
+  </si>
+  <si>
+    <t>S-mvt98j5o-pzrih</t>
   </si>
 </sst>
 </file>
@@ -2704,7 +2710,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1485"/>
+  <dimension ref="A1:L1499"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -59148,8 +59154,540 @@
         <v>694</v>
       </c>
     </row>
+    <row r="1486" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1486" s="20" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1486" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1486" s="20" t="s">
+        <v>471</v>
+      </c>
+      <c r="D1486" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1486" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1486" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1486" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1486" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1486" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1486" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1486" s="24" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1486" s="20" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1487" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1487" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1487" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1487" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1487" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1487" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1487" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1487" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1487" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1487" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1487" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1487" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1487" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1488" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1488" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1488" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1488" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1488" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1488" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1488" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1488" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1488" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1488" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1488" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1488" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1488" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1489" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1489" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1489" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1489" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="D1489" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1489" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1489" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1489" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1489" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1489" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1489" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1489" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1489" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1490" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1490" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1490" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1490" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1490" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1490" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1490" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1490" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1490" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1490" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1490" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1490" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1490" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1491" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1491" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1491" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1491" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="D1491" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1491" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1491" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1491" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1491" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1491" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1491" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1491" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1491" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1492" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1492" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1492" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1492" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D1492" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1492" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1492" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1492" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1492" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1492" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1492" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1492" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1492" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1493" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1493" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1493" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1493" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D1493" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1493" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1493" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1493" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1493" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1493" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1493" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1493" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1493" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1494" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1494" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1494" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1494" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="D1494" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1494" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1494" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1494" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1494" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1494" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1494" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1494" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1494" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1495" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1495" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1495" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1495" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="D1495" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1495" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1495" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1495" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1495" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1495" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1495" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1495" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1495" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1496" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1496" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1496" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1496" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1496" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1496" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1496" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1496" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1496" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1496" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1496" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1496" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1496" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1497" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1497" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1497" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1497" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1497" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1497" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1497" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1497" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1497" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1497" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1497" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1497" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1497" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1498" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1498" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1498" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1498" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1498" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1498" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1498" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1498" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1498" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1498" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1498" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1498" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1498" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="1499" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1499" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1499" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1499" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1499" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1499" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1499" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1499" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1499" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1499" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1499" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1499" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="L1499" s="2" t="s">
+        <v>694</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1485"/>
+  <autoFilter ref="A1:L1499"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-30T07:54:59.191Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17988" uniqueCount="707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18156" uniqueCount="713">
   <si>
     <t>Date</t>
   </si>
@@ -2135,6 +2135,24 @@
   </si>
   <si>
     <t>S-mvt98j5o-pzrih</t>
+  </si>
+  <si>
+    <t>06:22</t>
+  </si>
+  <si>
+    <t>S-mvtzp1sl-h3x2c</t>
+  </si>
+  <si>
+    <t>06:23</t>
+  </si>
+  <si>
+    <t>16:08</t>
+  </si>
+  <si>
+    <t>17:54</t>
+  </si>
+  <si>
+    <t>90%</t>
   </si>
 </sst>
 </file>
@@ -2710,7 +2728,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1499"/>
+  <dimension ref="A1:L1513"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -59686,8 +59704,540 @@
         <v>694</v>
       </c>
     </row>
+    <row r="1500" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1500" s="9" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1500" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1500" s="9" t="s">
+        <v>707</v>
+      </c>
+      <c r="D1500" s="11" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1500" s="11" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1500" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1500" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1500" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1500" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1500" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1500" s="14" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1500" s="9" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1501" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1501" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1501" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1501" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1501" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1501" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1501" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1501" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1501" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1501" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1501" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1501" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1501" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1502" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1502" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1502" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1502" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1502" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1502" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1502" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1502" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1502" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1502" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1502" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1502" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1502" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1503" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1503" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1503" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1503" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1503" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1503" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1503" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1503" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1503" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1503" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1503" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1503" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1503" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1504" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1504" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1504" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1504" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1504" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1504" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1504" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1504" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1504" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1504" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1504" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1504" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1504" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1505" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1505" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1505" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1505" s="15" t="s">
+        <v>709</v>
+      </c>
+      <c r="D1505" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1505" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1505" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1505" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1505" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1505" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1505" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1505" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1505" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1506" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1506" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1506" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1506" s="15" t="s">
+        <v>293</v>
+      </c>
+      <c r="D1506" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1506" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1506" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1506" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1506" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1506" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1506" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1506" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1506" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1507" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1507" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1507" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1507" s="15" t="s">
+        <v>710</v>
+      </c>
+      <c r="D1507" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1507" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1507" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1507" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1507" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1507" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1507" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1507" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1507" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1508" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1508" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1508" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1508" s="15" t="s">
+        <v>711</v>
+      </c>
+      <c r="D1508" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1508" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1508" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1508" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1508" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1508" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1508" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1508" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1508" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1509" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1509" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1509" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1509" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="D1509" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1509" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1509" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1509" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1509" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1509" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1509" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1509" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1509" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1510" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1510" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1510" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1510" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1510" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1510" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1510" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1510" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1510" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1510" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1510" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1510" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1510" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1511" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1511" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1511" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1511" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1511" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1511" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1511" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1511" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1511" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1511" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1511" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1511" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1511" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1512" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1512" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1512" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1512" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1512" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1512" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1512" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1512" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1512" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1512" s="17" t="s">
+        <v>712</v>
+      </c>
+      <c r="J1512" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1512" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1512" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1513" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1513" s="15" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1513" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1513" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1513" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="E1513" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="F1513" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1513" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1513" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1513" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1513" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1513" s="19" t="s">
+        <v>708</v>
+      </c>
+      <c r="L1513" s="15" t="s">
+        <v>705</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1499"/>
+  <autoFilter ref="A1:L1513"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-30T19:34:48.044Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18156" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18324" uniqueCount="719">
   <si>
     <t>Date</t>
   </si>
@@ -2153,6 +2153,24 @@
   </si>
   <si>
     <t>90%</t>
+  </si>
+  <si>
+    <t>2026-10-31</t>
+  </si>
+  <si>
+    <t>19:35</t>
+  </si>
+  <si>
+    <t>S-mvus0nr4-n2m1y</t>
+  </si>
+  <si>
+    <t>20:50</t>
+  </si>
+  <si>
+    <t>03:47</t>
+  </si>
+  <si>
+    <t>04:21</t>
   </si>
 </sst>
 </file>
@@ -2728,7 +2746,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1513"/>
+  <dimension ref="A1:L1527"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -60236,8 +60254,540 @@
         <v>705</v>
       </c>
     </row>
+    <row r="1514" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1514" s="20" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1514" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1514" s="20" t="s">
+        <v>714</v>
+      </c>
+      <c r="D1514" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1514" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1514" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1514" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1514" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1514" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1514" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1514" s="24" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1514" s="20" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1515" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1515" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1515" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1515" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1515" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1515" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1515" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1515" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1515" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1515" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1515" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1515" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1515" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1516" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1516" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1516" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1516" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1516" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1516" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1516" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1516" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1516" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1516" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1516" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1516" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1516" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1517" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1517" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1517" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1517" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="D1517" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1517" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1517" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1517" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1517" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1517" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1517" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1517" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1517" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1518" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1518" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1518" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1518" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1518" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1518" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1518" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1518" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1518" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1518" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1518" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1518" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1518" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1519" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1519" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1519" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1519" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="D1519" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1519" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1519" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1519" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1519" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1519" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1519" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1519" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1519" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1520" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1520" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1520" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1520" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="D1520" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1520" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1520" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1520" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1520" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1520" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1520" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1520" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1520" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1521" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1521" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1521" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1521" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="D1521" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1521" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1521" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1521" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1521" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1521" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1521" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1521" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1521" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1522" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1522" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1522" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1522" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="D1522" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1522" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1522" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1522" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1522" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1522" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1522" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1522" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1522" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1523" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1523" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1523" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1523" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="D1523" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1523" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1523" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1523" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1523" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1523" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1523" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1523" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1523" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1524" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1524" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1524" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1524" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1524" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1524" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1524" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1524" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1524" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1524" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1524" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1524" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1524" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1525" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1525" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1525" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1525" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1525" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1525" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1525" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1525" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1525" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1525" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1525" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1525" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1525" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1526" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1526" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1526" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1526" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1526" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1526" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1526" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1526" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1526" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1526" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1526" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1526" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1526" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1527" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1527" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1527" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1527" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1527" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1527" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1527" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1527" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1527" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1527" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1527" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1527" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="L1527" s="2" t="s">
+        <v>705</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1513"/>
+  <autoFilter ref="A1:L1527"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Checklist log update 2026-10-31T07:35:41.543Z
</commit_message>
<xml_diff>
--- a/newlog.xlsx
+++ b/newlog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18324" uniqueCount="719">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18492" uniqueCount="723">
   <si>
     <t>Date</t>
   </si>
@@ -2171,6 +2171,18 @@
   </si>
   <si>
     <t>04:21</t>
+  </si>
+  <si>
+    <t>DH KYB</t>
+  </si>
+  <si>
+    <t>S-mvven3c0-h4yfp</t>
+  </si>
+  <si>
+    <t>09:19</t>
+  </si>
+  <si>
+    <t>17:04</t>
   </si>
 </sst>
 </file>
@@ -2746,7 +2758,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L1527"/>
+  <dimension ref="A1:L1541"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -60786,8 +60798,540 @@
         <v>705</v>
       </c>
     </row>
+    <row r="1528" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1528" s="9" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1528" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1528" s="9" t="s">
+        <v>589</v>
+      </c>
+      <c r="D1528" s="11" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1528" s="11" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1528" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1528" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1528" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1528" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1528" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1528" s="14" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1528" s="9" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1529" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1529" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1529" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1529" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1529" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1529" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1529" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1529" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1529" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1529" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1529" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1529" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1529" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1530" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1530" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1530" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1530" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1530" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1530" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1530" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1530" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1530" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1530" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1530" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1530" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1530" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1531" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1531" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1531" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1531" s="15" t="s">
+        <v>659</v>
+      </c>
+      <c r="D1531" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1531" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1531" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1531" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1531" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1531" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1531" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1531" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1531" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1532" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1532" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1532" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1532" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1532" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1532" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1532" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1532" s="17" t="s">
+        <v>631</v>
+      </c>
+      <c r="H1532" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1532" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1532" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1532" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1532" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1533" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1533" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1533" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1533" s="15" t="s">
+        <v>589</v>
+      </c>
+      <c r="D1533" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1533" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1533" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1533" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1533" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1533" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1533" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1533" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1533" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1534" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1534" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1534" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1534" s="15" t="s">
+        <v>721</v>
+      </c>
+      <c r="D1534" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1534" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1534" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1534" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1534" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1534" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1534" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1534" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1534" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1535" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1535" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1535" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1535" s="15" t="s">
+        <v>383</v>
+      </c>
+      <c r="D1535" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1535" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1535" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1535" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1535" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1535" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1535" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1535" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1535" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1536" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1536" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1536" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1536" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="D1536" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1536" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1536" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1536" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1536" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1536" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1536" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1536" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1536" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1537" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1537" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1537" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1537" s="15" t="s">
+        <v>722</v>
+      </c>
+      <c r="D1537" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1537" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1537" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1537" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1537" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1537" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1537" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1537" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1537" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1538" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1538" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1538" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1538" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1538" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1538" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1538" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1538" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1538" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1538" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1538" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1538" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1538" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1539" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1539" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1539" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1539" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1539" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1539" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1539" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1539" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1539" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1539" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1539" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1539" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1539" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1540" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1540" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1540" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1540" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1540" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1540" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1540" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1540" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1540" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1540" s="17" t="s">
+        <v>712</v>
+      </c>
+      <c r="J1540" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1540" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1540" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="1541" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1541" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1541" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1541" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="D1541" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="E1541" s="17" t="s">
+        <v>719</v>
+      </c>
+      <c r="F1541" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1541" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1541" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1541" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1541" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1541" s="19" t="s">
+        <v>720</v>
+      </c>
+      <c r="L1541" s="15" t="s">
+        <v>713</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1527"/>
+  <autoFilter ref="A1:L1541"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>